<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@ce7d8265d2bcff6ee633535c32a5831470cfbd1d 🚀
</commit_message>
<xml_diff>
--- a/StructureDefinition-Flag.xlsx
+++ b/StructureDefinition-Flag.xlsx
@@ -10,13 +10,13 @@
     <sheet name="Elements" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AP$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AP$47</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1664" uniqueCount="309">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1817" uniqueCount="313">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-07-19T13:11:18+00:00</t>
+    <t>2024-07-19T13:53:40+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -678,6 +678,58 @@
     <t>class</t>
   </si>
   <si>
+    <t>Flag.category.id</t>
+  </si>
+  <si>
+    <t>Flag.category.extension</t>
+  </si>
+  <si>
+    <t>Flag.category.coding</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coding
+</t>
+  </si>
+  <si>
+    <t>Code defined by a terminology system</t>
+  </si>
+  <si>
+    <t>A reference to a code defined by a terminology system.</t>
+  </si>
+  <si>
+    <t>Codes may be defined very casually in enumerations, or code lists, up to very formal definitions such as SNOMED CT - see the HL7 v3 Core Principles for more information.  Ordering of codings is undefined and SHALL NOT be used to infer meaning. Generally, at most only one of the coding values will be labeled as UserSelected = true.</t>
+  </si>
+  <si>
+    <t>Allows for translations and alternate encodings within a code system.  Also supports communication of the same instance to systems requiring different encodings.</t>
+  </si>
+  <si>
+    <t>CodeableConcept.coding</t>
+  </si>
+  <si>
+    <t>union(., ./translation)</t>
+  </si>
+  <si>
+    <t>Flag.category.text</t>
+  </si>
+  <si>
+    <t>Plain text representation of the concept</t>
+  </si>
+  <si>
+    <t>A human language representation of the concept as seen/selected/uttered by the user who entered the data and/or which represents the intended meaning of the user.</t>
+  </si>
+  <si>
+    <t>Very often the text is the same as a displayName of one of the codings.</t>
+  </si>
+  <si>
+    <t>The codes from the terminologies do not always capture the correct meaning with all the nuances of the human using them, or sometimes there is no appropriate code at all. In these cases, the text is used to capture the full meaning of the source.</t>
+  </si>
+  <si>
+    <t>CodeableConcept.text</t>
+  </si>
+  <si>
+    <t>./originalText[mediaType/code="text/plain"]/data</t>
+  </si>
+  <si>
     <t>Flag.code</t>
   </si>
   <si>
@@ -725,47 +777,7 @@
     <t>Flag.code.coding</t>
   </si>
   <si>
-    <t xml:space="preserve">Coding
-</t>
-  </si>
-  <si>
-    <t>Code defined by a terminology system</t>
-  </si>
-  <si>
-    <t>A reference to a code defined by a terminology system.</t>
-  </si>
-  <si>
-    <t>Codes may be defined very casually in enumerations, or code lists, up to very formal definitions such as SNOMED CT - see the HL7 v3 Core Principles for more information.  Ordering of codings is undefined and SHALL NOT be used to infer meaning. Generally, at most only one of the coding values will be labeled as UserSelected = true.</t>
-  </si>
-  <si>
-    <t>Allows for translations and alternate encodings within a code system.  Also supports communication of the same instance to systems requiring different encodings.</t>
-  </si>
-  <si>
-    <t>CodeableConcept.coding</t>
-  </si>
-  <si>
-    <t>union(., ./translation)</t>
-  </si>
-  <si>
     <t>Flag.code.text</t>
-  </si>
-  <si>
-    <t>Plain text representation of the concept</t>
-  </si>
-  <si>
-    <t>A human language representation of the concept as seen/selected/uttered by the user who entered the data and/or which represents the intended meaning of the user.</t>
-  </si>
-  <si>
-    <t>Very often the text is the same as a displayName of one of the codings.</t>
-  </si>
-  <si>
-    <t>The codes from the terminologies do not always capture the correct meaning with all the nuances of the human using them, or sometimes there is no appropriate code at all. In these cases, the text is used to capture the full meaning of the source.</t>
-  </si>
-  <si>
-    <t>CodeableConcept.text</t>
-  </si>
-  <si>
-    <t>./originalText[mediaType/code="text/plain"]/data</t>
   </si>
   <si>
     <t>Flag.subject</t>
@@ -1321,7 +1333,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AP43"/>
+  <dimension ref="A1:AP47"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="61.9609375" customWidth="true" bestFit="true"/>
@@ -3532,11 +3544,11 @@
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
-        <v>210</v>
+        <v>81</v>
       </c>
       <c r="E19" s="2"/>
       <c r="F19" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="G19" t="s" s="2">
         <v>89</v>
@@ -3548,20 +3560,18 @@
         <v>81</v>
       </c>
       <c r="J19" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="K19" t="s" s="2">
-        <v>201</v>
+        <v>151</v>
       </c>
       <c r="L19" t="s" s="2">
-        <v>211</v>
+        <v>152</v>
       </c>
       <c r="M19" t="s" s="2">
-        <v>212</v>
-      </c>
-      <c r="N19" t="s" s="2">
-        <v>213</v>
-      </c>
+        <v>153</v>
+      </c>
+      <c r="N19" s="2"/>
       <c r="O19" s="2"/>
       <c r="P19" t="s" s="2">
         <v>81</v>
@@ -3574,7 +3584,7 @@
         <v>81</v>
       </c>
       <c r="T19" t="s" s="2">
-        <v>214</v>
+        <v>81</v>
       </c>
       <c r="U19" t="s" s="2">
         <v>81</v>
@@ -3586,11 +3596,13 @@
         <v>81</v>
       </c>
       <c r="X19" t="s" s="2">
-        <v>112</v>
-      </c>
-      <c r="Y19" s="2"/>
+        <v>81</v>
+      </c>
+      <c r="Y19" t="s" s="2">
+        <v>81</v>
+      </c>
       <c r="Z19" t="s" s="2">
-        <v>215</v>
+        <v>81</v>
       </c>
       <c r="AA19" t="s" s="2">
         <v>81</v>
@@ -3608,10 +3620,10 @@
         <v>81</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>209</v>
+        <v>154</v>
       </c>
       <c r="AG19" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="AH19" t="s" s="2">
         <v>89</v>
@@ -3623,41 +3635,41 @@
         <v>81</v>
       </c>
       <c r="AK19" t="s" s="2">
-        <v>216</v>
+        <v>81</v>
       </c>
       <c r="AL19" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AM19" t="s" s="2">
-        <v>216</v>
+        <v>81</v>
       </c>
       <c r="AN19" t="s" s="2">
-        <v>216</v>
+        <v>81</v>
       </c>
       <c r="AO19" t="s" s="2">
-        <v>217</v>
+        <v>155</v>
       </c>
       <c r="AP19" t="s" s="2">
-        <v>218</v>
+        <v>81</v>
       </c>
     </row>
     <row r="20" hidden="true">
       <c r="A20" t="s" s="2">
-        <v>219</v>
+        <v>210</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>219</v>
+        <v>210</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" t="s" s="2">
-        <v>81</v>
+        <v>158</v>
       </c>
       <c r="E20" s="2"/>
       <c r="F20" t="s" s="2">
         <v>79</v>
       </c>
       <c r="G20" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="H20" t="s" s="2">
         <v>81</v>
@@ -3669,15 +3681,17 @@
         <v>81</v>
       </c>
       <c r="K20" t="s" s="2">
-        <v>151</v>
+        <v>134</v>
       </c>
       <c r="L20" t="s" s="2">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="M20" t="s" s="2">
-        <v>153</v>
-      </c>
-      <c r="N20" s="2"/>
+        <v>160</v>
+      </c>
+      <c r="N20" t="s" s="2">
+        <v>161</v>
+      </c>
       <c r="O20" s="2"/>
       <c r="P20" t="s" s="2">
         <v>81</v>
@@ -3714,25 +3728,25 @@
         <v>81</v>
       </c>
       <c r="AB20" t="s" s="2">
-        <v>81</v>
+        <v>137</v>
       </c>
       <c r="AC20" t="s" s="2">
-        <v>81</v>
+        <v>162</v>
       </c>
       <c r="AD20" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AE20" t="s" s="2">
-        <v>81</v>
+        <v>138</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="AG20" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH20" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="AI20" t="s" s="2">
         <v>81</v>
@@ -3761,14 +3775,14 @@
     </row>
     <row r="21" hidden="true">
       <c r="A21" t="s" s="2">
-        <v>220</v>
+        <v>211</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>220</v>
+        <v>211</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
-        <v>158</v>
+        <v>81</v>
       </c>
       <c r="E21" s="2"/>
       <c r="F21" t="s" s="2">
@@ -3784,21 +3798,23 @@
         <v>81</v>
       </c>
       <c r="J21" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="K21" t="s" s="2">
-        <v>134</v>
+        <v>212</v>
       </c>
       <c r="L21" t="s" s="2">
-        <v>159</v>
+        <v>213</v>
       </c>
       <c r="M21" t="s" s="2">
-        <v>160</v>
+        <v>214</v>
       </c>
       <c r="N21" t="s" s="2">
-        <v>161</v>
-      </c>
-      <c r="O21" s="2"/>
+        <v>215</v>
+      </c>
+      <c r="O21" t="s" s="2">
+        <v>216</v>
+      </c>
       <c r="P21" t="s" s="2">
         <v>81</v>
       </c>
@@ -3834,19 +3850,19 @@
         <v>81</v>
       </c>
       <c r="AB21" t="s" s="2">
-        <v>137</v>
+        <v>81</v>
       </c>
       <c r="AC21" t="s" s="2">
-        <v>162</v>
+        <v>81</v>
       </c>
       <c r="AD21" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AE21" t="s" s="2">
-        <v>138</v>
+        <v>81</v>
       </c>
       <c r="AF21" t="s" s="2">
-        <v>163</v>
+        <v>217</v>
       </c>
       <c r="AG21" t="s" s="2">
         <v>79</v>
@@ -3873,7 +3889,7 @@
         <v>81</v>
       </c>
       <c r="AO21" t="s" s="2">
-        <v>155</v>
+        <v>218</v>
       </c>
       <c r="AP21" t="s" s="2">
         <v>81</v>
@@ -3881,10 +3897,10 @@
     </row>
     <row r="22" hidden="true">
       <c r="A22" t="s" s="2">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
@@ -3895,10 +3911,10 @@
         <v>79</v>
       </c>
       <c r="G22" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="H22" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="I22" t="s" s="2">
         <v>81</v>
@@ -3907,19 +3923,19 @@
         <v>90</v>
       </c>
       <c r="K22" t="s" s="2">
+        <v>151</v>
+      </c>
+      <c r="L22" t="s" s="2">
+        <v>220</v>
+      </c>
+      <c r="M22" t="s" s="2">
+        <v>221</v>
+      </c>
+      <c r="N22" t="s" s="2">
         <v>222</v>
       </c>
-      <c r="L22" t="s" s="2">
+      <c r="O22" t="s" s="2">
         <v>223</v>
-      </c>
-      <c r="M22" t="s" s="2">
-        <v>224</v>
-      </c>
-      <c r="N22" t="s" s="2">
-        <v>225</v>
-      </c>
-      <c r="O22" t="s" s="2">
-        <v>226</v>
       </c>
       <c r="P22" t="s" s="2">
         <v>81</v>
@@ -3968,13 +3984,13 @@
         <v>81</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH22" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="AI22" t="s" s="2">
         <v>81</v>
@@ -3995,7 +4011,7 @@
         <v>81</v>
       </c>
       <c r="AO22" t="s" s="2">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="AP22" t="s" s="2">
         <v>81</v>
@@ -4003,24 +4019,24 @@
     </row>
     <row r="23" hidden="true">
       <c r="A23" t="s" s="2">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
-        <v>81</v>
+        <v>227</v>
       </c>
       <c r="E23" s="2"/>
       <c r="F23" t="s" s="2">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="G23" t="s" s="2">
         <v>89</v>
       </c>
       <c r="H23" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="I23" t="s" s="2">
         <v>81</v>
@@ -4029,20 +4045,18 @@
         <v>90</v>
       </c>
       <c r="K23" t="s" s="2">
-        <v>151</v>
+        <v>201</v>
       </c>
       <c r="L23" t="s" s="2">
+        <v>228</v>
+      </c>
+      <c r="M23" t="s" s="2">
+        <v>229</v>
+      </c>
+      <c r="N23" t="s" s="2">
         <v>230</v>
       </c>
-      <c r="M23" t="s" s="2">
-        <v>231</v>
-      </c>
-      <c r="N23" t="s" s="2">
-        <v>232</v>
-      </c>
-      <c r="O23" t="s" s="2">
-        <v>233</v>
-      </c>
+      <c r="O23" s="2"/>
       <c r="P23" t="s" s="2">
         <v>81</v>
       </c>
@@ -4054,7 +4068,7 @@
         <v>81</v>
       </c>
       <c r="T23" t="s" s="2">
-        <v>81</v>
+        <v>231</v>
       </c>
       <c r="U23" t="s" s="2">
         <v>81</v>
@@ -4066,13 +4080,11 @@
         <v>81</v>
       </c>
       <c r="X23" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="Y23" t="s" s="2">
-        <v>81</v>
-      </c>
+        <v>112</v>
+      </c>
+      <c r="Y23" s="2"/>
       <c r="Z23" t="s" s="2">
-        <v>81</v>
+        <v>232</v>
       </c>
       <c r="AA23" t="s" s="2">
         <v>81</v>
@@ -4090,10 +4102,10 @@
         <v>81</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>234</v>
+        <v>226</v>
       </c>
       <c r="AG23" t="s" s="2">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="AH23" t="s" s="2">
         <v>89</v>
@@ -4105,22 +4117,22 @@
         <v>81</v>
       </c>
       <c r="AK23" t="s" s="2">
-        <v>81</v>
+        <v>233</v>
       </c>
       <c r="AL23" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AM23" t="s" s="2">
-        <v>81</v>
+        <v>233</v>
       </c>
       <c r="AN23" t="s" s="2">
-        <v>81</v>
+        <v>233</v>
       </c>
       <c r="AO23" t="s" s="2">
+        <v>234</v>
+      </c>
+      <c r="AP23" t="s" s="2">
         <v>235</v>
-      </c>
-      <c r="AP23" t="s" s="2">
-        <v>81</v>
       </c>
     </row>
     <row r="24" hidden="true">
@@ -4136,7 +4148,7 @@
       </c>
       <c r="E24" s="2"/>
       <c r="F24" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="G24" t="s" s="2">
         <v>89</v>
@@ -4148,16 +4160,16 @@
         <v>81</v>
       </c>
       <c r="J24" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="K24" t="s" s="2">
-        <v>237</v>
+        <v>151</v>
       </c>
       <c r="L24" t="s" s="2">
-        <v>238</v>
+        <v>152</v>
       </c>
       <c r="M24" t="s" s="2">
-        <v>239</v>
+        <v>153</v>
       </c>
       <c r="N24" s="2"/>
       <c r="O24" s="2"/>
@@ -4208,10 +4220,10 @@
         <v>81</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>236</v>
+        <v>154</v>
       </c>
       <c r="AG24" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="AH24" t="s" s="2">
         <v>89</v>
@@ -4235,29 +4247,29 @@
         <v>81</v>
       </c>
       <c r="AO24" t="s" s="2">
-        <v>240</v>
+        <v>155</v>
       </c>
       <c r="AP24" t="s" s="2">
-        <v>241</v>
+        <v>81</v>
       </c>
     </row>
     <row r="25" hidden="true">
       <c r="A25" t="s" s="2">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
-        <v>81</v>
+        <v>158</v>
       </c>
       <c r="E25" s="2"/>
       <c r="F25" t="s" s="2">
         <v>79</v>
       </c>
       <c r="G25" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="H25" t="s" s="2">
         <v>81</v>
@@ -4269,15 +4281,17 @@
         <v>81</v>
       </c>
       <c r="K25" t="s" s="2">
-        <v>151</v>
+        <v>134</v>
       </c>
       <c r="L25" t="s" s="2">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>153</v>
-      </c>
-      <c r="N25" s="2"/>
+        <v>160</v>
+      </c>
+      <c r="N25" t="s" s="2">
+        <v>161</v>
+      </c>
       <c r="O25" s="2"/>
       <c r="P25" t="s" s="2">
         <v>81</v>
@@ -4314,25 +4328,25 @@
         <v>81</v>
       </c>
       <c r="AB25" t="s" s="2">
-        <v>81</v>
+        <v>137</v>
       </c>
       <c r="AC25" t="s" s="2">
-        <v>81</v>
+        <v>162</v>
       </c>
       <c r="AD25" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AE25" t="s" s="2">
-        <v>81</v>
+        <v>138</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH25" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="AI25" t="s" s="2">
         <v>81</v>
@@ -4361,10 +4375,10 @@
     </row>
     <row r="26" hidden="true">
       <c r="A26" t="s" s="2">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
@@ -4384,19 +4398,23 @@
         <v>81</v>
       </c>
       <c r="J26" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="K26" t="s" s="2">
-        <v>134</v>
+        <v>212</v>
       </c>
       <c r="L26" t="s" s="2">
-        <v>135</v>
+        <v>213</v>
       </c>
       <c r="M26" t="s" s="2">
-        <v>136</v>
-      </c>
-      <c r="N26" s="2"/>
-      <c r="O26" s="2"/>
+        <v>214</v>
+      </c>
+      <c r="N26" t="s" s="2">
+        <v>215</v>
+      </c>
+      <c r="O26" t="s" s="2">
+        <v>216</v>
+      </c>
       <c r="P26" t="s" s="2">
         <v>81</v>
       </c>
@@ -4432,19 +4450,19 @@
         <v>81</v>
       </c>
       <c r="AB26" t="s" s="2">
-        <v>137</v>
+        <v>81</v>
       </c>
       <c r="AC26" t="s" s="2">
-        <v>162</v>
+        <v>81</v>
       </c>
       <c r="AD26" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AE26" t="s" s="2">
-        <v>138</v>
+        <v>81</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>163</v>
+        <v>217</v>
       </c>
       <c r="AG26" t="s" s="2">
         <v>79</v>
@@ -4471,7 +4489,7 @@
         <v>81</v>
       </c>
       <c r="AO26" t="s" s="2">
-        <v>81</v>
+        <v>218</v>
       </c>
       <c r="AP26" t="s" s="2">
         <v>81</v>
@@ -4479,14 +4497,12 @@
     </row>
     <row r="27" hidden="true">
       <c r="A27" t="s" s="2">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>243</v>
-      </c>
-      <c r="C27" t="s" s="2">
-        <v>245</v>
-      </c>
+        <v>239</v>
+      </c>
+      <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
         <v>81</v>
       </c>
@@ -4498,25 +4514,29 @@
         <v>89</v>
       </c>
       <c r="H27" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="I27" t="s" s="2">
         <v>81</v>
       </c>
       <c r="J27" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="K27" t="s" s="2">
-        <v>246</v>
+        <v>151</v>
       </c>
       <c r="L27" t="s" s="2">
-        <v>247</v>
+        <v>220</v>
       </c>
       <c r="M27" t="s" s="2">
-        <v>248</v>
-      </c>
-      <c r="N27" s="2"/>
-      <c r="O27" s="2"/>
+        <v>221</v>
+      </c>
+      <c r="N27" t="s" s="2">
+        <v>222</v>
+      </c>
+      <c r="O27" t="s" s="2">
+        <v>223</v>
+      </c>
       <c r="P27" t="s" s="2">
         <v>81</v>
       </c>
@@ -4564,13 +4584,13 @@
         <v>81</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>163</v>
+        <v>224</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH27" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="AI27" t="s" s="2">
         <v>81</v>
@@ -4591,7 +4611,7 @@
         <v>81</v>
       </c>
       <c r="AO27" t="s" s="2">
-        <v>132</v>
+        <v>225</v>
       </c>
       <c r="AP27" t="s" s="2">
         <v>81</v>
@@ -4599,10 +4619,10 @@
     </row>
     <row r="28" hidden="true">
       <c r="A28" t="s" s="2">
-        <v>249</v>
+        <v>240</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>249</v>
+        <v>240</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -4610,7 +4630,7 @@
       </c>
       <c r="E28" s="2"/>
       <c r="F28" t="s" s="2">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="G28" t="s" s="2">
         <v>89</v>
@@ -4625,17 +4645,15 @@
         <v>90</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>151</v>
+        <v>241</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>250</v>
+        <v>242</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>251</v>
-      </c>
-      <c r="N28" t="s" s="2">
-        <v>252</v>
-      </c>
+        <v>243</v>
+      </c>
+      <c r="N28" s="2"/>
       <c r="O28" s="2"/>
       <c r="P28" t="s" s="2">
         <v>81</v>
@@ -4684,16 +4702,16 @@
         <v>81</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>253</v>
+        <v>240</v>
       </c>
       <c r="AG28" t="s" s="2">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="AH28" t="s" s="2">
         <v>89</v>
       </c>
       <c r="AI28" t="s" s="2">
-        <v>254</v>
+        <v>81</v>
       </c>
       <c r="AJ28" t="s" s="2">
         <v>81</v>
@@ -4711,18 +4729,18 @@
         <v>81</v>
       </c>
       <c r="AO28" t="s" s="2">
-        <v>132</v>
+        <v>244</v>
       </c>
       <c r="AP28" t="s" s="2">
-        <v>81</v>
+        <v>245</v>
       </c>
     </row>
     <row r="29" hidden="true">
       <c r="A29" t="s" s="2">
-        <v>255</v>
+        <v>246</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>255</v>
+        <v>246</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -4742,20 +4760,18 @@
         <v>81</v>
       </c>
       <c r="J29" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>184</v>
+        <v>151</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>256</v>
+        <v>152</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>257</v>
-      </c>
-      <c r="N29" t="s" s="2">
-        <v>258</v>
-      </c>
+        <v>153</v>
+      </c>
+      <c r="N29" s="2"/>
       <c r="O29" s="2"/>
       <c r="P29" t="s" s="2">
         <v>81</v>
@@ -4804,7 +4820,7 @@
         <v>81</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>259</v>
+        <v>154</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>79</v>
@@ -4831,7 +4847,7 @@
         <v>81</v>
       </c>
       <c r="AO29" t="s" s="2">
-        <v>260</v>
+        <v>155</v>
       </c>
       <c r="AP29" t="s" s="2">
         <v>81</v>
@@ -4839,10 +4855,10 @@
     </row>
     <row r="30" hidden="true">
       <c r="A30" t="s" s="2">
-        <v>261</v>
+        <v>247</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>261</v>
+        <v>247</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
@@ -4853,7 +4869,7 @@
         <v>79</v>
       </c>
       <c r="G30" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="H30" t="s" s="2">
         <v>81</v>
@@ -4862,20 +4878,18 @@
         <v>81</v>
       </c>
       <c r="J30" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>151</v>
+        <v>134</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>262</v>
+        <v>135</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>263</v>
-      </c>
-      <c r="N30" t="s" s="2">
-        <v>264</v>
-      </c>
+        <v>136</v>
+      </c>
+      <c r="N30" s="2"/>
       <c r="O30" s="2"/>
       <c r="P30" t="s" s="2">
         <v>81</v>
@@ -4912,25 +4926,25 @@
         <v>81</v>
       </c>
       <c r="AB30" t="s" s="2">
-        <v>81</v>
+        <v>137</v>
       </c>
       <c r="AC30" t="s" s="2">
-        <v>81</v>
+        <v>162</v>
       </c>
       <c r="AD30" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AE30" t="s" s="2">
-        <v>81</v>
+        <v>138</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>265</v>
+        <v>163</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH30" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="AI30" t="s" s="2">
         <v>81</v>
@@ -4951,7 +4965,7 @@
         <v>81</v>
       </c>
       <c r="AO30" t="s" s="2">
-        <v>132</v>
+        <v>81</v>
       </c>
       <c r="AP30" t="s" s="2">
         <v>81</v>
@@ -4959,12 +4973,14 @@
     </row>
     <row r="31" hidden="true">
       <c r="A31" t="s" s="2">
-        <v>266</v>
+        <v>248</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>266</v>
-      </c>
-      <c r="C31" s="2"/>
+        <v>247</v>
+      </c>
+      <c r="C31" t="s" s="2">
+        <v>249</v>
+      </c>
       <c r="D31" t="s" s="2">
         <v>81</v>
       </c>
@@ -4982,16 +4998,16 @@
         <v>81</v>
       </c>
       <c r="J31" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="K31" t="s" s="2">
-        <v>267</v>
+        <v>250</v>
       </c>
       <c r="L31" t="s" s="2">
-        <v>268</v>
+        <v>251</v>
       </c>
       <c r="M31" t="s" s="2">
-        <v>269</v>
+        <v>252</v>
       </c>
       <c r="N31" s="2"/>
       <c r="O31" s="2"/>
@@ -5042,13 +5058,13 @@
         <v>81</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>266</v>
+        <v>163</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH31" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="AI31" t="s" s="2">
         <v>81</v>
@@ -5069,18 +5085,18 @@
         <v>81</v>
       </c>
       <c r="AO31" t="s" s="2">
-        <v>81</v>
+        <v>132</v>
       </c>
       <c r="AP31" t="s" s="2">
-        <v>270</v>
+        <v>81</v>
       </c>
     </row>
     <row r="32" hidden="true">
       <c r="A32" t="s" s="2">
-        <v>271</v>
+        <v>253</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>271</v>
+        <v>253</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
@@ -5100,18 +5116,20 @@
         <v>81</v>
       </c>
       <c r="J32" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="K32" t="s" s="2">
         <v>151</v>
       </c>
       <c r="L32" t="s" s="2">
-        <v>152</v>
+        <v>254</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>153</v>
-      </c>
-      <c r="N32" s="2"/>
+        <v>255</v>
+      </c>
+      <c r="N32" t="s" s="2">
+        <v>256</v>
+      </c>
       <c r="O32" s="2"/>
       <c r="P32" t="s" s="2">
         <v>81</v>
@@ -5160,7 +5178,7 @@
         <v>81</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>154</v>
+        <v>257</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>79</v>
@@ -5169,7 +5187,7 @@
         <v>89</v>
       </c>
       <c r="AI32" t="s" s="2">
-        <v>81</v>
+        <v>258</v>
       </c>
       <c r="AJ32" t="s" s="2">
         <v>81</v>
@@ -5187,7 +5205,7 @@
         <v>81</v>
       </c>
       <c r="AO32" t="s" s="2">
-        <v>155</v>
+        <v>132</v>
       </c>
       <c r="AP32" t="s" s="2">
         <v>81</v>
@@ -5195,21 +5213,21 @@
     </row>
     <row r="33" hidden="true">
       <c r="A33" t="s" s="2">
-        <v>272</v>
+        <v>259</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>272</v>
+        <v>259</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
-        <v>158</v>
+        <v>81</v>
       </c>
       <c r="E33" s="2"/>
       <c r="F33" t="s" s="2">
         <v>79</v>
       </c>
       <c r="G33" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="H33" t="s" s="2">
         <v>81</v>
@@ -5218,19 +5236,19 @@
         <v>81</v>
       </c>
       <c r="J33" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="K33" t="s" s="2">
-        <v>134</v>
+        <v>184</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>159</v>
+        <v>260</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>160</v>
+        <v>261</v>
       </c>
       <c r="N33" t="s" s="2">
-        <v>161</v>
+        <v>262</v>
       </c>
       <c r="O33" s="2"/>
       <c r="P33" t="s" s="2">
@@ -5268,25 +5286,25 @@
         <v>81</v>
       </c>
       <c r="AB33" t="s" s="2">
-        <v>137</v>
+        <v>81</v>
       </c>
       <c r="AC33" t="s" s="2">
-        <v>162</v>
+        <v>81</v>
       </c>
       <c r="AD33" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AE33" t="s" s="2">
-        <v>138</v>
+        <v>81</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>163</v>
+        <v>263</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH33" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="AI33" t="s" s="2">
         <v>81</v>
@@ -5307,7 +5325,7 @@
         <v>81</v>
       </c>
       <c r="AO33" t="s" s="2">
-        <v>155</v>
+        <v>264</v>
       </c>
       <c r="AP33" t="s" s="2">
         <v>81</v>
@@ -5315,14 +5333,14 @@
     </row>
     <row r="34" hidden="true">
       <c r="A34" t="s" s="2">
-        <v>273</v>
+        <v>265</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>273</v>
+        <v>265</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
-        <v>274</v>
+        <v>81</v>
       </c>
       <c r="E34" s="2"/>
       <c r="F34" t="s" s="2">
@@ -5332,7 +5350,7 @@
         <v>89</v>
       </c>
       <c r="H34" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="I34" t="s" s="2">
         <v>81</v>
@@ -5341,16 +5359,16 @@
         <v>90</v>
       </c>
       <c r="K34" t="s" s="2">
-        <v>275</v>
+        <v>151</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>276</v>
+        <v>266</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>277</v>
+        <v>267</v>
       </c>
       <c r="N34" t="s" s="2">
-        <v>278</v>
+        <v>268</v>
       </c>
       <c r="O34" s="2"/>
       <c r="P34" t="s" s="2">
@@ -5364,7 +5382,7 @@
         <v>81</v>
       </c>
       <c r="T34" t="s" s="2">
-        <v>279</v>
+        <v>81</v>
       </c>
       <c r="U34" t="s" s="2">
         <v>81</v>
@@ -5400,7 +5418,7 @@
         <v>81</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>280</v>
+        <v>269</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>79</v>
@@ -5409,25 +5427,25 @@
         <v>89</v>
       </c>
       <c r="AI34" t="s" s="2">
-        <v>281</v>
+        <v>81</v>
       </c>
       <c r="AJ34" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AK34" t="s" s="2">
-        <v>282</v>
+        <v>81</v>
       </c>
       <c r="AL34" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AM34" t="s" s="2">
-        <v>282</v>
+        <v>81</v>
       </c>
       <c r="AN34" t="s" s="2">
-        <v>282</v>
+        <v>81</v>
       </c>
       <c r="AO34" t="s" s="2">
-        <v>283</v>
+        <v>132</v>
       </c>
       <c r="AP34" t="s" s="2">
         <v>81</v>
@@ -5435,10 +5453,10 @@
     </row>
     <row r="35" hidden="true">
       <c r="A35" t="s" s="2">
-        <v>284</v>
+        <v>270</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>284</v>
+        <v>270</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -5461,24 +5479,20 @@
         <v>90</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>285</v>
+        <v>272</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>286</v>
-      </c>
-      <c r="N35" t="s" s="2">
-        <v>287</v>
-      </c>
+        <v>273</v>
+      </c>
+      <c r="N35" s="2"/>
       <c r="O35" s="2"/>
       <c r="P35" t="s" s="2">
         <v>81</v>
       </c>
-      <c r="Q35" t="s" s="2">
-        <v>288</v>
-      </c>
+      <c r="Q35" s="2"/>
       <c r="R35" t="s" s="2">
         <v>81</v>
       </c>
@@ -5522,7 +5536,7 @@
         <v>81</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>289</v>
+        <v>270</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>79</v>
@@ -5531,7 +5545,7 @@
         <v>89</v>
       </c>
       <c r="AI35" t="s" s="2">
-        <v>281</v>
+        <v>81</v>
       </c>
       <c r="AJ35" t="s" s="2">
         <v>81</v>
@@ -5549,18 +5563,18 @@
         <v>81</v>
       </c>
       <c r="AO35" t="s" s="2">
-        <v>290</v>
+        <v>81</v>
       </c>
       <c r="AP35" t="s" s="2">
-        <v>81</v>
+        <v>274</v>
       </c>
     </row>
     <row r="36" hidden="true">
       <c r="A36" t="s" s="2">
-        <v>291</v>
+        <v>275</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>291</v>
+        <v>275</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
@@ -5580,20 +5594,18 @@
         <v>81</v>
       </c>
       <c r="J36" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="K36" t="s" s="2">
-        <v>292</v>
+        <v>151</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>293</v>
+        <v>152</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>294</v>
-      </c>
-      <c r="N36" t="s" s="2">
-        <v>295</v>
-      </c>
+        <v>153</v>
+      </c>
+      <c r="N36" s="2"/>
       <c r="O36" s="2"/>
       <c r="P36" t="s" s="2">
         <v>81</v>
@@ -5642,7 +5654,7 @@
         <v>81</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>291</v>
+        <v>154</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>79</v>
@@ -5669,29 +5681,29 @@
         <v>81</v>
       </c>
       <c r="AO36" t="s" s="2">
-        <v>81</v>
+        <v>155</v>
       </c>
       <c r="AP36" t="s" s="2">
-        <v>270</v>
+        <v>81</v>
       </c>
     </row>
     <row r="37" hidden="true">
       <c r="A37" t="s" s="2">
-        <v>296</v>
+        <v>276</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>296</v>
+        <v>276</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
-        <v>81</v>
+        <v>158</v>
       </c>
       <c r="E37" s="2"/>
       <c r="F37" t="s" s="2">
         <v>79</v>
       </c>
       <c r="G37" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="H37" t="s" s="2">
         <v>81</v>
@@ -5700,18 +5712,20 @@
         <v>81</v>
       </c>
       <c r="J37" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="K37" t="s" s="2">
-        <v>297</v>
+        <v>134</v>
       </c>
       <c r="L37" t="s" s="2">
-        <v>298</v>
+        <v>159</v>
       </c>
       <c r="M37" t="s" s="2">
-        <v>299</v>
-      </c>
-      <c r="N37" s="2"/>
+        <v>160</v>
+      </c>
+      <c r="N37" t="s" s="2">
+        <v>161</v>
+      </c>
       <c r="O37" s="2"/>
       <c r="P37" t="s" s="2">
         <v>81</v>
@@ -5748,25 +5762,25 @@
         <v>81</v>
       </c>
       <c r="AB37" t="s" s="2">
-        <v>81</v>
+        <v>137</v>
       </c>
       <c r="AC37" t="s" s="2">
-        <v>81</v>
+        <v>162</v>
       </c>
       <c r="AD37" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AE37" t="s" s="2">
-        <v>81</v>
+        <v>138</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>296</v>
+        <v>163</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH37" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="AI37" t="s" s="2">
         <v>81</v>
@@ -5778,7 +5792,7 @@
         <v>81</v>
       </c>
       <c r="AL37" t="s" s="2">
-        <v>300</v>
+        <v>81</v>
       </c>
       <c r="AM37" t="s" s="2">
         <v>81</v>
@@ -5787,22 +5801,22 @@
         <v>81</v>
       </c>
       <c r="AO37" t="s" s="2">
-        <v>301</v>
+        <v>155</v>
       </c>
       <c r="AP37" t="s" s="2">
-        <v>302</v>
+        <v>81</v>
       </c>
     </row>
     <row r="38" hidden="true">
       <c r="A38" t="s" s="2">
-        <v>303</v>
+        <v>277</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>303</v>
+        <v>277</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
-        <v>81</v>
+        <v>278</v>
       </c>
       <c r="E38" s="2"/>
       <c r="F38" t="s" s="2">
@@ -5812,24 +5826,26 @@
         <v>89</v>
       </c>
       <c r="H38" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="I38" t="s" s="2">
         <v>81</v>
       </c>
       <c r="J38" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="K38" t="s" s="2">
-        <v>151</v>
+        <v>279</v>
       </c>
       <c r="L38" t="s" s="2">
-        <v>152</v>
+        <v>280</v>
       </c>
       <c r="M38" t="s" s="2">
-        <v>153</v>
-      </c>
-      <c r="N38" s="2"/>
+        <v>281</v>
+      </c>
+      <c r="N38" t="s" s="2">
+        <v>282</v>
+      </c>
       <c r="O38" s="2"/>
       <c r="P38" t="s" s="2">
         <v>81</v>
@@ -5842,7 +5858,7 @@
         <v>81</v>
       </c>
       <c r="T38" t="s" s="2">
-        <v>81</v>
+        <v>283</v>
       </c>
       <c r="U38" t="s" s="2">
         <v>81</v>
@@ -5878,7 +5894,7 @@
         <v>81</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>154</v>
+        <v>284</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>79</v>
@@ -5887,25 +5903,25 @@
         <v>89</v>
       </c>
       <c r="AI38" t="s" s="2">
-        <v>81</v>
+        <v>285</v>
       </c>
       <c r="AJ38" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AK38" t="s" s="2">
-        <v>81</v>
+        <v>286</v>
       </c>
       <c r="AL38" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AM38" t="s" s="2">
-        <v>81</v>
+        <v>286</v>
       </c>
       <c r="AN38" t="s" s="2">
-        <v>81</v>
+        <v>286</v>
       </c>
       <c r="AO38" t="s" s="2">
-        <v>155</v>
+        <v>287</v>
       </c>
       <c r="AP38" t="s" s="2">
         <v>81</v>
@@ -5913,10 +5929,10 @@
     </row>
     <row r="39" hidden="true">
       <c r="A39" t="s" s="2">
-        <v>304</v>
+        <v>288</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>304</v>
+        <v>288</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
@@ -5927,7 +5943,7 @@
         <v>79</v>
       </c>
       <c r="G39" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="H39" t="s" s="2">
         <v>81</v>
@@ -5936,23 +5952,27 @@
         <v>81</v>
       </c>
       <c r="J39" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="K39" t="s" s="2">
-        <v>134</v>
+        <v>279</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>135</v>
+        <v>289</v>
       </c>
       <c r="M39" t="s" s="2">
-        <v>136</v>
-      </c>
-      <c r="N39" s="2"/>
+        <v>290</v>
+      </c>
+      <c r="N39" t="s" s="2">
+        <v>291</v>
+      </c>
       <c r="O39" s="2"/>
       <c r="P39" t="s" s="2">
         <v>81</v>
       </c>
-      <c r="Q39" s="2"/>
+      <c r="Q39" t="s" s="2">
+        <v>292</v>
+      </c>
       <c r="R39" t="s" s="2">
         <v>81</v>
       </c>
@@ -5984,28 +6004,28 @@
         <v>81</v>
       </c>
       <c r="AB39" t="s" s="2">
-        <v>137</v>
+        <v>81</v>
       </c>
       <c r="AC39" t="s" s="2">
-        <v>162</v>
+        <v>81</v>
       </c>
       <c r="AD39" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AE39" t="s" s="2">
-        <v>138</v>
+        <v>81</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>163</v>
+        <v>293</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH39" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="AI39" t="s" s="2">
-        <v>81</v>
+        <v>285</v>
       </c>
       <c r="AJ39" t="s" s="2">
         <v>81</v>
@@ -6023,7 +6043,7 @@
         <v>81</v>
       </c>
       <c r="AO39" t="s" s="2">
-        <v>81</v>
+        <v>294</v>
       </c>
       <c r="AP39" t="s" s="2">
         <v>81</v>
@@ -6031,14 +6051,12 @@
     </row>
     <row r="40" hidden="true">
       <c r="A40" t="s" s="2">
-        <v>305</v>
+        <v>295</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>304</v>
-      </c>
-      <c r="C40" t="s" s="2">
-        <v>245</v>
-      </c>
+        <v>295</v>
+      </c>
+      <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
         <v>81</v>
       </c>
@@ -6056,18 +6074,20 @@
         <v>81</v>
       </c>
       <c r="J40" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="K40" t="s" s="2">
-        <v>246</v>
+        <v>296</v>
       </c>
       <c r="L40" t="s" s="2">
-        <v>247</v>
+        <v>297</v>
       </c>
       <c r="M40" t="s" s="2">
-        <v>248</v>
-      </c>
-      <c r="N40" s="2"/>
+        <v>298</v>
+      </c>
+      <c r="N40" t="s" s="2">
+        <v>299</v>
+      </c>
       <c r="O40" s="2"/>
       <c r="P40" t="s" s="2">
         <v>81</v>
@@ -6116,13 +6136,13 @@
         <v>81</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>163</v>
+        <v>295</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH40" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="AI40" t="s" s="2">
         <v>81</v>
@@ -6143,18 +6163,18 @@
         <v>81</v>
       </c>
       <c r="AO40" t="s" s="2">
-        <v>132</v>
+        <v>81</v>
       </c>
       <c r="AP40" t="s" s="2">
-        <v>81</v>
+        <v>274</v>
       </c>
     </row>
     <row r="41" hidden="true">
       <c r="A41" t="s" s="2">
-        <v>306</v>
+        <v>300</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>306</v>
+        <v>300</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
@@ -6177,17 +6197,15 @@
         <v>90</v>
       </c>
       <c r="K41" t="s" s="2">
-        <v>151</v>
+        <v>301</v>
       </c>
       <c r="L41" t="s" s="2">
-        <v>250</v>
+        <v>302</v>
       </c>
       <c r="M41" t="s" s="2">
-        <v>251</v>
-      </c>
-      <c r="N41" t="s" s="2">
-        <v>252</v>
-      </c>
+        <v>303</v>
+      </c>
+      <c r="N41" s="2"/>
       <c r="O41" s="2"/>
       <c r="P41" t="s" s="2">
         <v>81</v>
@@ -6236,7 +6254,7 @@
         <v>81</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>253</v>
+        <v>300</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>79</v>
@@ -6245,7 +6263,7 @@
         <v>89</v>
       </c>
       <c r="AI41" t="s" s="2">
-        <v>254</v>
+        <v>81</v>
       </c>
       <c r="AJ41" t="s" s="2">
         <v>81</v>
@@ -6254,7 +6272,7 @@
         <v>81</v>
       </c>
       <c r="AL41" t="s" s="2">
-        <v>81</v>
+        <v>304</v>
       </c>
       <c r="AM41" t="s" s="2">
         <v>81</v>
@@ -6263,10 +6281,10 @@
         <v>81</v>
       </c>
       <c r="AO41" t="s" s="2">
-        <v>132</v>
+        <v>305</v>
       </c>
       <c r="AP41" t="s" s="2">
-        <v>81</v>
+        <v>306</v>
       </c>
     </row>
     <row r="42" hidden="true">
@@ -6294,20 +6312,18 @@
         <v>81</v>
       </c>
       <c r="J42" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="K42" t="s" s="2">
-        <v>184</v>
+        <v>151</v>
       </c>
       <c r="L42" t="s" s="2">
-        <v>256</v>
+        <v>152</v>
       </c>
       <c r="M42" t="s" s="2">
-        <v>257</v>
-      </c>
-      <c r="N42" t="s" s="2">
-        <v>258</v>
-      </c>
+        <v>153</v>
+      </c>
+      <c r="N42" s="2"/>
       <c r="O42" s="2"/>
       <c r="P42" t="s" s="2">
         <v>81</v>
@@ -6356,7 +6372,7 @@
         <v>81</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>259</v>
+        <v>154</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>79</v>
@@ -6383,7 +6399,7 @@
         <v>81</v>
       </c>
       <c r="AO42" t="s" s="2">
-        <v>260</v>
+        <v>155</v>
       </c>
       <c r="AP42" t="s" s="2">
         <v>81</v>
@@ -6405,7 +6421,7 @@
         <v>79</v>
       </c>
       <c r="G43" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="H43" t="s" s="2">
         <v>81</v>
@@ -6414,20 +6430,18 @@
         <v>81</v>
       </c>
       <c r="J43" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="K43" t="s" s="2">
-        <v>151</v>
+        <v>134</v>
       </c>
       <c r="L43" t="s" s="2">
-        <v>262</v>
+        <v>135</v>
       </c>
       <c r="M43" t="s" s="2">
-        <v>263</v>
-      </c>
-      <c r="N43" t="s" s="2">
-        <v>264</v>
-      </c>
+        <v>136</v>
+      </c>
+      <c r="N43" s="2"/>
       <c r="O43" s="2"/>
       <c r="P43" t="s" s="2">
         <v>81</v>
@@ -6464,53 +6478,533 @@
         <v>81</v>
       </c>
       <c r="AB43" t="s" s="2">
-        <v>81</v>
+        <v>137</v>
       </c>
       <c r="AC43" t="s" s="2">
-        <v>81</v>
+        <v>162</v>
       </c>
       <c r="AD43" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AE43" t="s" s="2">
-        <v>81</v>
+        <v>138</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>265</v>
+        <v>163</v>
       </c>
       <c r="AG43" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH43" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AI43" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AJ43" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK43" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL43" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM43" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AN43" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AO43" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AP43" t="s" s="2">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="44" hidden="true">
+      <c r="A44" t="s" s="2">
+        <v>309</v>
+      </c>
+      <c r="B44" t="s" s="2">
+        <v>308</v>
+      </c>
+      <c r="C44" t="s" s="2">
+        <v>249</v>
+      </c>
+      <c r="D44" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="E44" s="2"/>
+      <c r="F44" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="G44" t="s" s="2">
         <v>89</v>
       </c>
-      <c r="AI43" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AJ43" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AK43" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AL43" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AM43" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AN43" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AO43" t="s" s="2">
+      <c r="H44" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="I44" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="J44" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="K44" t="s" s="2">
+        <v>250</v>
+      </c>
+      <c r="L44" t="s" s="2">
+        <v>251</v>
+      </c>
+      <c r="M44" t="s" s="2">
+        <v>252</v>
+      </c>
+      <c r="N44" s="2"/>
+      <c r="O44" s="2"/>
+      <c r="P44" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Q44" s="2"/>
+      <c r="R44" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="S44" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="T44" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="U44" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="V44" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="W44" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="X44" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Y44" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Z44" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AA44" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AB44" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AC44" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AD44" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AE44" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AF44" t="s" s="2">
+        <v>163</v>
+      </c>
+      <c r="AG44" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AI44" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AJ44" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK44" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL44" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM44" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AN44" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AO44" t="s" s="2">
         <v>132</v>
       </c>
-      <c r="AP43" t="s" s="2">
+      <c r="AP44" t="s" s="2">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="45" hidden="true">
+      <c r="A45" t="s" s="2">
+        <v>310</v>
+      </c>
+      <c r="B45" t="s" s="2">
+        <v>310</v>
+      </c>
+      <c r="C45" s="2"/>
+      <c r="D45" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="E45" s="2"/>
+      <c r="F45" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="G45" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="H45" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="I45" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="J45" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="K45" t="s" s="2">
+        <v>151</v>
+      </c>
+      <c r="L45" t="s" s="2">
+        <v>254</v>
+      </c>
+      <c r="M45" t="s" s="2">
+        <v>255</v>
+      </c>
+      <c r="N45" t="s" s="2">
+        <v>256</v>
+      </c>
+      <c r="O45" s="2"/>
+      <c r="P45" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Q45" s="2"/>
+      <c r="R45" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="S45" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="T45" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="U45" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="V45" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="W45" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="X45" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Y45" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Z45" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AA45" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AB45" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AC45" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AD45" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AE45" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AF45" t="s" s="2">
+        <v>257</v>
+      </c>
+      <c r="AG45" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH45" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="AI45" t="s" s="2">
+        <v>258</v>
+      </c>
+      <c r="AJ45" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK45" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL45" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM45" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AN45" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AO45" t="s" s="2">
+        <v>132</v>
+      </c>
+      <c r="AP45" t="s" s="2">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="46" hidden="true">
+      <c r="A46" t="s" s="2">
+        <v>311</v>
+      </c>
+      <c r="B46" t="s" s="2">
+        <v>311</v>
+      </c>
+      <c r="C46" s="2"/>
+      <c r="D46" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="E46" s="2"/>
+      <c r="F46" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="G46" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="H46" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="I46" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="J46" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="K46" t="s" s="2">
+        <v>184</v>
+      </c>
+      <c r="L46" t="s" s="2">
+        <v>260</v>
+      </c>
+      <c r="M46" t="s" s="2">
+        <v>261</v>
+      </c>
+      <c r="N46" t="s" s="2">
+        <v>262</v>
+      </c>
+      <c r="O46" s="2"/>
+      <c r="P46" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Q46" s="2"/>
+      <c r="R46" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="S46" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="T46" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="U46" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="V46" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="W46" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="X46" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Y46" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Z46" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AA46" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AB46" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AC46" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AD46" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AE46" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AF46" t="s" s="2">
+        <v>263</v>
+      </c>
+      <c r="AG46" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH46" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="AI46" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AJ46" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK46" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL46" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM46" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AN46" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AO46" t="s" s="2">
+        <v>264</v>
+      </c>
+      <c r="AP46" t="s" s="2">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="47" hidden="true">
+      <c r="A47" t="s" s="2">
+        <v>312</v>
+      </c>
+      <c r="B47" t="s" s="2">
+        <v>312</v>
+      </c>
+      <c r="C47" s="2"/>
+      <c r="D47" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="E47" s="2"/>
+      <c r="F47" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="G47" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="H47" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="I47" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="J47" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="K47" t="s" s="2">
+        <v>151</v>
+      </c>
+      <c r="L47" t="s" s="2">
+        <v>266</v>
+      </c>
+      <c r="M47" t="s" s="2">
+        <v>267</v>
+      </c>
+      <c r="N47" t="s" s="2">
+        <v>268</v>
+      </c>
+      <c r="O47" s="2"/>
+      <c r="P47" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Q47" s="2"/>
+      <c r="R47" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="S47" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="T47" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="U47" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="V47" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="W47" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="X47" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Y47" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Z47" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AA47" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AB47" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AC47" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AD47" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AE47" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AF47" t="s" s="2">
+        <v>269</v>
+      </c>
+      <c r="AG47" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH47" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="AI47" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AJ47" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK47" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL47" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM47" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AN47" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AO47" t="s" s="2">
+        <v>132</v>
+      </c>
+      <c r="AP47" t="s" s="2">
         <v>81</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AP43">
+  <autoFilter ref="A1:AP47">
     <filterColumn colId="6">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
@@ -6520,7 +7014,7 @@
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>
-  <conditionalFormatting sqref="A2:AI42">
+  <conditionalFormatting sqref="A2:AI46">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$G2&lt;&gt;"Y"</formula>
     </cfRule>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@9e92668d2464dee0884fd57d6963a29fd01da82b 🚀
</commit_message>
<xml_diff>
--- a/StructureDefinition-Flag.xlsx
+++ b/StructureDefinition-Flag.xlsx
@@ -10,13 +10,13 @@
     <sheet name="Elements" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AP$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AP$61</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1817" uniqueCount="313">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2351" uniqueCount="355">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-09-16T06:13:27+00:00</t>
+    <t>2024-09-20T12:46:12+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -709,6 +709,112 @@
     <t>union(., ./translation)</t>
   </si>
   <si>
+    <t>Flag.category.coding.id</t>
+  </si>
+  <si>
+    <t>Flag.category.coding.extension</t>
+  </si>
+  <si>
+    <t>Flag.category.coding.system</t>
+  </si>
+  <si>
+    <t>Identity of the terminology system</t>
+  </si>
+  <si>
+    <t>The identification of the code system that defines the meaning of the symbol in the code.</t>
+  </si>
+  <si>
+    <t>The URI may be an OID (urn:oid:...) or a UUID (urn:uuid:...).  OIDs and UUIDs SHALL be references to the HL7 OID registry. Otherwise, the URI should come from HL7's list of FHIR defined special URIs or it should de-reference to some definition that establish the system clearly and unambiguously.</t>
+  </si>
+  <si>
+    <t>Need to be unambiguous about the source of the definition of the symbol.</t>
+  </si>
+  <si>
+    <t>Coding.system</t>
+  </si>
+  <si>
+    <t>./codeSystem</t>
+  </si>
+  <si>
+    <t>Flag.category.coding.version</t>
+  </si>
+  <si>
+    <t>Version of the system - if relevant</t>
+  </si>
+  <si>
+    <t>The version of the code system which was used when choosing this code. Note that a well-maintained code system does not need the version reported, because the meaning of codes is consistent across versions. However this cannot consistently be assured. and when the meaning is not guaranteed to be consistent, the version SHOULD be exchanged.</t>
+  </si>
+  <si>
+    <t>Where the terminology does not clearly define what string should be used to identify code system versions, the recommendation is to use the date (expressed in FHIR date format) on which that version was officially published as the version date.</t>
+  </si>
+  <si>
+    <t>Coding.version</t>
+  </si>
+  <si>
+    <t>./codeSystemVersion</t>
+  </si>
+  <si>
+    <t>Flag.category.coding.code</t>
+  </si>
+  <si>
+    <t>Symbol in syntax defined by the system</t>
+  </si>
+  <si>
+    <t>A symbol in syntax defined by the system. The symbol may be a predefined code or an expression in a syntax defined by the coding system (e.g. post-coordination).</t>
+  </si>
+  <si>
+    <t>Need to refer to a particular code in the system.</t>
+  </si>
+  <si>
+    <t>Coding.code</t>
+  </si>
+  <si>
+    <t>./code</t>
+  </si>
+  <si>
+    <t>Flag.category.coding.display</t>
+  </si>
+  <si>
+    <t>Representation defined by the system</t>
+  </si>
+  <si>
+    <t>A representation of the meaning of the code in the system, following the rules of the system.</t>
+  </si>
+  <si>
+    <t>Need to be able to carry a human-readable meaning of the code for readers that do not know  the system.</t>
+  </si>
+  <si>
+    <t>Coding.display</t>
+  </si>
+  <si>
+    <t>CV.displayName</t>
+  </si>
+  <si>
+    <t>Flag.category.coding.userSelected</t>
+  </si>
+  <si>
+    <t xml:space="preserve">boolean
+</t>
+  </si>
+  <si>
+    <t>If this coding was chosen directly by the user</t>
+  </si>
+  <si>
+    <t>Indicates that this coding was chosen by a user directly - i.e. off a pick list of available items (codes or displays).</t>
+  </si>
+  <si>
+    <t>Amongst a set of alternatives, a directly chosen code is the most appropriate starting point for new translations. There is some ambiguity about what exactly 'directly chosen' implies, and trading partner agreement may be needed to clarify the use of this element and its consequences more completely.</t>
+  </si>
+  <si>
+    <t>This has been identified as a clinical safety criterium - that this exact system/code pair was chosen explicitly, rather than inferred by the system based on some rules or language processing.</t>
+  </si>
+  <si>
+    <t>Coding.userSelected</t>
+  </si>
+  <si>
+    <t>CD.codingRationale</t>
+  </si>
+  <si>
     <t>Flag.category.text</t>
   </si>
   <si>
@@ -775,6 +881,27 @@
   </si>
   <si>
     <t>Flag.code.coding</t>
+  </si>
+  <si>
+    <t>Flag.code.coding.id</t>
+  </si>
+  <si>
+    <t>Flag.code.coding.extension</t>
+  </si>
+  <si>
+    <t>Flag.code.coding.system</t>
+  </si>
+  <si>
+    <t>Flag.code.coding.version</t>
+  </si>
+  <si>
+    <t>Flag.code.coding.code</t>
+  </si>
+  <si>
+    <t>Flag.code.coding.display</t>
+  </si>
+  <si>
+    <t>Flag.code.coding.userSelected</t>
   </si>
   <si>
     <t>Flag.code.text</t>
@@ -1333,11 +1460,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AP47"/>
+  <dimension ref="A1:AP61"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="61.9609375" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="29.39453125" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="32.8203125" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="18.015625" customWidth="true" bestFit="true" hidden="true"/>
     <col min="4" max="4" width="39.9140625" customWidth="true" bestFit="true" hidden="true"/>
     <col min="5" max="5" width="6.77734375" customWidth="true" bestFit="true"/>
@@ -3914,29 +4041,25 @@
         <v>89</v>
       </c>
       <c r="H22" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="I22" t="s" s="2">
         <v>81</v>
       </c>
       <c r="J22" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="K22" t="s" s="2">
         <v>151</v>
       </c>
       <c r="L22" t="s" s="2">
-        <v>220</v>
+        <v>152</v>
       </c>
       <c r="M22" t="s" s="2">
-        <v>221</v>
-      </c>
-      <c r="N22" t="s" s="2">
-        <v>222</v>
-      </c>
-      <c r="O22" t="s" s="2">
-        <v>223</v>
-      </c>
+        <v>153</v>
+      </c>
+      <c r="N22" s="2"/>
+      <c r="O22" s="2"/>
       <c r="P22" t="s" s="2">
         <v>81</v>
       </c>
@@ -3984,7 +4107,7 @@
         <v>81</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>224</v>
+        <v>154</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>79</v>
@@ -4011,7 +4134,7 @@
         <v>81</v>
       </c>
       <c r="AO22" t="s" s="2">
-        <v>225</v>
+        <v>155</v>
       </c>
       <c r="AP22" t="s" s="2">
         <v>81</v>
@@ -4019,21 +4142,21 @@
     </row>
     <row r="23" hidden="true">
       <c r="A23" t="s" s="2">
-        <v>226</v>
+        <v>220</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>226</v>
+        <v>220</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
-        <v>227</v>
+        <v>158</v>
       </c>
       <c r="E23" s="2"/>
       <c r="F23" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="G23" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="H23" t="s" s="2">
         <v>81</v>
@@ -4042,19 +4165,19 @@
         <v>81</v>
       </c>
       <c r="J23" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="K23" t="s" s="2">
-        <v>201</v>
+        <v>134</v>
       </c>
       <c r="L23" t="s" s="2">
-        <v>228</v>
+        <v>159</v>
       </c>
       <c r="M23" t="s" s="2">
-        <v>229</v>
+        <v>160</v>
       </c>
       <c r="N23" t="s" s="2">
-        <v>230</v>
+        <v>161</v>
       </c>
       <c r="O23" s="2"/>
       <c r="P23" t="s" s="2">
@@ -4068,7 +4191,7 @@
         <v>81</v>
       </c>
       <c r="T23" t="s" s="2">
-        <v>231</v>
+        <v>81</v>
       </c>
       <c r="U23" t="s" s="2">
         <v>81</v>
@@ -4080,35 +4203,37 @@
         <v>81</v>
       </c>
       <c r="X23" t="s" s="2">
-        <v>112</v>
-      </c>
-      <c r="Y23" s="2"/>
+        <v>81</v>
+      </c>
+      <c r="Y23" t="s" s="2">
+        <v>81</v>
+      </c>
       <c r="Z23" t="s" s="2">
-        <v>232</v>
+        <v>81</v>
       </c>
       <c r="AA23" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AB23" t="s" s="2">
-        <v>81</v>
+        <v>137</v>
       </c>
       <c r="AC23" t="s" s="2">
-        <v>81</v>
+        <v>162</v>
       </c>
       <c r="AD23" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AE23" t="s" s="2">
-        <v>81</v>
+        <v>138</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>226</v>
+        <v>163</v>
       </c>
       <c r="AG23" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="AH23" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="AI23" t="s" s="2">
         <v>81</v>
@@ -4117,30 +4242,30 @@
         <v>81</v>
       </c>
       <c r="AK23" t="s" s="2">
-        <v>233</v>
+        <v>81</v>
       </c>
       <c r="AL23" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AM23" t="s" s="2">
-        <v>233</v>
+        <v>81</v>
       </c>
       <c r="AN23" t="s" s="2">
-        <v>233</v>
+        <v>81</v>
       </c>
       <c r="AO23" t="s" s="2">
-        <v>234</v>
+        <v>155</v>
       </c>
       <c r="AP23" t="s" s="2">
-        <v>235</v>
+        <v>81</v>
       </c>
     </row>
     <row r="24" hidden="true">
       <c r="A24" t="s" s="2">
-        <v>236</v>
+        <v>221</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>236</v>
+        <v>221</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -4160,19 +4285,23 @@
         <v>81</v>
       </c>
       <c r="J24" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="K24" t="s" s="2">
-        <v>151</v>
+        <v>102</v>
       </c>
       <c r="L24" t="s" s="2">
-        <v>152</v>
+        <v>222</v>
       </c>
       <c r="M24" t="s" s="2">
-        <v>153</v>
-      </c>
-      <c r="N24" s="2"/>
-      <c r="O24" s="2"/>
+        <v>223</v>
+      </c>
+      <c r="N24" t="s" s="2">
+        <v>224</v>
+      </c>
+      <c r="O24" t="s" s="2">
+        <v>225</v>
+      </c>
       <c r="P24" t="s" s="2">
         <v>81</v>
       </c>
@@ -4220,7 +4349,7 @@
         <v>81</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>154</v>
+        <v>226</v>
       </c>
       <c r="AG24" t="s" s="2">
         <v>79</v>
@@ -4247,7 +4376,7 @@
         <v>81</v>
       </c>
       <c r="AO24" t="s" s="2">
-        <v>155</v>
+        <v>227</v>
       </c>
       <c r="AP24" t="s" s="2">
         <v>81</v>
@@ -4255,21 +4384,21 @@
     </row>
     <row r="25" hidden="true">
       <c r="A25" t="s" s="2">
-        <v>237</v>
+        <v>228</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>237</v>
+        <v>228</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
-        <v>158</v>
+        <v>81</v>
       </c>
       <c r="E25" s="2"/>
       <c r="F25" t="s" s="2">
         <v>79</v>
       </c>
       <c r="G25" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="H25" t="s" s="2">
         <v>81</v>
@@ -4278,19 +4407,19 @@
         <v>81</v>
       </c>
       <c r="J25" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="K25" t="s" s="2">
-        <v>134</v>
+        <v>151</v>
       </c>
       <c r="L25" t="s" s="2">
-        <v>159</v>
+        <v>229</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>160</v>
+        <v>230</v>
       </c>
       <c r="N25" t="s" s="2">
-        <v>161</v>
+        <v>231</v>
       </c>
       <c r="O25" s="2"/>
       <c r="P25" t="s" s="2">
@@ -4328,25 +4457,25 @@
         <v>81</v>
       </c>
       <c r="AB25" t="s" s="2">
-        <v>137</v>
+        <v>81</v>
       </c>
       <c r="AC25" t="s" s="2">
-        <v>162</v>
+        <v>81</v>
       </c>
       <c r="AD25" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AE25" t="s" s="2">
-        <v>138</v>
+        <v>81</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>163</v>
+        <v>232</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH25" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="AI25" t="s" s="2">
         <v>81</v>
@@ -4367,7 +4496,7 @@
         <v>81</v>
       </c>
       <c r="AO25" t="s" s="2">
-        <v>155</v>
+        <v>233</v>
       </c>
       <c r="AP25" t="s" s="2">
         <v>81</v>
@@ -4375,10 +4504,10 @@
     </row>
     <row r="26" hidden="true">
       <c r="A26" t="s" s="2">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
@@ -4389,7 +4518,7 @@
         <v>79</v>
       </c>
       <c r="G26" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="H26" t="s" s="2">
         <v>81</v>
@@ -4401,19 +4530,17 @@
         <v>90</v>
       </c>
       <c r="K26" t="s" s="2">
-        <v>212</v>
+        <v>108</v>
       </c>
       <c r="L26" t="s" s="2">
-        <v>213</v>
+        <v>235</v>
       </c>
       <c r="M26" t="s" s="2">
-        <v>214</v>
-      </c>
-      <c r="N26" t="s" s="2">
-        <v>215</v>
-      </c>
+        <v>236</v>
+      </c>
+      <c r="N26" s="2"/>
       <c r="O26" t="s" s="2">
-        <v>216</v>
+        <v>237</v>
       </c>
       <c r="P26" t="s" s="2">
         <v>81</v>
@@ -4462,13 +4589,13 @@
         <v>81</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>217</v>
+        <v>238</v>
       </c>
       <c r="AG26" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH26" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="AI26" t="s" s="2">
         <v>81</v>
@@ -4489,7 +4616,7 @@
         <v>81</v>
       </c>
       <c r="AO26" t="s" s="2">
-        <v>218</v>
+        <v>239</v>
       </c>
       <c r="AP26" t="s" s="2">
         <v>81</v>
@@ -4497,10 +4624,10 @@
     </row>
     <row r="27" hidden="true">
       <c r="A27" t="s" s="2">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
@@ -4526,16 +4653,14 @@
         <v>151</v>
       </c>
       <c r="L27" t="s" s="2">
-        <v>220</v>
+        <v>241</v>
       </c>
       <c r="M27" t="s" s="2">
-        <v>221</v>
-      </c>
-      <c r="N27" t="s" s="2">
-        <v>222</v>
-      </c>
+        <v>242</v>
+      </c>
+      <c r="N27" s="2"/>
       <c r="O27" t="s" s="2">
-        <v>223</v>
+        <v>243</v>
       </c>
       <c r="P27" t="s" s="2">
         <v>81</v>
@@ -4584,7 +4709,7 @@
         <v>81</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>224</v>
+        <v>244</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>79</v>
@@ -4611,7 +4736,7 @@
         <v>81</v>
       </c>
       <c r="AO27" t="s" s="2">
-        <v>225</v>
+        <v>245</v>
       </c>
       <c r="AP27" t="s" s="2">
         <v>81</v>
@@ -4619,10 +4744,10 @@
     </row>
     <row r="28" hidden="true">
       <c r="A28" t="s" s="2">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -4630,7 +4755,7 @@
       </c>
       <c r="E28" s="2"/>
       <c r="F28" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="G28" t="s" s="2">
         <v>89</v>
@@ -4645,16 +4770,20 @@
         <v>90</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>243</v>
-      </c>
-      <c r="N28" s="2"/>
-      <c r="O28" s="2"/>
+        <v>249</v>
+      </c>
+      <c r="N28" t="s" s="2">
+        <v>250</v>
+      </c>
+      <c r="O28" t="s" s="2">
+        <v>251</v>
+      </c>
       <c r="P28" t="s" s="2">
         <v>81</v>
       </c>
@@ -4702,10 +4831,10 @@
         <v>81</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>240</v>
+        <v>252</v>
       </c>
       <c r="AG28" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="AH28" t="s" s="2">
         <v>89</v>
@@ -4729,18 +4858,18 @@
         <v>81</v>
       </c>
       <c r="AO28" t="s" s="2">
-        <v>244</v>
+        <v>253</v>
       </c>
       <c r="AP28" t="s" s="2">
-        <v>245</v>
+        <v>81</v>
       </c>
     </row>
     <row r="29" hidden="true">
       <c r="A29" t="s" s="2">
-        <v>246</v>
+        <v>254</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>246</v>
+        <v>254</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -4754,25 +4883,29 @@
         <v>89</v>
       </c>
       <c r="H29" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="I29" t="s" s="2">
         <v>81</v>
       </c>
       <c r="J29" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="K29" t="s" s="2">
         <v>151</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>152</v>
+        <v>255</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>153</v>
-      </c>
-      <c r="N29" s="2"/>
-      <c r="O29" s="2"/>
+        <v>256</v>
+      </c>
+      <c r="N29" t="s" s="2">
+        <v>257</v>
+      </c>
+      <c r="O29" t="s" s="2">
+        <v>258</v>
+      </c>
       <c r="P29" t="s" s="2">
         <v>81</v>
       </c>
@@ -4820,7 +4953,7 @@
         <v>81</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>154</v>
+        <v>259</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>79</v>
@@ -4847,7 +4980,7 @@
         <v>81</v>
       </c>
       <c r="AO29" t="s" s="2">
-        <v>155</v>
+        <v>260</v>
       </c>
       <c r="AP29" t="s" s="2">
         <v>81</v>
@@ -4855,21 +4988,21 @@
     </row>
     <row r="30" hidden="true">
       <c r="A30" t="s" s="2">
-        <v>247</v>
+        <v>261</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>247</v>
+        <v>261</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
-        <v>81</v>
+        <v>262</v>
       </c>
       <c r="E30" s="2"/>
       <c r="F30" t="s" s="2">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="G30" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="H30" t="s" s="2">
         <v>81</v>
@@ -4878,18 +5011,20 @@
         <v>81</v>
       </c>
       <c r="J30" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>134</v>
+        <v>201</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>135</v>
+        <v>263</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>136</v>
-      </c>
-      <c r="N30" s="2"/>
+        <v>264</v>
+      </c>
+      <c r="N30" t="s" s="2">
+        <v>265</v>
+      </c>
       <c r="O30" s="2"/>
       <c r="P30" t="s" s="2">
         <v>81</v>
@@ -4902,7 +5037,7 @@
         <v>81</v>
       </c>
       <c r="T30" t="s" s="2">
-        <v>81</v>
+        <v>266</v>
       </c>
       <c r="U30" t="s" s="2">
         <v>81</v>
@@ -4914,37 +5049,35 @@
         <v>81</v>
       </c>
       <c r="X30" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="Y30" t="s" s="2">
-        <v>81</v>
-      </c>
+        <v>112</v>
+      </c>
+      <c r="Y30" s="2"/>
       <c r="Z30" t="s" s="2">
-        <v>81</v>
+        <v>267</v>
       </c>
       <c r="AA30" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AB30" t="s" s="2">
-        <v>137</v>
+        <v>81</v>
       </c>
       <c r="AC30" t="s" s="2">
-        <v>162</v>
+        <v>81</v>
       </c>
       <c r="AD30" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AE30" t="s" s="2">
-        <v>138</v>
+        <v>81</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>163</v>
+        <v>261</v>
       </c>
       <c r="AG30" t="s" s="2">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="AH30" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="AI30" t="s" s="2">
         <v>81</v>
@@ -4953,34 +5086,32 @@
         <v>81</v>
       </c>
       <c r="AK30" t="s" s="2">
-        <v>81</v>
+        <v>268</v>
       </c>
       <c r="AL30" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AM30" t="s" s="2">
-        <v>81</v>
+        <v>268</v>
       </c>
       <c r="AN30" t="s" s="2">
-        <v>81</v>
+        <v>268</v>
       </c>
       <c r="AO30" t="s" s="2">
-        <v>81</v>
+        <v>269</v>
       </c>
       <c r="AP30" t="s" s="2">
-        <v>81</v>
+        <v>270</v>
       </c>
     </row>
     <row r="31" hidden="true">
       <c r="A31" t="s" s="2">
-        <v>248</v>
+        <v>271</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>247</v>
-      </c>
-      <c r="C31" t="s" s="2">
-        <v>249</v>
-      </c>
+        <v>271</v>
+      </c>
+      <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
         <v>81</v>
       </c>
@@ -5001,13 +5132,13 @@
         <v>81</v>
       </c>
       <c r="K31" t="s" s="2">
-        <v>250</v>
+        <v>151</v>
       </c>
       <c r="L31" t="s" s="2">
-        <v>251</v>
+        <v>152</v>
       </c>
       <c r="M31" t="s" s="2">
-        <v>252</v>
+        <v>153</v>
       </c>
       <c r="N31" s="2"/>
       <c r="O31" s="2"/>
@@ -5058,13 +5189,13 @@
         <v>81</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>163</v>
+        <v>154</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH31" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="AI31" t="s" s="2">
         <v>81</v>
@@ -5085,7 +5216,7 @@
         <v>81</v>
       </c>
       <c r="AO31" t="s" s="2">
-        <v>132</v>
+        <v>155</v>
       </c>
       <c r="AP31" t="s" s="2">
         <v>81</v>
@@ -5093,21 +5224,21 @@
     </row>
     <row r="32" hidden="true">
       <c r="A32" t="s" s="2">
-        <v>253</v>
+        <v>272</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>253</v>
+        <v>272</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
-        <v>81</v>
+        <v>158</v>
       </c>
       <c r="E32" s="2"/>
       <c r="F32" t="s" s="2">
         <v>79</v>
       </c>
       <c r="G32" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="H32" t="s" s="2">
         <v>81</v>
@@ -5116,19 +5247,19 @@
         <v>81</v>
       </c>
       <c r="J32" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="K32" t="s" s="2">
-        <v>151</v>
+        <v>134</v>
       </c>
       <c r="L32" t="s" s="2">
-        <v>254</v>
+        <v>159</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>255</v>
+        <v>160</v>
       </c>
       <c r="N32" t="s" s="2">
-        <v>256</v>
+        <v>161</v>
       </c>
       <c r="O32" s="2"/>
       <c r="P32" t="s" s="2">
@@ -5166,28 +5297,28 @@
         <v>81</v>
       </c>
       <c r="AB32" t="s" s="2">
-        <v>81</v>
+        <v>137</v>
       </c>
       <c r="AC32" t="s" s="2">
-        <v>81</v>
+        <v>162</v>
       </c>
       <c r="AD32" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AE32" t="s" s="2">
-        <v>81</v>
+        <v>138</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>257</v>
+        <v>163</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH32" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="AI32" t="s" s="2">
-        <v>258</v>
+        <v>81</v>
       </c>
       <c r="AJ32" t="s" s="2">
         <v>81</v>
@@ -5205,7 +5336,7 @@
         <v>81</v>
       </c>
       <c r="AO32" t="s" s="2">
-        <v>132</v>
+        <v>155</v>
       </c>
       <c r="AP32" t="s" s="2">
         <v>81</v>
@@ -5213,10 +5344,10 @@
     </row>
     <row r="33" hidden="true">
       <c r="A33" t="s" s="2">
-        <v>259</v>
+        <v>273</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>259</v>
+        <v>273</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
@@ -5227,7 +5358,7 @@
         <v>79</v>
       </c>
       <c r="G33" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="H33" t="s" s="2">
         <v>81</v>
@@ -5239,18 +5370,20 @@
         <v>90</v>
       </c>
       <c r="K33" t="s" s="2">
-        <v>184</v>
+        <v>212</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>260</v>
+        <v>213</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>261</v>
+        <v>214</v>
       </c>
       <c r="N33" t="s" s="2">
-        <v>262</v>
-      </c>
-      <c r="O33" s="2"/>
+        <v>215</v>
+      </c>
+      <c r="O33" t="s" s="2">
+        <v>216</v>
+      </c>
       <c r="P33" t="s" s="2">
         <v>81</v>
       </c>
@@ -5298,13 +5431,13 @@
         <v>81</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>263</v>
+        <v>217</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH33" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="AI33" t="s" s="2">
         <v>81</v>
@@ -5325,7 +5458,7 @@
         <v>81</v>
       </c>
       <c r="AO33" t="s" s="2">
-        <v>264</v>
+        <v>218</v>
       </c>
       <c r="AP33" t="s" s="2">
         <v>81</v>
@@ -5333,10 +5466,10 @@
     </row>
     <row r="34" hidden="true">
       <c r="A34" t="s" s="2">
-        <v>265</v>
+        <v>274</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>265</v>
+        <v>274</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
@@ -5356,20 +5489,18 @@
         <v>81</v>
       </c>
       <c r="J34" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="K34" t="s" s="2">
         <v>151</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>266</v>
+        <v>152</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>267</v>
-      </c>
-      <c r="N34" t="s" s="2">
-        <v>268</v>
-      </c>
+        <v>153</v>
+      </c>
+      <c r="N34" s="2"/>
       <c r="O34" s="2"/>
       <c r="P34" t="s" s="2">
         <v>81</v>
@@ -5418,7 +5549,7 @@
         <v>81</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>269</v>
+        <v>154</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>79</v>
@@ -5445,7 +5576,7 @@
         <v>81</v>
       </c>
       <c r="AO34" t="s" s="2">
-        <v>132</v>
+        <v>155</v>
       </c>
       <c r="AP34" t="s" s="2">
         <v>81</v>
@@ -5453,21 +5584,21 @@
     </row>
     <row r="35" hidden="true">
       <c r="A35" t="s" s="2">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
-        <v>81</v>
+        <v>158</v>
       </c>
       <c r="E35" s="2"/>
       <c r="F35" t="s" s="2">
         <v>79</v>
       </c>
       <c r="G35" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="H35" t="s" s="2">
         <v>81</v>
@@ -5476,18 +5607,20 @@
         <v>81</v>
       </c>
       <c r="J35" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>271</v>
+        <v>134</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>272</v>
+        <v>159</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>273</v>
-      </c>
-      <c r="N35" s="2"/>
+        <v>160</v>
+      </c>
+      <c r="N35" t="s" s="2">
+        <v>161</v>
+      </c>
       <c r="O35" s="2"/>
       <c r="P35" t="s" s="2">
         <v>81</v>
@@ -5524,25 +5657,25 @@
         <v>81</v>
       </c>
       <c r="AB35" t="s" s="2">
-        <v>81</v>
+        <v>137</v>
       </c>
       <c r="AC35" t="s" s="2">
-        <v>81</v>
+        <v>162</v>
       </c>
       <c r="AD35" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AE35" t="s" s="2">
-        <v>81</v>
+        <v>138</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>270</v>
+        <v>163</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH35" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="AI35" t="s" s="2">
         <v>81</v>
@@ -5563,18 +5696,18 @@
         <v>81</v>
       </c>
       <c r="AO35" t="s" s="2">
-        <v>81</v>
+        <v>155</v>
       </c>
       <c r="AP35" t="s" s="2">
-        <v>274</v>
+        <v>81</v>
       </c>
     </row>
     <row r="36" hidden="true">
       <c r="A36" t="s" s="2">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
@@ -5594,19 +5727,23 @@
         <v>81</v>
       </c>
       <c r="J36" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="K36" t="s" s="2">
-        <v>151</v>
+        <v>102</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>152</v>
+        <v>222</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>153</v>
-      </c>
-      <c r="N36" s="2"/>
-      <c r="O36" s="2"/>
+        <v>223</v>
+      </c>
+      <c r="N36" t="s" s="2">
+        <v>224</v>
+      </c>
+      <c r="O36" t="s" s="2">
+        <v>225</v>
+      </c>
       <c r="P36" t="s" s="2">
         <v>81</v>
       </c>
@@ -5654,7 +5791,7 @@
         <v>81</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>154</v>
+        <v>226</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>79</v>
@@ -5681,7 +5818,7 @@
         <v>81</v>
       </c>
       <c r="AO36" t="s" s="2">
-        <v>155</v>
+        <v>227</v>
       </c>
       <c r="AP36" t="s" s="2">
         <v>81</v>
@@ -5689,21 +5826,21 @@
     </row>
     <row r="37" hidden="true">
       <c r="A37" t="s" s="2">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
-        <v>158</v>
+        <v>81</v>
       </c>
       <c r="E37" s="2"/>
       <c r="F37" t="s" s="2">
         <v>79</v>
       </c>
       <c r="G37" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="H37" t="s" s="2">
         <v>81</v>
@@ -5712,19 +5849,19 @@
         <v>81</v>
       </c>
       <c r="J37" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="K37" t="s" s="2">
-        <v>134</v>
+        <v>151</v>
       </c>
       <c r="L37" t="s" s="2">
-        <v>159</v>
+        <v>229</v>
       </c>
       <c r="M37" t="s" s="2">
-        <v>160</v>
+        <v>230</v>
       </c>
       <c r="N37" t="s" s="2">
-        <v>161</v>
+        <v>231</v>
       </c>
       <c r="O37" s="2"/>
       <c r="P37" t="s" s="2">
@@ -5762,25 +5899,25 @@
         <v>81</v>
       </c>
       <c r="AB37" t="s" s="2">
-        <v>137</v>
+        <v>81</v>
       </c>
       <c r="AC37" t="s" s="2">
-        <v>162</v>
+        <v>81</v>
       </c>
       <c r="AD37" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AE37" t="s" s="2">
-        <v>138</v>
+        <v>81</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>163</v>
+        <v>232</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH37" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="AI37" t="s" s="2">
         <v>81</v>
@@ -5801,7 +5938,7 @@
         <v>81</v>
       </c>
       <c r="AO37" t="s" s="2">
-        <v>155</v>
+        <v>233</v>
       </c>
       <c r="AP37" t="s" s="2">
         <v>81</v>
@@ -5809,14 +5946,14 @@
     </row>
     <row r="38" hidden="true">
       <c r="A38" t="s" s="2">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
-        <v>278</v>
+        <v>81</v>
       </c>
       <c r="E38" s="2"/>
       <c r="F38" t="s" s="2">
@@ -5826,7 +5963,7 @@
         <v>89</v>
       </c>
       <c r="H38" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="I38" t="s" s="2">
         <v>81</v>
@@ -5835,18 +5972,18 @@
         <v>90</v>
       </c>
       <c r="K38" t="s" s="2">
-        <v>279</v>
+        <v>108</v>
       </c>
       <c r="L38" t="s" s="2">
-        <v>280</v>
+        <v>235</v>
       </c>
       <c r="M38" t="s" s="2">
-        <v>281</v>
-      </c>
-      <c r="N38" t="s" s="2">
-        <v>282</v>
-      </c>
-      <c r="O38" s="2"/>
+        <v>236</v>
+      </c>
+      <c r="N38" s="2"/>
+      <c r="O38" t="s" s="2">
+        <v>237</v>
+      </c>
       <c r="P38" t="s" s="2">
         <v>81</v>
       </c>
@@ -5858,7 +5995,7 @@
         <v>81</v>
       </c>
       <c r="T38" t="s" s="2">
-        <v>283</v>
+        <v>81</v>
       </c>
       <c r="U38" t="s" s="2">
         <v>81</v>
@@ -5894,7 +6031,7 @@
         <v>81</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>284</v>
+        <v>238</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>79</v>
@@ -5903,25 +6040,25 @@
         <v>89</v>
       </c>
       <c r="AI38" t="s" s="2">
-        <v>285</v>
+        <v>81</v>
       </c>
       <c r="AJ38" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AK38" t="s" s="2">
-        <v>286</v>
+        <v>81</v>
       </c>
       <c r="AL38" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AM38" t="s" s="2">
-        <v>286</v>
+        <v>81</v>
       </c>
       <c r="AN38" t="s" s="2">
-        <v>286</v>
+        <v>81</v>
       </c>
       <c r="AO38" t="s" s="2">
-        <v>287</v>
+        <v>239</v>
       </c>
       <c r="AP38" t="s" s="2">
         <v>81</v>
@@ -5929,10 +6066,10 @@
     </row>
     <row r="39" hidden="true">
       <c r="A39" t="s" s="2">
-        <v>288</v>
+        <v>279</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>288</v>
+        <v>279</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
@@ -5946,7 +6083,7 @@
         <v>89</v>
       </c>
       <c r="H39" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="I39" t="s" s="2">
         <v>81</v>
@@ -5955,24 +6092,22 @@
         <v>90</v>
       </c>
       <c r="K39" t="s" s="2">
-        <v>279</v>
+        <v>151</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>289</v>
+        <v>241</v>
       </c>
       <c r="M39" t="s" s="2">
-        <v>290</v>
-      </c>
-      <c r="N39" t="s" s="2">
-        <v>291</v>
-      </c>
-      <c r="O39" s="2"/>
+        <v>242</v>
+      </c>
+      <c r="N39" s="2"/>
+      <c r="O39" t="s" s="2">
+        <v>243</v>
+      </c>
       <c r="P39" t="s" s="2">
         <v>81</v>
       </c>
-      <c r="Q39" t="s" s="2">
-        <v>292</v>
-      </c>
+      <c r="Q39" s="2"/>
       <c r="R39" t="s" s="2">
         <v>81</v>
       </c>
@@ -6016,7 +6151,7 @@
         <v>81</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>293</v>
+        <v>244</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>79</v>
@@ -6025,7 +6160,7 @@
         <v>89</v>
       </c>
       <c r="AI39" t="s" s="2">
-        <v>285</v>
+        <v>81</v>
       </c>
       <c r="AJ39" t="s" s="2">
         <v>81</v>
@@ -6043,7 +6178,7 @@
         <v>81</v>
       </c>
       <c r="AO39" t="s" s="2">
-        <v>294</v>
+        <v>245</v>
       </c>
       <c r="AP39" t="s" s="2">
         <v>81</v>
@@ -6051,10 +6186,10 @@
     </row>
     <row r="40" hidden="true">
       <c r="A40" t="s" s="2">
-        <v>295</v>
+        <v>280</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>295</v>
+        <v>280</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -6077,18 +6212,20 @@
         <v>90</v>
       </c>
       <c r="K40" t="s" s="2">
-        <v>296</v>
+        <v>247</v>
       </c>
       <c r="L40" t="s" s="2">
-        <v>297</v>
+        <v>248</v>
       </c>
       <c r="M40" t="s" s="2">
-        <v>298</v>
+        <v>249</v>
       </c>
       <c r="N40" t="s" s="2">
-        <v>299</v>
-      </c>
-      <c r="O40" s="2"/>
+        <v>250</v>
+      </c>
+      <c r="O40" t="s" s="2">
+        <v>251</v>
+      </c>
       <c r="P40" t="s" s="2">
         <v>81</v>
       </c>
@@ -6136,7 +6273,7 @@
         <v>81</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>295</v>
+        <v>252</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>79</v>
@@ -6163,18 +6300,18 @@
         <v>81</v>
       </c>
       <c r="AO40" t="s" s="2">
-        <v>81</v>
+        <v>253</v>
       </c>
       <c r="AP40" t="s" s="2">
-        <v>274</v>
+        <v>81</v>
       </c>
     </row>
     <row r="41" hidden="true">
       <c r="A41" t="s" s="2">
-        <v>300</v>
+        <v>281</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>300</v>
+        <v>281</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
@@ -6188,7 +6325,7 @@
         <v>89</v>
       </c>
       <c r="H41" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="I41" t="s" s="2">
         <v>81</v>
@@ -6197,16 +6334,20 @@
         <v>90</v>
       </c>
       <c r="K41" t="s" s="2">
-        <v>301</v>
+        <v>151</v>
       </c>
       <c r="L41" t="s" s="2">
-        <v>302</v>
+        <v>255</v>
       </c>
       <c r="M41" t="s" s="2">
-        <v>303</v>
-      </c>
-      <c r="N41" s="2"/>
-      <c r="O41" s="2"/>
+        <v>256</v>
+      </c>
+      <c r="N41" t="s" s="2">
+        <v>257</v>
+      </c>
+      <c r="O41" t="s" s="2">
+        <v>258</v>
+      </c>
       <c r="P41" t="s" s="2">
         <v>81</v>
       </c>
@@ -6254,7 +6395,7 @@
         <v>81</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>300</v>
+        <v>259</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>79</v>
@@ -6272,7 +6413,7 @@
         <v>81</v>
       </c>
       <c r="AL41" t="s" s="2">
-        <v>304</v>
+        <v>81</v>
       </c>
       <c r="AM41" t="s" s="2">
         <v>81</v>
@@ -6281,18 +6422,18 @@
         <v>81</v>
       </c>
       <c r="AO41" t="s" s="2">
-        <v>305</v>
+        <v>260</v>
       </c>
       <c r="AP41" t="s" s="2">
-        <v>306</v>
+        <v>81</v>
       </c>
     </row>
     <row r="42" hidden="true">
       <c r="A42" t="s" s="2">
-        <v>307</v>
+        <v>282</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>307</v>
+        <v>282</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
@@ -6300,7 +6441,7 @@
       </c>
       <c r="E42" s="2"/>
       <c r="F42" t="s" s="2">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="G42" t="s" s="2">
         <v>89</v>
@@ -6312,16 +6453,16 @@
         <v>81</v>
       </c>
       <c r="J42" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="K42" t="s" s="2">
-        <v>151</v>
+        <v>283</v>
       </c>
       <c r="L42" t="s" s="2">
-        <v>152</v>
+        <v>284</v>
       </c>
       <c r="M42" t="s" s="2">
-        <v>153</v>
+        <v>285</v>
       </c>
       <c r="N42" s="2"/>
       <c r="O42" s="2"/>
@@ -6372,10 +6513,10 @@
         <v>81</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>154</v>
+        <v>282</v>
       </c>
       <c r="AG42" t="s" s="2">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="AH42" t="s" s="2">
         <v>89</v>
@@ -6399,18 +6540,18 @@
         <v>81</v>
       </c>
       <c r="AO42" t="s" s="2">
-        <v>155</v>
+        <v>286</v>
       </c>
       <c r="AP42" t="s" s="2">
-        <v>81</v>
+        <v>287</v>
       </c>
     </row>
     <row r="43" hidden="true">
       <c r="A43" t="s" s="2">
-        <v>308</v>
+        <v>288</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>308</v>
+        <v>288</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
@@ -6421,7 +6562,7 @@
         <v>79</v>
       </c>
       <c r="G43" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="H43" t="s" s="2">
         <v>81</v>
@@ -6433,13 +6574,13 @@
         <v>81</v>
       </c>
       <c r="K43" t="s" s="2">
-        <v>134</v>
+        <v>151</v>
       </c>
       <c r="L43" t="s" s="2">
-        <v>135</v>
+        <v>152</v>
       </c>
       <c r="M43" t="s" s="2">
-        <v>136</v>
+        <v>153</v>
       </c>
       <c r="N43" s="2"/>
       <c r="O43" s="2"/>
@@ -6478,25 +6619,25 @@
         <v>81</v>
       </c>
       <c r="AB43" t="s" s="2">
-        <v>137</v>
+        <v>81</v>
       </c>
       <c r="AC43" t="s" s="2">
-        <v>162</v>
+        <v>81</v>
       </c>
       <c r="AD43" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AE43" t="s" s="2">
-        <v>138</v>
+        <v>81</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>163</v>
+        <v>154</v>
       </c>
       <c r="AG43" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH43" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="AI43" t="s" s="2">
         <v>81</v>
@@ -6517,7 +6658,7 @@
         <v>81</v>
       </c>
       <c r="AO43" t="s" s="2">
-        <v>81</v>
+        <v>155</v>
       </c>
       <c r="AP43" t="s" s="2">
         <v>81</v>
@@ -6525,14 +6666,12 @@
     </row>
     <row r="44" hidden="true">
       <c r="A44" t="s" s="2">
-        <v>309</v>
+        <v>289</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>308</v>
-      </c>
-      <c r="C44" t="s" s="2">
-        <v>249</v>
-      </c>
+        <v>289</v>
+      </c>
+      <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
         <v>81</v>
       </c>
@@ -6541,7 +6680,7 @@
         <v>79</v>
       </c>
       <c r="G44" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="H44" t="s" s="2">
         <v>81</v>
@@ -6553,13 +6692,13 @@
         <v>81</v>
       </c>
       <c r="K44" t="s" s="2">
-        <v>250</v>
+        <v>134</v>
       </c>
       <c r="L44" t="s" s="2">
-        <v>251</v>
+        <v>135</v>
       </c>
       <c r="M44" t="s" s="2">
-        <v>252</v>
+        <v>136</v>
       </c>
       <c r="N44" s="2"/>
       <c r="O44" s="2"/>
@@ -6598,16 +6737,16 @@
         <v>81</v>
       </c>
       <c r="AB44" t="s" s="2">
-        <v>81</v>
+        <v>137</v>
       </c>
       <c r="AC44" t="s" s="2">
-        <v>81</v>
+        <v>162</v>
       </c>
       <c r="AD44" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AE44" t="s" s="2">
-        <v>81</v>
+        <v>138</v>
       </c>
       <c r="AF44" t="s" s="2">
         <v>163</v>
@@ -6637,7 +6776,7 @@
         <v>81</v>
       </c>
       <c r="AO44" t="s" s="2">
-        <v>132</v>
+        <v>81</v>
       </c>
       <c r="AP44" t="s" s="2">
         <v>81</v>
@@ -6645,12 +6784,14 @@
     </row>
     <row r="45" hidden="true">
       <c r="A45" t="s" s="2">
-        <v>310</v>
+        <v>290</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>310</v>
-      </c>
-      <c r="C45" s="2"/>
+        <v>289</v>
+      </c>
+      <c r="C45" t="s" s="2">
+        <v>291</v>
+      </c>
       <c r="D45" t="s" s="2">
         <v>81</v>
       </c>
@@ -6668,20 +6809,18 @@
         <v>81</v>
       </c>
       <c r="J45" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="K45" t="s" s="2">
-        <v>151</v>
+        <v>292</v>
       </c>
       <c r="L45" t="s" s="2">
-        <v>254</v>
+        <v>293</v>
       </c>
       <c r="M45" t="s" s="2">
-        <v>255</v>
-      </c>
-      <c r="N45" t="s" s="2">
-        <v>256</v>
-      </c>
+        <v>294</v>
+      </c>
+      <c r="N45" s="2"/>
       <c r="O45" s="2"/>
       <c r="P45" t="s" s="2">
         <v>81</v>
@@ -6730,16 +6869,16 @@
         <v>81</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>257</v>
+        <v>163</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH45" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="AI45" t="s" s="2">
-        <v>258</v>
+        <v>81</v>
       </c>
       <c r="AJ45" t="s" s="2">
         <v>81</v>
@@ -6765,10 +6904,10 @@
     </row>
     <row r="46" hidden="true">
       <c r="A46" t="s" s="2">
-        <v>311</v>
+        <v>295</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>311</v>
+        <v>295</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
@@ -6791,16 +6930,16 @@
         <v>90</v>
       </c>
       <c r="K46" t="s" s="2">
-        <v>184</v>
+        <v>151</v>
       </c>
       <c r="L46" t="s" s="2">
-        <v>260</v>
+        <v>296</v>
       </c>
       <c r="M46" t="s" s="2">
-        <v>261</v>
+        <v>297</v>
       </c>
       <c r="N46" t="s" s="2">
-        <v>262</v>
+        <v>298</v>
       </c>
       <c r="O46" s="2"/>
       <c r="P46" t="s" s="2">
@@ -6850,7 +6989,7 @@
         <v>81</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>263</v>
+        <v>299</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>79</v>
@@ -6859,7 +6998,7 @@
         <v>89</v>
       </c>
       <c r="AI46" t="s" s="2">
-        <v>81</v>
+        <v>300</v>
       </c>
       <c r="AJ46" t="s" s="2">
         <v>81</v>
@@ -6877,7 +7016,7 @@
         <v>81</v>
       </c>
       <c r="AO46" t="s" s="2">
-        <v>264</v>
+        <v>132</v>
       </c>
       <c r="AP46" t="s" s="2">
         <v>81</v>
@@ -6885,10 +7024,10 @@
     </row>
     <row r="47" hidden="true">
       <c r="A47" t="s" s="2">
-        <v>312</v>
+        <v>301</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>312</v>
+        <v>301</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
@@ -6911,16 +7050,16 @@
         <v>90</v>
       </c>
       <c r="K47" t="s" s="2">
-        <v>151</v>
+        <v>184</v>
       </c>
       <c r="L47" t="s" s="2">
-        <v>266</v>
+        <v>302</v>
       </c>
       <c r="M47" t="s" s="2">
-        <v>267</v>
+        <v>303</v>
       </c>
       <c r="N47" t="s" s="2">
-        <v>268</v>
+        <v>304</v>
       </c>
       <c r="O47" s="2"/>
       <c r="P47" t="s" s="2">
@@ -6970,7 +7109,7 @@
         <v>81</v>
       </c>
       <c r="AF47" t="s" s="2">
-        <v>269</v>
+        <v>305</v>
       </c>
       <c r="AG47" t="s" s="2">
         <v>79</v>
@@ -6997,14 +7136,1686 @@
         <v>81</v>
       </c>
       <c r="AO47" t="s" s="2">
+        <v>306</v>
+      </c>
+      <c r="AP47" t="s" s="2">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="48" hidden="true">
+      <c r="A48" t="s" s="2">
+        <v>307</v>
+      </c>
+      <c r="B48" t="s" s="2">
+        <v>307</v>
+      </c>
+      <c r="C48" s="2"/>
+      <c r="D48" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="E48" s="2"/>
+      <c r="F48" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="G48" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="H48" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="I48" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="J48" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="K48" t="s" s="2">
+        <v>151</v>
+      </c>
+      <c r="L48" t="s" s="2">
+        <v>308</v>
+      </c>
+      <c r="M48" t="s" s="2">
+        <v>309</v>
+      </c>
+      <c r="N48" t="s" s="2">
+        <v>310</v>
+      </c>
+      <c r="O48" s="2"/>
+      <c r="P48" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Q48" s="2"/>
+      <c r="R48" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="S48" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="T48" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="U48" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="V48" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="W48" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="X48" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Y48" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Z48" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AA48" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AB48" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AC48" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AD48" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AE48" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AF48" t="s" s="2">
+        <v>311</v>
+      </c>
+      <c r="AG48" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH48" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="AI48" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AJ48" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK48" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL48" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM48" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AN48" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AO48" t="s" s="2">
         <v>132</v>
       </c>
-      <c r="AP47" t="s" s="2">
+      <c r="AP48" t="s" s="2">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="49" hidden="true">
+      <c r="A49" t="s" s="2">
+        <v>312</v>
+      </c>
+      <c r="B49" t="s" s="2">
+        <v>312</v>
+      </c>
+      <c r="C49" s="2"/>
+      <c r="D49" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="E49" s="2"/>
+      <c r="F49" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="G49" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="H49" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="I49" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="J49" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="K49" t="s" s="2">
+        <v>313</v>
+      </c>
+      <c r="L49" t="s" s="2">
+        <v>314</v>
+      </c>
+      <c r="M49" t="s" s="2">
+        <v>315</v>
+      </c>
+      <c r="N49" s="2"/>
+      <c r="O49" s="2"/>
+      <c r="P49" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Q49" s="2"/>
+      <c r="R49" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="S49" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="T49" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="U49" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="V49" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="W49" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="X49" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Y49" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Z49" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AA49" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AB49" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AC49" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AD49" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AE49" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AF49" t="s" s="2">
+        <v>312</v>
+      </c>
+      <c r="AG49" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH49" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="AI49" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AJ49" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK49" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL49" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM49" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AN49" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AO49" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AP49" t="s" s="2">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="50" hidden="true">
+      <c r="A50" t="s" s="2">
+        <v>317</v>
+      </c>
+      <c r="B50" t="s" s="2">
+        <v>317</v>
+      </c>
+      <c r="C50" s="2"/>
+      <c r="D50" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="E50" s="2"/>
+      <c r="F50" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="G50" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="H50" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="I50" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="J50" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="K50" t="s" s="2">
+        <v>151</v>
+      </c>
+      <c r="L50" t="s" s="2">
+        <v>152</v>
+      </c>
+      <c r="M50" t="s" s="2">
+        <v>153</v>
+      </c>
+      <c r="N50" s="2"/>
+      <c r="O50" s="2"/>
+      <c r="P50" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Q50" s="2"/>
+      <c r="R50" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="S50" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="T50" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="U50" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="V50" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="W50" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="X50" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Y50" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Z50" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AA50" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AB50" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AC50" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AD50" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AE50" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AF50" t="s" s="2">
+        <v>154</v>
+      </c>
+      <c r="AG50" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH50" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="AI50" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AJ50" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK50" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL50" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM50" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AN50" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AO50" t="s" s="2">
+        <v>155</v>
+      </c>
+      <c r="AP50" t="s" s="2">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="51" hidden="true">
+      <c r="A51" t="s" s="2">
+        <v>318</v>
+      </c>
+      <c r="B51" t="s" s="2">
+        <v>318</v>
+      </c>
+      <c r="C51" s="2"/>
+      <c r="D51" t="s" s="2">
+        <v>158</v>
+      </c>
+      <c r="E51" s="2"/>
+      <c r="F51" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="G51" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="H51" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="I51" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="J51" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="K51" t="s" s="2">
+        <v>134</v>
+      </c>
+      <c r="L51" t="s" s="2">
+        <v>159</v>
+      </c>
+      <c r="M51" t="s" s="2">
+        <v>160</v>
+      </c>
+      <c r="N51" t="s" s="2">
+        <v>161</v>
+      </c>
+      <c r="O51" s="2"/>
+      <c r="P51" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Q51" s="2"/>
+      <c r="R51" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="S51" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="T51" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="U51" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="V51" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="W51" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="X51" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Y51" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Z51" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AA51" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AB51" t="s" s="2">
+        <v>137</v>
+      </c>
+      <c r="AC51" t="s" s="2">
+        <v>162</v>
+      </c>
+      <c r="AD51" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AE51" t="s" s="2">
+        <v>138</v>
+      </c>
+      <c r="AF51" t="s" s="2">
+        <v>163</v>
+      </c>
+      <c r="AG51" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH51" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AI51" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AJ51" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK51" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL51" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM51" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AN51" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AO51" t="s" s="2">
+        <v>155</v>
+      </c>
+      <c r="AP51" t="s" s="2">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="52" hidden="true">
+      <c r="A52" t="s" s="2">
+        <v>319</v>
+      </c>
+      <c r="B52" t="s" s="2">
+        <v>319</v>
+      </c>
+      <c r="C52" s="2"/>
+      <c r="D52" t="s" s="2">
+        <v>320</v>
+      </c>
+      <c r="E52" s="2"/>
+      <c r="F52" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="G52" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="H52" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="I52" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="J52" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="K52" t="s" s="2">
+        <v>321</v>
+      </c>
+      <c r="L52" t="s" s="2">
+        <v>322</v>
+      </c>
+      <c r="M52" t="s" s="2">
+        <v>323</v>
+      </c>
+      <c r="N52" t="s" s="2">
+        <v>324</v>
+      </c>
+      <c r="O52" s="2"/>
+      <c r="P52" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Q52" s="2"/>
+      <c r="R52" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="S52" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="T52" t="s" s="2">
+        <v>325</v>
+      </c>
+      <c r="U52" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="V52" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="W52" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="X52" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Y52" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Z52" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AA52" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AB52" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AC52" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AD52" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AE52" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AF52" t="s" s="2">
+        <v>326</v>
+      </c>
+      <c r="AG52" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH52" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="AI52" t="s" s="2">
+        <v>327</v>
+      </c>
+      <c r="AJ52" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK52" t="s" s="2">
+        <v>328</v>
+      </c>
+      <c r="AL52" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM52" t="s" s="2">
+        <v>328</v>
+      </c>
+      <c r="AN52" t="s" s="2">
+        <v>328</v>
+      </c>
+      <c r="AO52" t="s" s="2">
+        <v>329</v>
+      </c>
+      <c r="AP52" t="s" s="2">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="53" hidden="true">
+      <c r="A53" t="s" s="2">
+        <v>330</v>
+      </c>
+      <c r="B53" t="s" s="2">
+        <v>330</v>
+      </c>
+      <c r="C53" s="2"/>
+      <c r="D53" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="E53" s="2"/>
+      <c r="F53" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="G53" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="H53" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="I53" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="J53" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="K53" t="s" s="2">
+        <v>321</v>
+      </c>
+      <c r="L53" t="s" s="2">
+        <v>331</v>
+      </c>
+      <c r="M53" t="s" s="2">
+        <v>332</v>
+      </c>
+      <c r="N53" t="s" s="2">
+        <v>333</v>
+      </c>
+      <c r="O53" s="2"/>
+      <c r="P53" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Q53" t="s" s="2">
+        <v>334</v>
+      </c>
+      <c r="R53" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="S53" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="T53" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="U53" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="V53" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="W53" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="X53" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Y53" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Z53" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AA53" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AB53" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AC53" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AD53" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AE53" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AF53" t="s" s="2">
+        <v>335</v>
+      </c>
+      <c r="AG53" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH53" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="AI53" t="s" s="2">
+        <v>327</v>
+      </c>
+      <c r="AJ53" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK53" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL53" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM53" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AN53" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AO53" t="s" s="2">
+        <v>336</v>
+      </c>
+      <c r="AP53" t="s" s="2">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="54" hidden="true">
+      <c r="A54" t="s" s="2">
+        <v>337</v>
+      </c>
+      <c r="B54" t="s" s="2">
+        <v>337</v>
+      </c>
+      <c r="C54" s="2"/>
+      <c r="D54" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="E54" s="2"/>
+      <c r="F54" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="G54" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="H54" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="I54" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="J54" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="K54" t="s" s="2">
+        <v>338</v>
+      </c>
+      <c r="L54" t="s" s="2">
+        <v>339</v>
+      </c>
+      <c r="M54" t="s" s="2">
+        <v>340</v>
+      </c>
+      <c r="N54" t="s" s="2">
+        <v>341</v>
+      </c>
+      <c r="O54" s="2"/>
+      <c r="P54" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Q54" s="2"/>
+      <c r="R54" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="S54" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="T54" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="U54" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="V54" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="W54" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="X54" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Y54" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Z54" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AA54" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AB54" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AC54" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AD54" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AE54" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AF54" t="s" s="2">
+        <v>337</v>
+      </c>
+      <c r="AG54" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH54" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="AI54" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AJ54" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK54" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL54" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM54" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AN54" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AO54" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AP54" t="s" s="2">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="55" hidden="true">
+      <c r="A55" t="s" s="2">
+        <v>342</v>
+      </c>
+      <c r="B55" t="s" s="2">
+        <v>342</v>
+      </c>
+      <c r="C55" s="2"/>
+      <c r="D55" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="E55" s="2"/>
+      <c r="F55" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="G55" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="H55" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="I55" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="J55" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="K55" t="s" s="2">
+        <v>343</v>
+      </c>
+      <c r="L55" t="s" s="2">
+        <v>344</v>
+      </c>
+      <c r="M55" t="s" s="2">
+        <v>345</v>
+      </c>
+      <c r="N55" s="2"/>
+      <c r="O55" s="2"/>
+      <c r="P55" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Q55" s="2"/>
+      <c r="R55" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="S55" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="T55" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="U55" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="V55" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="W55" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="X55" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Y55" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Z55" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AA55" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AB55" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AC55" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AD55" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AE55" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AF55" t="s" s="2">
+        <v>342</v>
+      </c>
+      <c r="AG55" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH55" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="AI55" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AJ55" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK55" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL55" t="s" s="2">
+        <v>346</v>
+      </c>
+      <c r="AM55" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AN55" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AO55" t="s" s="2">
+        <v>347</v>
+      </c>
+      <c r="AP55" t="s" s="2">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="56" hidden="true">
+      <c r="A56" t="s" s="2">
+        <v>349</v>
+      </c>
+      <c r="B56" t="s" s="2">
+        <v>349</v>
+      </c>
+      <c r="C56" s="2"/>
+      <c r="D56" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="E56" s="2"/>
+      <c r="F56" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="G56" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="H56" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="I56" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="J56" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="K56" t="s" s="2">
+        <v>151</v>
+      </c>
+      <c r="L56" t="s" s="2">
+        <v>152</v>
+      </c>
+      <c r="M56" t="s" s="2">
+        <v>153</v>
+      </c>
+      <c r="N56" s="2"/>
+      <c r="O56" s="2"/>
+      <c r="P56" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Q56" s="2"/>
+      <c r="R56" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="S56" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="T56" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="U56" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="V56" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="W56" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="X56" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Y56" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Z56" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AA56" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AB56" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AC56" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AD56" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AE56" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AF56" t="s" s="2">
+        <v>154</v>
+      </c>
+      <c r="AG56" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH56" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="AI56" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AJ56" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK56" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL56" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM56" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AN56" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AO56" t="s" s="2">
+        <v>155</v>
+      </c>
+      <c r="AP56" t="s" s="2">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="57" hidden="true">
+      <c r="A57" t="s" s="2">
+        <v>350</v>
+      </c>
+      <c r="B57" t="s" s="2">
+        <v>350</v>
+      </c>
+      <c r="C57" s="2"/>
+      <c r="D57" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="E57" s="2"/>
+      <c r="F57" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="G57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="H57" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="I57" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="J57" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="K57" t="s" s="2">
+        <v>134</v>
+      </c>
+      <c r="L57" t="s" s="2">
+        <v>135</v>
+      </c>
+      <c r="M57" t="s" s="2">
+        <v>136</v>
+      </c>
+      <c r="N57" s="2"/>
+      <c r="O57" s="2"/>
+      <c r="P57" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Q57" s="2"/>
+      <c r="R57" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="S57" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="T57" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="U57" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="V57" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="W57" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="X57" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Y57" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Z57" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AA57" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AB57" t="s" s="2">
+        <v>137</v>
+      </c>
+      <c r="AC57" t="s" s="2">
+        <v>162</v>
+      </c>
+      <c r="AD57" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AE57" t="s" s="2">
+        <v>138</v>
+      </c>
+      <c r="AF57" t="s" s="2">
+        <v>163</v>
+      </c>
+      <c r="AG57" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH57" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AI57" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AJ57" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK57" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL57" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM57" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AN57" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AO57" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AP57" t="s" s="2">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="58" hidden="true">
+      <c r="A58" t="s" s="2">
+        <v>351</v>
+      </c>
+      <c r="B58" t="s" s="2">
+        <v>350</v>
+      </c>
+      <c r="C58" t="s" s="2">
+        <v>291</v>
+      </c>
+      <c r="D58" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="E58" s="2"/>
+      <c r="F58" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="G58" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="H58" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="I58" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="J58" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="K58" t="s" s="2">
+        <v>292</v>
+      </c>
+      <c r="L58" t="s" s="2">
+        <v>293</v>
+      </c>
+      <c r="M58" t="s" s="2">
+        <v>294</v>
+      </c>
+      <c r="N58" s="2"/>
+      <c r="O58" s="2"/>
+      <c r="P58" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Q58" s="2"/>
+      <c r="R58" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="S58" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="T58" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="U58" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="V58" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="W58" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="X58" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Y58" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Z58" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AA58" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AB58" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AC58" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AD58" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AE58" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AF58" t="s" s="2">
+        <v>163</v>
+      </c>
+      <c r="AG58" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH58" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AI58" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AJ58" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK58" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL58" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM58" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AN58" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AO58" t="s" s="2">
+        <v>132</v>
+      </c>
+      <c r="AP58" t="s" s="2">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="59" hidden="true">
+      <c r="A59" t="s" s="2">
+        <v>352</v>
+      </c>
+      <c r="B59" t="s" s="2">
+        <v>352</v>
+      </c>
+      <c r="C59" s="2"/>
+      <c r="D59" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="E59" s="2"/>
+      <c r="F59" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="G59" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="H59" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="I59" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="J59" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="K59" t="s" s="2">
+        <v>151</v>
+      </c>
+      <c r="L59" t="s" s="2">
+        <v>296</v>
+      </c>
+      <c r="M59" t="s" s="2">
+        <v>297</v>
+      </c>
+      <c r="N59" t="s" s="2">
+        <v>298</v>
+      </c>
+      <c r="O59" s="2"/>
+      <c r="P59" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Q59" s="2"/>
+      <c r="R59" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="S59" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="T59" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="U59" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="V59" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="W59" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="X59" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Y59" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Z59" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AA59" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AB59" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AC59" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AD59" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AE59" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AF59" t="s" s="2">
+        <v>299</v>
+      </c>
+      <c r="AG59" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH59" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="AI59" t="s" s="2">
+        <v>300</v>
+      </c>
+      <c r="AJ59" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK59" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL59" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM59" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AN59" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AO59" t="s" s="2">
+        <v>132</v>
+      </c>
+      <c r="AP59" t="s" s="2">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="60" hidden="true">
+      <c r="A60" t="s" s="2">
+        <v>353</v>
+      </c>
+      <c r="B60" t="s" s="2">
+        <v>353</v>
+      </c>
+      <c r="C60" s="2"/>
+      <c r="D60" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="E60" s="2"/>
+      <c r="F60" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="G60" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="H60" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="I60" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="J60" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="K60" t="s" s="2">
+        <v>184</v>
+      </c>
+      <c r="L60" t="s" s="2">
+        <v>302</v>
+      </c>
+      <c r="M60" t="s" s="2">
+        <v>303</v>
+      </c>
+      <c r="N60" t="s" s="2">
+        <v>304</v>
+      </c>
+      <c r="O60" s="2"/>
+      <c r="P60" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Q60" s="2"/>
+      <c r="R60" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="S60" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="T60" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="U60" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="V60" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="W60" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="X60" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Y60" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Z60" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AA60" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AB60" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AC60" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AD60" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AE60" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AF60" t="s" s="2">
+        <v>305</v>
+      </c>
+      <c r="AG60" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH60" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="AI60" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AJ60" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK60" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL60" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM60" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AN60" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AO60" t="s" s="2">
+        <v>306</v>
+      </c>
+      <c r="AP60" t="s" s="2">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="61" hidden="true">
+      <c r="A61" t="s" s="2">
+        <v>354</v>
+      </c>
+      <c r="B61" t="s" s="2">
+        <v>354</v>
+      </c>
+      <c r="C61" s="2"/>
+      <c r="D61" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="E61" s="2"/>
+      <c r="F61" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="G61" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="H61" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="I61" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="J61" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="K61" t="s" s="2">
+        <v>151</v>
+      </c>
+      <c r="L61" t="s" s="2">
+        <v>308</v>
+      </c>
+      <c r="M61" t="s" s="2">
+        <v>309</v>
+      </c>
+      <c r="N61" t="s" s="2">
+        <v>310</v>
+      </c>
+      <c r="O61" s="2"/>
+      <c r="P61" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Q61" s="2"/>
+      <c r="R61" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="S61" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="T61" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="U61" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="V61" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="W61" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="X61" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Y61" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Z61" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AA61" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AB61" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AC61" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AD61" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AE61" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AF61" t="s" s="2">
+        <v>311</v>
+      </c>
+      <c r="AG61" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH61" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="AI61" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AJ61" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK61" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL61" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM61" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AN61" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AO61" t="s" s="2">
+        <v>132</v>
+      </c>
+      <c r="AP61" t="s" s="2">
         <v>81</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AP47">
+  <autoFilter ref="A1:AP61">
     <filterColumn colId="6">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
@@ -7014,7 +8825,7 @@
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>
-  <conditionalFormatting sqref="A2:AI46">
+  <conditionalFormatting sqref="A2:AI60">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$G2&lt;&gt;"Y"</formula>
     </cfRule>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@441abad856144f92dec004589b5dac4064ee84e6 🚀
</commit_message>
<xml_diff>
--- a/StructureDefinition-Flag.xlsx
+++ b/StructureDefinition-Flag.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2351" uniqueCount="355">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2351" uniqueCount="353">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-11-04T07:59:20+00:00</t>
+    <t>2024-11-06T14:12:43+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -459,19 +459,14 @@
     <t>ConcernReference</t>
   </si>
   <si>
-    <t xml:space="preserve">Conditie
-</t>
-  </si>
-  <si>
     <t xml:space="preserve">Extension {flag-detail}
 </t>
   </si>
   <si>
-    <t>Condition</t>
-  </si>
-  <si>
-    <t>The patient’s health problem or condition that is the subject of the alert. This could involve a patient’s episode of care, problem, condition or diagnosis that is seen as a contraindication in prescribing medication or which has to be taken into account when shaping diagnostic and therapeutic policy. This can be in the patient’s own interest, or it can involve a problem or disorder that can make the patient a risk to their surroundings, such as an infection hazard. These are references to conditions included on the patient’s problem list.
-If there is a contraindication, the code system G-Standard Contraindications (Table 40) from the ProblemNameCodeList of the ConcernTransfer information model should be used.</t>
+    <t>Resource with details for flag</t>
+  </si>
+  <si>
+    <t>Points to the Observation, AllergyIntolerance or other record that provides additional supporting information about this flag.</t>
   </si>
   <si>
     <t xml:space="preserve">ele-1
@@ -480,9 +475,6 @@
   <si>
     <t>ele-1:All FHIR elements must have a @value or children {hasValue() | (children().count() &gt; id.count())}
 ext-1:Must have either extensions or value[x], not both {extension.exists() != value.exists()}</t>
-  </si>
-  <si>
-    <t>NL-CM:8.3.3</t>
   </si>
   <si>
     <t>Flag.extension:ConcernReference.id</t>
@@ -2597,7 +2589,7 @@
         <v>141</v>
       </c>
       <c r="D10" t="s" s="2">
-        <v>142</v>
+        <v>81</v>
       </c>
       <c r="E10" s="2"/>
       <c r="F10" t="s" s="2">
@@ -2607,7 +2599,7 @@
         <v>89</v>
       </c>
       <c r="H10" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="I10" t="s" s="2">
         <v>81</v>
@@ -2616,13 +2608,13 @@
         <v>81</v>
       </c>
       <c r="K10" t="s" s="2">
+        <v>142</v>
+      </c>
+      <c r="L10" t="s" s="2">
         <v>143</v>
       </c>
-      <c r="L10" t="s" s="2">
+      <c r="M10" t="s" s="2">
         <v>144</v>
-      </c>
-      <c r="M10" t="s" s="2">
-        <v>145</v>
       </c>
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
@@ -2682,22 +2674,22 @@
         <v>80</v>
       </c>
       <c r="AI10" t="s" s="2">
+        <v>145</v>
+      </c>
+      <c r="AJ10" t="s" s="2">
         <v>146</v>
       </c>
-      <c r="AJ10" t="s" s="2">
-        <v>147</v>
-      </c>
       <c r="AK10" t="s" s="2">
-        <v>148</v>
+        <v>81</v>
       </c>
       <c r="AL10" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AM10" t="s" s="2">
-        <v>148</v>
+        <v>81</v>
       </c>
       <c r="AN10" t="s" s="2">
-        <v>148</v>
+        <v>81</v>
       </c>
       <c r="AO10" t="s" s="2">
         <v>81</v>
@@ -2708,10 +2700,10 @@
     </row>
     <row r="11" hidden="true">
       <c r="A11" t="s" s="2">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B11" t="s" s="2">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" t="s" s="2">
@@ -2734,13 +2726,13 @@
         <v>81</v>
       </c>
       <c r="K11" t="s" s="2">
+        <v>149</v>
+      </c>
+      <c r="L11" t="s" s="2">
+        <v>150</v>
+      </c>
+      <c r="M11" t="s" s="2">
         <v>151</v>
-      </c>
-      <c r="L11" t="s" s="2">
-        <v>152</v>
-      </c>
-      <c r="M11" t="s" s="2">
-        <v>153</v>
       </c>
       <c r="N11" s="2"/>
       <c r="O11" s="2"/>
@@ -2791,7 +2783,7 @@
         <v>81</v>
       </c>
       <c r="AF11" t="s" s="2">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="AG11" t="s" s="2">
         <v>79</v>
@@ -2818,7 +2810,7 @@
         <v>81</v>
       </c>
       <c r="AO11" t="s" s="2">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="AP11" t="s" s="2">
         <v>81</v>
@@ -2826,14 +2818,14 @@
     </row>
     <row r="12" hidden="true">
       <c r="A12" t="s" s="2">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" t="s" s="2">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="E12" s="2"/>
       <c r="F12" t="s" s="2">
@@ -2855,13 +2847,13 @@
         <v>134</v>
       </c>
       <c r="L12" t="s" s="2">
+        <v>157</v>
+      </c>
+      <c r="M12" t="s" s="2">
+        <v>158</v>
+      </c>
+      <c r="N12" t="s" s="2">
         <v>159</v>
-      </c>
-      <c r="M12" t="s" s="2">
-        <v>160</v>
-      </c>
-      <c r="N12" t="s" s="2">
-        <v>161</v>
       </c>
       <c r="O12" s="2"/>
       <c r="P12" t="s" s="2">
@@ -2902,7 +2894,7 @@
         <v>137</v>
       </c>
       <c r="AC12" t="s" s="2">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="AD12" t="s" s="2">
         <v>81</v>
@@ -2911,7 +2903,7 @@
         <v>138</v>
       </c>
       <c r="AF12" t="s" s="2">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="AG12" t="s" s="2">
         <v>79</v>
@@ -2938,7 +2930,7 @@
         <v>81</v>
       </c>
       <c r="AO12" t="s" s="2">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="AP12" t="s" s="2">
         <v>81</v>
@@ -2946,10 +2938,10 @@
     </row>
     <row r="13" hidden="true">
       <c r="A13" t="s" s="2">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" t="s" s="2">
@@ -2975,13 +2967,13 @@
         <v>102</v>
       </c>
       <c r="L13" t="s" s="2">
+        <v>164</v>
+      </c>
+      <c r="M13" t="s" s="2">
+        <v>165</v>
+      </c>
+      <c r="N13" t="s" s="2">
         <v>166</v>
-      </c>
-      <c r="M13" t="s" s="2">
-        <v>167</v>
-      </c>
-      <c r="N13" t="s" s="2">
-        <v>168</v>
       </c>
       <c r="O13" s="2"/>
       <c r="P13" t="s" s="2">
@@ -2989,7 +2981,7 @@
       </c>
       <c r="Q13" s="2"/>
       <c r="R13" t="s" s="2">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="S13" t="s" s="2">
         <v>81</v>
@@ -3031,7 +3023,7 @@
         <v>81</v>
       </c>
       <c r="AF13" t="s" s="2">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="AG13" t="s" s="2">
         <v>89</v>
@@ -3066,13 +3058,13 @@
     </row>
     <row r="14" hidden="true">
       <c r="A14" t="s" s="2">
+        <v>169</v>
+      </c>
+      <c r="B14" t="s" s="2">
+        <v>170</v>
+      </c>
+      <c r="C14" t="s" s="2">
         <v>171</v>
-      </c>
-      <c r="B14" t="s" s="2">
-        <v>172</v>
-      </c>
-      <c r="C14" t="s" s="2">
-        <v>173</v>
       </c>
       <c r="D14" t="s" s="2">
         <v>81</v>
@@ -3094,16 +3086,16 @@
         <v>81</v>
       </c>
       <c r="K14" t="s" s="2">
+        <v>172</v>
+      </c>
+      <c r="L14" t="s" s="2">
+        <v>173</v>
+      </c>
+      <c r="M14" t="s" s="2">
         <v>174</v>
       </c>
-      <c r="L14" t="s" s="2">
+      <c r="N14" t="s" s="2">
         <v>175</v>
-      </c>
-      <c r="M14" t="s" s="2">
-        <v>176</v>
-      </c>
-      <c r="N14" t="s" s="2">
-        <v>177</v>
       </c>
       <c r="O14" s="2"/>
       <c r="P14" t="s" s="2">
@@ -3153,7 +3145,7 @@
         <v>81</v>
       </c>
       <c r="AF14" t="s" s="2">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="AG14" t="s" s="2">
         <v>79</v>
@@ -3188,14 +3180,14 @@
     </row>
     <row r="15" hidden="true">
       <c r="A15" t="s" s="2">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B15" t="s" s="2">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" t="s" s="2">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="E15" s="2"/>
       <c r="F15" t="s" s="2">
@@ -3217,13 +3209,13 @@
         <v>134</v>
       </c>
       <c r="L15" t="s" s="2">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="M15" t="s" s="2">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="N15" t="s" s="2">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="O15" s="2"/>
       <c r="P15" t="s" s="2">
@@ -3273,7 +3265,7 @@
         <v>81</v>
       </c>
       <c r="AF15" t="s" s="2">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="AG15" t="s" s="2">
         <v>79</v>
@@ -3308,10 +3300,10 @@
     </row>
     <row r="16" hidden="true">
       <c r="A16" t="s" s="2">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" t="s" s="2">
@@ -3334,13 +3326,13 @@
         <v>90</v>
       </c>
       <c r="K16" t="s" s="2">
+        <v>182</v>
+      </c>
+      <c r="L16" t="s" s="2">
+        <v>183</v>
+      </c>
+      <c r="M16" t="s" s="2">
         <v>184</v>
-      </c>
-      <c r="L16" t="s" s="2">
-        <v>185</v>
-      </c>
-      <c r="M16" t="s" s="2">
-        <v>186</v>
       </c>
       <c r="N16" s="2"/>
       <c r="O16" s="2"/>
@@ -3391,7 +3383,7 @@
         <v>81</v>
       </c>
       <c r="AF16" t="s" s="2">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="AG16" t="s" s="2">
         <v>79</v>
@@ -3409,27 +3401,27 @@
         <v>81</v>
       </c>
       <c r="AL16" t="s" s="2">
+        <v>185</v>
+      </c>
+      <c r="AM16" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AN16" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AO16" t="s" s="2">
+        <v>186</v>
+      </c>
+      <c r="AP16" t="s" s="2">
         <v>187</v>
-      </c>
-      <c r="AM16" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AN16" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AO16" t="s" s="2">
-        <v>188</v>
-      </c>
-      <c r="AP16" t="s" s="2">
-        <v>189</v>
       </c>
     </row>
     <row r="17" hidden="true">
       <c r="A17" t="s" s="2">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" t="s" s="2">
@@ -3455,13 +3447,13 @@
         <v>108</v>
       </c>
       <c r="L17" t="s" s="2">
+        <v>189</v>
+      </c>
+      <c r="M17" t="s" s="2">
+        <v>190</v>
+      </c>
+      <c r="N17" t="s" s="2">
         <v>191</v>
-      </c>
-      <c r="M17" t="s" s="2">
-        <v>192</v>
-      </c>
-      <c r="N17" t="s" s="2">
-        <v>193</v>
       </c>
       <c r="O17" s="2"/>
       <c r="P17" t="s" s="2">
@@ -3487,73 +3479,73 @@
         <v>81</v>
       </c>
       <c r="X17" t="s" s="2">
+        <v>192</v>
+      </c>
+      <c r="Y17" t="s" s="2">
+        <v>193</v>
+      </c>
+      <c r="Z17" t="s" s="2">
         <v>194</v>
       </c>
-      <c r="Y17" t="s" s="2">
+      <c r="AA17" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AB17" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AC17" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AD17" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AE17" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AF17" t="s" s="2">
+        <v>188</v>
+      </c>
+      <c r="AG17" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="AH17" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="AI17" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AJ17" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK17" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL17" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM17" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AN17" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AO17" t="s" s="2">
         <v>195</v>
       </c>
-      <c r="Z17" t="s" s="2">
+      <c r="AP17" t="s" s="2">
         <v>196</v>
-      </c>
-      <c r="AA17" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AB17" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AC17" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AD17" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AE17" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AF17" t="s" s="2">
-        <v>190</v>
-      </c>
-      <c r="AG17" t="s" s="2">
-        <v>89</v>
-      </c>
-      <c r="AH17" t="s" s="2">
-        <v>89</v>
-      </c>
-      <c r="AI17" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AJ17" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AK17" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AL17" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AM17" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AN17" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AO17" t="s" s="2">
-        <v>197</v>
-      </c>
-      <c r="AP17" t="s" s="2">
-        <v>198</v>
       </c>
     </row>
     <row r="18" hidden="true">
       <c r="A18" t="s" s="2">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" t="s" s="2">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="E18" s="2"/>
       <c r="F18" t="s" s="2">
@@ -3572,13 +3564,13 @@
         <v>90</v>
       </c>
       <c r="K18" t="s" s="2">
+        <v>199</v>
+      </c>
+      <c r="L18" t="s" s="2">
+        <v>200</v>
+      </c>
+      <c r="M18" t="s" s="2">
         <v>201</v>
-      </c>
-      <c r="L18" t="s" s="2">
-        <v>202</v>
-      </c>
-      <c r="M18" t="s" s="2">
-        <v>203</v>
       </c>
       <c r="N18" s="2"/>
       <c r="O18" s="2"/>
@@ -3593,7 +3585,7 @@
         <v>81</v>
       </c>
       <c r="T18" t="s" s="2">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="U18" t="s" s="2">
         <v>81</v>
@@ -3608,66 +3600,66 @@
         <v>112</v>
       </c>
       <c r="Y18" t="s" s="2">
+        <v>201</v>
+      </c>
+      <c r="Z18" t="s" s="2">
         <v>203</v>
       </c>
-      <c r="Z18" t="s" s="2">
+      <c r="AA18" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AB18" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AC18" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AD18" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AE18" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AF18" t="s" s="2">
+        <v>197</v>
+      </c>
+      <c r="AG18" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH18" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="AI18" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AJ18" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK18" t="s" s="2">
+        <v>204</v>
+      </c>
+      <c r="AL18" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM18" t="s" s="2">
+        <v>204</v>
+      </c>
+      <c r="AN18" t="s" s="2">
+        <v>204</v>
+      </c>
+      <c r="AO18" t="s" s="2">
         <v>205</v>
       </c>
-      <c r="AA18" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AB18" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AC18" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AD18" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AE18" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AF18" t="s" s="2">
-        <v>199</v>
-      </c>
-      <c r="AG18" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH18" t="s" s="2">
-        <v>89</v>
-      </c>
-      <c r="AI18" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AJ18" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AK18" t="s" s="2">
+      <c r="AP18" t="s" s="2">
         <v>206</v>
-      </c>
-      <c r="AL18" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AM18" t="s" s="2">
-        <v>206</v>
-      </c>
-      <c r="AN18" t="s" s="2">
-        <v>206</v>
-      </c>
-      <c r="AO18" t="s" s="2">
-        <v>207</v>
-      </c>
-      <c r="AP18" t="s" s="2">
-        <v>208</v>
       </c>
     </row>
     <row r="19" hidden="true">
       <c r="A19" t="s" s="2">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
@@ -3690,13 +3682,13 @@
         <v>81</v>
       </c>
       <c r="K19" t="s" s="2">
+        <v>149</v>
+      </c>
+      <c r="L19" t="s" s="2">
+        <v>150</v>
+      </c>
+      <c r="M19" t="s" s="2">
         <v>151</v>
-      </c>
-      <c r="L19" t="s" s="2">
-        <v>152</v>
-      </c>
-      <c r="M19" t="s" s="2">
-        <v>153</v>
       </c>
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
@@ -3747,7 +3739,7 @@
         <v>81</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="AG19" t="s" s="2">
         <v>79</v>
@@ -3774,7 +3766,7 @@
         <v>81</v>
       </c>
       <c r="AO19" t="s" s="2">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="AP19" t="s" s="2">
         <v>81</v>
@@ -3782,14 +3774,14 @@
     </row>
     <row r="20" hidden="true">
       <c r="A20" t="s" s="2">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" t="s" s="2">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="E20" s="2"/>
       <c r="F20" t="s" s="2">
@@ -3811,13 +3803,13 @@
         <v>134</v>
       </c>
       <c r="L20" t="s" s="2">
+        <v>157</v>
+      </c>
+      <c r="M20" t="s" s="2">
+        <v>158</v>
+      </c>
+      <c r="N20" t="s" s="2">
         <v>159</v>
-      </c>
-      <c r="M20" t="s" s="2">
-        <v>160</v>
-      </c>
-      <c r="N20" t="s" s="2">
-        <v>161</v>
       </c>
       <c r="O20" s="2"/>
       <c r="P20" t="s" s="2">
@@ -3858,7 +3850,7 @@
         <v>137</v>
       </c>
       <c r="AC20" t="s" s="2">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="AD20" t="s" s="2">
         <v>81</v>
@@ -3867,7 +3859,7 @@
         <v>138</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="AG20" t="s" s="2">
         <v>79</v>
@@ -3894,7 +3886,7 @@
         <v>81</v>
       </c>
       <c r="AO20" t="s" s="2">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="AP20" t="s" s="2">
         <v>81</v>
@@ -3902,10 +3894,10 @@
     </row>
     <row r="21" hidden="true">
       <c r="A21" t="s" s="2">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
@@ -3928,19 +3920,19 @@
         <v>90</v>
       </c>
       <c r="K21" t="s" s="2">
+        <v>210</v>
+      </c>
+      <c r="L21" t="s" s="2">
+        <v>211</v>
+      </c>
+      <c r="M21" t="s" s="2">
         <v>212</v>
       </c>
-      <c r="L21" t="s" s="2">
+      <c r="N21" t="s" s="2">
         <v>213</v>
       </c>
-      <c r="M21" t="s" s="2">
+      <c r="O21" t="s" s="2">
         <v>214</v>
-      </c>
-      <c r="N21" t="s" s="2">
-        <v>215</v>
-      </c>
-      <c r="O21" t="s" s="2">
-        <v>216</v>
       </c>
       <c r="P21" t="s" s="2">
         <v>81</v>
@@ -3989,7 +3981,7 @@
         <v>81</v>
       </c>
       <c r="AF21" t="s" s="2">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="AG21" t="s" s="2">
         <v>79</v>
@@ -4016,7 +4008,7 @@
         <v>81</v>
       </c>
       <c r="AO21" t="s" s="2">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="AP21" t="s" s="2">
         <v>81</v>
@@ -4024,10 +4016,10 @@
     </row>
     <row r="22" hidden="true">
       <c r="A22" t="s" s="2">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
@@ -4050,13 +4042,13 @@
         <v>81</v>
       </c>
       <c r="K22" t="s" s="2">
+        <v>149</v>
+      </c>
+      <c r="L22" t="s" s="2">
+        <v>150</v>
+      </c>
+      <c r="M22" t="s" s="2">
         <v>151</v>
-      </c>
-      <c r="L22" t="s" s="2">
-        <v>152</v>
-      </c>
-      <c r="M22" t="s" s="2">
-        <v>153</v>
       </c>
       <c r="N22" s="2"/>
       <c r="O22" s="2"/>
@@ -4107,7 +4099,7 @@
         <v>81</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>79</v>
@@ -4134,7 +4126,7 @@
         <v>81</v>
       </c>
       <c r="AO22" t="s" s="2">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="AP22" t="s" s="2">
         <v>81</v>
@@ -4142,14 +4134,14 @@
     </row>
     <row r="23" hidden="true">
       <c r="A23" t="s" s="2">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="E23" s="2"/>
       <c r="F23" t="s" s="2">
@@ -4171,13 +4163,13 @@
         <v>134</v>
       </c>
       <c r="L23" t="s" s="2">
+        <v>157</v>
+      </c>
+      <c r="M23" t="s" s="2">
+        <v>158</v>
+      </c>
+      <c r="N23" t="s" s="2">
         <v>159</v>
-      </c>
-      <c r="M23" t="s" s="2">
-        <v>160</v>
-      </c>
-      <c r="N23" t="s" s="2">
-        <v>161</v>
       </c>
       <c r="O23" s="2"/>
       <c r="P23" t="s" s="2">
@@ -4218,7 +4210,7 @@
         <v>137</v>
       </c>
       <c r="AC23" t="s" s="2">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="AD23" t="s" s="2">
         <v>81</v>
@@ -4227,7 +4219,7 @@
         <v>138</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="AG23" t="s" s="2">
         <v>79</v>
@@ -4254,7 +4246,7 @@
         <v>81</v>
       </c>
       <c r="AO23" t="s" s="2">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="AP23" t="s" s="2">
         <v>81</v>
@@ -4262,10 +4254,10 @@
     </row>
     <row r="24" hidden="true">
       <c r="A24" t="s" s="2">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -4291,16 +4283,16 @@
         <v>102</v>
       </c>
       <c r="L24" t="s" s="2">
+        <v>220</v>
+      </c>
+      <c r="M24" t="s" s="2">
+        <v>221</v>
+      </c>
+      <c r="N24" t="s" s="2">
         <v>222</v>
       </c>
-      <c r="M24" t="s" s="2">
+      <c r="O24" t="s" s="2">
         <v>223</v>
-      </c>
-      <c r="N24" t="s" s="2">
-        <v>224</v>
-      </c>
-      <c r="O24" t="s" s="2">
-        <v>225</v>
       </c>
       <c r="P24" t="s" s="2">
         <v>81</v>
@@ -4349,7 +4341,7 @@
         <v>81</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="AG24" t="s" s="2">
         <v>79</v>
@@ -4376,7 +4368,7 @@
         <v>81</v>
       </c>
       <c r="AO24" t="s" s="2">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="AP24" t="s" s="2">
         <v>81</v>
@@ -4384,10 +4376,10 @@
     </row>
     <row r="25" hidden="true">
       <c r="A25" t="s" s="2">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
@@ -4410,16 +4402,16 @@
         <v>90</v>
       </c>
       <c r="K25" t="s" s="2">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="L25" t="s" s="2">
+        <v>227</v>
+      </c>
+      <c r="M25" t="s" s="2">
+        <v>228</v>
+      </c>
+      <c r="N25" t="s" s="2">
         <v>229</v>
-      </c>
-      <c r="M25" t="s" s="2">
-        <v>230</v>
-      </c>
-      <c r="N25" t="s" s="2">
-        <v>231</v>
       </c>
       <c r="O25" s="2"/>
       <c r="P25" t="s" s="2">
@@ -4469,7 +4461,7 @@
         <v>81</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>79</v>
@@ -4496,7 +4488,7 @@
         <v>81</v>
       </c>
       <c r="AO25" t="s" s="2">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="AP25" t="s" s="2">
         <v>81</v>
@@ -4504,10 +4496,10 @@
     </row>
     <row r="26" hidden="true">
       <c r="A26" t="s" s="2">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
@@ -4533,14 +4525,14 @@
         <v>108</v>
       </c>
       <c r="L26" t="s" s="2">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="M26" t="s" s="2">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="N26" s="2"/>
       <c r="O26" t="s" s="2">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="P26" t="s" s="2">
         <v>81</v>
@@ -4589,7 +4581,7 @@
         <v>81</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="AG26" t="s" s="2">
         <v>79</v>
@@ -4616,7 +4608,7 @@
         <v>81</v>
       </c>
       <c r="AO26" t="s" s="2">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="AP26" t="s" s="2">
         <v>81</v>
@@ -4624,10 +4616,10 @@
     </row>
     <row r="27" hidden="true">
       <c r="A27" t="s" s="2">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
@@ -4650,17 +4642,17 @@
         <v>90</v>
       </c>
       <c r="K27" t="s" s="2">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="L27" t="s" s="2">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="M27" t="s" s="2">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="N27" s="2"/>
       <c r="O27" t="s" s="2">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="P27" t="s" s="2">
         <v>81</v>
@@ -4709,7 +4701,7 @@
         <v>81</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>79</v>
@@ -4736,7 +4728,7 @@
         <v>81</v>
       </c>
       <c r="AO27" t="s" s="2">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="AP27" t="s" s="2">
         <v>81</v>
@@ -4744,10 +4736,10 @@
     </row>
     <row r="28" hidden="true">
       <c r="A28" t="s" s="2">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -4770,19 +4762,19 @@
         <v>90</v>
       </c>
       <c r="K28" t="s" s="2">
+        <v>245</v>
+      </c>
+      <c r="L28" t="s" s="2">
+        <v>246</v>
+      </c>
+      <c r="M28" t="s" s="2">
         <v>247</v>
       </c>
-      <c r="L28" t="s" s="2">
+      <c r="N28" t="s" s="2">
         <v>248</v>
       </c>
-      <c r="M28" t="s" s="2">
+      <c r="O28" t="s" s="2">
         <v>249</v>
-      </c>
-      <c r="N28" t="s" s="2">
-        <v>250</v>
-      </c>
-      <c r="O28" t="s" s="2">
-        <v>251</v>
       </c>
       <c r="P28" t="s" s="2">
         <v>81</v>
@@ -4831,7 +4823,7 @@
         <v>81</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>79</v>
@@ -4858,7 +4850,7 @@
         <v>81</v>
       </c>
       <c r="AO28" t="s" s="2">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="AP28" t="s" s="2">
         <v>81</v>
@@ -4866,10 +4858,10 @@
     </row>
     <row r="29" hidden="true">
       <c r="A29" t="s" s="2">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -4892,19 +4884,19 @@
         <v>90</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="L29" t="s" s="2">
+        <v>253</v>
+      </c>
+      <c r="M29" t="s" s="2">
+        <v>254</v>
+      </c>
+      <c r="N29" t="s" s="2">
         <v>255</v>
       </c>
-      <c r="M29" t="s" s="2">
+      <c r="O29" t="s" s="2">
         <v>256</v>
-      </c>
-      <c r="N29" t="s" s="2">
-        <v>257</v>
-      </c>
-      <c r="O29" t="s" s="2">
-        <v>258</v>
       </c>
       <c r="P29" t="s" s="2">
         <v>81</v>
@@ -4953,7 +4945,7 @@
         <v>81</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>79</v>
@@ -4980,7 +4972,7 @@
         <v>81</v>
       </c>
       <c r="AO29" t="s" s="2">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="AP29" t="s" s="2">
         <v>81</v>
@@ -4988,14 +4980,14 @@
     </row>
     <row r="30" hidden="true">
       <c r="A30" t="s" s="2">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="E30" s="2"/>
       <c r="F30" t="s" s="2">
@@ -5014,16 +5006,16 @@
         <v>90</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="L30" t="s" s="2">
+        <v>261</v>
+      </c>
+      <c r="M30" t="s" s="2">
+        <v>262</v>
+      </c>
+      <c r="N30" t="s" s="2">
         <v>263</v>
-      </c>
-      <c r="M30" t="s" s="2">
-        <v>264</v>
-      </c>
-      <c r="N30" t="s" s="2">
-        <v>265</v>
       </c>
       <c r="O30" s="2"/>
       <c r="P30" t="s" s="2">
@@ -5037,7 +5029,7 @@
         <v>81</v>
       </c>
       <c r="T30" t="s" s="2">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="U30" t="s" s="2">
         <v>81</v>
@@ -5053,63 +5045,63 @@
       </c>
       <c r="Y30" s="2"/>
       <c r="Z30" t="s" s="2">
+        <v>265</v>
+      </c>
+      <c r="AA30" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AB30" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AC30" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AD30" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AE30" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AF30" t="s" s="2">
+        <v>259</v>
+      </c>
+      <c r="AG30" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="AH30" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="AI30" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AJ30" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK30" t="s" s="2">
+        <v>266</v>
+      </c>
+      <c r="AL30" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM30" t="s" s="2">
+        <v>266</v>
+      </c>
+      <c r="AN30" t="s" s="2">
+        <v>266</v>
+      </c>
+      <c r="AO30" t="s" s="2">
         <v>267</v>
       </c>
-      <c r="AA30" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AB30" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AC30" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AD30" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AE30" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AF30" t="s" s="2">
-        <v>261</v>
-      </c>
-      <c r="AG30" t="s" s="2">
-        <v>89</v>
-      </c>
-      <c r="AH30" t="s" s="2">
-        <v>89</v>
-      </c>
-      <c r="AI30" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AJ30" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AK30" t="s" s="2">
+      <c r="AP30" t="s" s="2">
         <v>268</v>
-      </c>
-      <c r="AL30" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AM30" t="s" s="2">
-        <v>268</v>
-      </c>
-      <c r="AN30" t="s" s="2">
-        <v>268</v>
-      </c>
-      <c r="AO30" t="s" s="2">
-        <v>269</v>
-      </c>
-      <c r="AP30" t="s" s="2">
-        <v>270</v>
       </c>
     </row>
     <row r="31" hidden="true">
       <c r="A31" t="s" s="2">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
@@ -5132,13 +5124,13 @@
         <v>81</v>
       </c>
       <c r="K31" t="s" s="2">
+        <v>149</v>
+      </c>
+      <c r="L31" t="s" s="2">
+        <v>150</v>
+      </c>
+      <c r="M31" t="s" s="2">
         <v>151</v>
-      </c>
-      <c r="L31" t="s" s="2">
-        <v>152</v>
-      </c>
-      <c r="M31" t="s" s="2">
-        <v>153</v>
       </c>
       <c r="N31" s="2"/>
       <c r="O31" s="2"/>
@@ -5189,7 +5181,7 @@
         <v>81</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>79</v>
@@ -5216,7 +5208,7 @@
         <v>81</v>
       </c>
       <c r="AO31" t="s" s="2">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="AP31" t="s" s="2">
         <v>81</v>
@@ -5224,14 +5216,14 @@
     </row>
     <row r="32" hidden="true">
       <c r="A32" t="s" s="2">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="E32" s="2"/>
       <c r="F32" t="s" s="2">
@@ -5253,13 +5245,13 @@
         <v>134</v>
       </c>
       <c r="L32" t="s" s="2">
+        <v>157</v>
+      </c>
+      <c r="M32" t="s" s="2">
+        <v>158</v>
+      </c>
+      <c r="N32" t="s" s="2">
         <v>159</v>
-      </c>
-      <c r="M32" t="s" s="2">
-        <v>160</v>
-      </c>
-      <c r="N32" t="s" s="2">
-        <v>161</v>
       </c>
       <c r="O32" s="2"/>
       <c r="P32" t="s" s="2">
@@ -5300,7 +5292,7 @@
         <v>137</v>
       </c>
       <c r="AC32" t="s" s="2">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="AD32" t="s" s="2">
         <v>81</v>
@@ -5309,7 +5301,7 @@
         <v>138</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>79</v>
@@ -5336,7 +5328,7 @@
         <v>81</v>
       </c>
       <c r="AO32" t="s" s="2">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="AP32" t="s" s="2">
         <v>81</v>
@@ -5344,10 +5336,10 @@
     </row>
     <row r="33" hidden="true">
       <c r="A33" t="s" s="2">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
@@ -5370,19 +5362,19 @@
         <v>90</v>
       </c>
       <c r="K33" t="s" s="2">
+        <v>210</v>
+      </c>
+      <c r="L33" t="s" s="2">
+        <v>211</v>
+      </c>
+      <c r="M33" t="s" s="2">
         <v>212</v>
       </c>
-      <c r="L33" t="s" s="2">
+      <c r="N33" t="s" s="2">
         <v>213</v>
       </c>
-      <c r="M33" t="s" s="2">
+      <c r="O33" t="s" s="2">
         <v>214</v>
-      </c>
-      <c r="N33" t="s" s="2">
-        <v>215</v>
-      </c>
-      <c r="O33" t="s" s="2">
-        <v>216</v>
       </c>
       <c r="P33" t="s" s="2">
         <v>81</v>
@@ -5431,7 +5423,7 @@
         <v>81</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>79</v>
@@ -5458,7 +5450,7 @@
         <v>81</v>
       </c>
       <c r="AO33" t="s" s="2">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="AP33" t="s" s="2">
         <v>81</v>
@@ -5466,10 +5458,10 @@
     </row>
     <row r="34" hidden="true">
       <c r="A34" t="s" s="2">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
@@ -5492,13 +5484,13 @@
         <v>81</v>
       </c>
       <c r="K34" t="s" s="2">
+        <v>149</v>
+      </c>
+      <c r="L34" t="s" s="2">
+        <v>150</v>
+      </c>
+      <c r="M34" t="s" s="2">
         <v>151</v>
-      </c>
-      <c r="L34" t="s" s="2">
-        <v>152</v>
-      </c>
-      <c r="M34" t="s" s="2">
-        <v>153</v>
       </c>
       <c r="N34" s="2"/>
       <c r="O34" s="2"/>
@@ -5549,7 +5541,7 @@
         <v>81</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>79</v>
@@ -5576,7 +5568,7 @@
         <v>81</v>
       </c>
       <c r="AO34" t="s" s="2">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="AP34" t="s" s="2">
         <v>81</v>
@@ -5584,14 +5576,14 @@
     </row>
     <row r="35" hidden="true">
       <c r="A35" t="s" s="2">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="E35" s="2"/>
       <c r="F35" t="s" s="2">
@@ -5613,13 +5605,13 @@
         <v>134</v>
       </c>
       <c r="L35" t="s" s="2">
+        <v>157</v>
+      </c>
+      <c r="M35" t="s" s="2">
+        <v>158</v>
+      </c>
+      <c r="N35" t="s" s="2">
         <v>159</v>
-      </c>
-      <c r="M35" t="s" s="2">
-        <v>160</v>
-      </c>
-      <c r="N35" t="s" s="2">
-        <v>161</v>
       </c>
       <c r="O35" s="2"/>
       <c r="P35" t="s" s="2">
@@ -5660,7 +5652,7 @@
         <v>137</v>
       </c>
       <c r="AC35" t="s" s="2">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="AD35" t="s" s="2">
         <v>81</v>
@@ -5669,7 +5661,7 @@
         <v>138</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>79</v>
@@ -5696,7 +5688,7 @@
         <v>81</v>
       </c>
       <c r="AO35" t="s" s="2">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="AP35" t="s" s="2">
         <v>81</v>
@@ -5704,10 +5696,10 @@
     </row>
     <row r="36" hidden="true">
       <c r="A36" t="s" s="2">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
@@ -5733,16 +5725,16 @@
         <v>102</v>
       </c>
       <c r="L36" t="s" s="2">
+        <v>220</v>
+      </c>
+      <c r="M36" t="s" s="2">
+        <v>221</v>
+      </c>
+      <c r="N36" t="s" s="2">
         <v>222</v>
       </c>
-      <c r="M36" t="s" s="2">
+      <c r="O36" t="s" s="2">
         <v>223</v>
-      </c>
-      <c r="N36" t="s" s="2">
-        <v>224</v>
-      </c>
-      <c r="O36" t="s" s="2">
-        <v>225</v>
       </c>
       <c r="P36" t="s" s="2">
         <v>81</v>
@@ -5791,7 +5783,7 @@
         <v>81</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>79</v>
@@ -5818,7 +5810,7 @@
         <v>81</v>
       </c>
       <c r="AO36" t="s" s="2">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="AP36" t="s" s="2">
         <v>81</v>
@@ -5826,10 +5818,10 @@
     </row>
     <row r="37" hidden="true">
       <c r="A37" t="s" s="2">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
@@ -5852,16 +5844,16 @@
         <v>90</v>
       </c>
       <c r="K37" t="s" s="2">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="L37" t="s" s="2">
+        <v>227</v>
+      </c>
+      <c r="M37" t="s" s="2">
+        <v>228</v>
+      </c>
+      <c r="N37" t="s" s="2">
         <v>229</v>
-      </c>
-      <c r="M37" t="s" s="2">
-        <v>230</v>
-      </c>
-      <c r="N37" t="s" s="2">
-        <v>231</v>
       </c>
       <c r="O37" s="2"/>
       <c r="P37" t="s" s="2">
@@ -5911,7 +5903,7 @@
         <v>81</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>79</v>
@@ -5938,7 +5930,7 @@
         <v>81</v>
       </c>
       <c r="AO37" t="s" s="2">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="AP37" t="s" s="2">
         <v>81</v>
@@ -5946,10 +5938,10 @@
     </row>
     <row r="38" hidden="true">
       <c r="A38" t="s" s="2">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
@@ -5975,14 +5967,14 @@
         <v>108</v>
       </c>
       <c r="L38" t="s" s="2">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="M38" t="s" s="2">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="N38" s="2"/>
       <c r="O38" t="s" s="2">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="P38" t="s" s="2">
         <v>81</v>
@@ -6031,7 +6023,7 @@
         <v>81</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>79</v>
@@ -6058,7 +6050,7 @@
         <v>81</v>
       </c>
       <c r="AO38" t="s" s="2">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="AP38" t="s" s="2">
         <v>81</v>
@@ -6066,10 +6058,10 @@
     </row>
     <row r="39" hidden="true">
       <c r="A39" t="s" s="2">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
@@ -6092,17 +6084,17 @@
         <v>90</v>
       </c>
       <c r="K39" t="s" s="2">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="M39" t="s" s="2">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="N39" s="2"/>
       <c r="O39" t="s" s="2">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="P39" t="s" s="2">
         <v>81</v>
@@ -6151,7 +6143,7 @@
         <v>81</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>79</v>
@@ -6178,7 +6170,7 @@
         <v>81</v>
       </c>
       <c r="AO39" t="s" s="2">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="AP39" t="s" s="2">
         <v>81</v>
@@ -6186,10 +6178,10 @@
     </row>
     <row r="40" hidden="true">
       <c r="A40" t="s" s="2">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -6212,19 +6204,19 @@
         <v>90</v>
       </c>
       <c r="K40" t="s" s="2">
+        <v>245</v>
+      </c>
+      <c r="L40" t="s" s="2">
+        <v>246</v>
+      </c>
+      <c r="M40" t="s" s="2">
         <v>247</v>
       </c>
-      <c r="L40" t="s" s="2">
+      <c r="N40" t="s" s="2">
         <v>248</v>
       </c>
-      <c r="M40" t="s" s="2">
+      <c r="O40" t="s" s="2">
         <v>249</v>
-      </c>
-      <c r="N40" t="s" s="2">
-        <v>250</v>
-      </c>
-      <c r="O40" t="s" s="2">
-        <v>251</v>
       </c>
       <c r="P40" t="s" s="2">
         <v>81</v>
@@ -6273,7 +6265,7 @@
         <v>81</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>79</v>
@@ -6300,7 +6292,7 @@
         <v>81</v>
       </c>
       <c r="AO40" t="s" s="2">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="AP40" t="s" s="2">
         <v>81</v>
@@ -6308,10 +6300,10 @@
     </row>
     <row r="41" hidden="true">
       <c r="A41" t="s" s="2">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
@@ -6334,19 +6326,19 @@
         <v>90</v>
       </c>
       <c r="K41" t="s" s="2">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="L41" t="s" s="2">
+        <v>253</v>
+      </c>
+      <c r="M41" t="s" s="2">
+        <v>254</v>
+      </c>
+      <c r="N41" t="s" s="2">
         <v>255</v>
       </c>
-      <c r="M41" t="s" s="2">
+      <c r="O41" t="s" s="2">
         <v>256</v>
-      </c>
-      <c r="N41" t="s" s="2">
-        <v>257</v>
-      </c>
-      <c r="O41" t="s" s="2">
-        <v>258</v>
       </c>
       <c r="P41" t="s" s="2">
         <v>81</v>
@@ -6395,7 +6387,7 @@
         <v>81</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>79</v>
@@ -6422,7 +6414,7 @@
         <v>81</v>
       </c>
       <c r="AO41" t="s" s="2">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="AP41" t="s" s="2">
         <v>81</v>
@@ -6430,10 +6422,10 @@
     </row>
     <row r="42" hidden="true">
       <c r="A42" t="s" s="2">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
@@ -6456,13 +6448,13 @@
         <v>90</v>
       </c>
       <c r="K42" t="s" s="2">
+        <v>281</v>
+      </c>
+      <c r="L42" t="s" s="2">
+        <v>282</v>
+      </c>
+      <c r="M42" t="s" s="2">
         <v>283</v>
-      </c>
-      <c r="L42" t="s" s="2">
-        <v>284</v>
-      </c>
-      <c r="M42" t="s" s="2">
-        <v>285</v>
       </c>
       <c r="N42" s="2"/>
       <c r="O42" s="2"/>
@@ -6513,7 +6505,7 @@
         <v>81</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>89</v>
@@ -6540,18 +6532,18 @@
         <v>81</v>
       </c>
       <c r="AO42" t="s" s="2">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="AP42" t="s" s="2">
-        <v>287</v>
+        <v>285</v>
       </c>
     </row>
     <row r="43" hidden="true">
       <c r="A43" t="s" s="2">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
@@ -6574,13 +6566,13 @@
         <v>81</v>
       </c>
       <c r="K43" t="s" s="2">
+        <v>149</v>
+      </c>
+      <c r="L43" t="s" s="2">
+        <v>150</v>
+      </c>
+      <c r="M43" t="s" s="2">
         <v>151</v>
-      </c>
-      <c r="L43" t="s" s="2">
-        <v>152</v>
-      </c>
-      <c r="M43" t="s" s="2">
-        <v>153</v>
       </c>
       <c r="N43" s="2"/>
       <c r="O43" s="2"/>
@@ -6631,7 +6623,7 @@
         <v>81</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="AG43" t="s" s="2">
         <v>79</v>
@@ -6658,7 +6650,7 @@
         <v>81</v>
       </c>
       <c r="AO43" t="s" s="2">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="AP43" t="s" s="2">
         <v>81</v>
@@ -6666,10 +6658,10 @@
     </row>
     <row r="44" hidden="true">
       <c r="A44" t="s" s="2">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
@@ -6740,7 +6732,7 @@
         <v>137</v>
       </c>
       <c r="AC44" t="s" s="2">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="AD44" t="s" s="2">
         <v>81</v>
@@ -6749,7 +6741,7 @@
         <v>138</v>
       </c>
       <c r="AF44" t="s" s="2">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="AG44" t="s" s="2">
         <v>79</v>
@@ -6784,13 +6776,13 @@
     </row>
     <row r="45" hidden="true">
       <c r="A45" t="s" s="2">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="B45" t="s" s="2">
+        <v>287</v>
+      </c>
+      <c r="C45" t="s" s="2">
         <v>289</v>
-      </c>
-      <c r="C45" t="s" s="2">
-        <v>291</v>
       </c>
       <c r="D45" t="s" s="2">
         <v>81</v>
@@ -6812,13 +6804,13 @@
         <v>81</v>
       </c>
       <c r="K45" t="s" s="2">
+        <v>290</v>
+      </c>
+      <c r="L45" t="s" s="2">
+        <v>291</v>
+      </c>
+      <c r="M45" t="s" s="2">
         <v>292</v>
-      </c>
-      <c r="L45" t="s" s="2">
-        <v>293</v>
-      </c>
-      <c r="M45" t="s" s="2">
-        <v>294</v>
       </c>
       <c r="N45" s="2"/>
       <c r="O45" s="2"/>
@@ -6869,7 +6861,7 @@
         <v>81</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>79</v>
@@ -6904,10 +6896,10 @@
     </row>
     <row r="46" hidden="true">
       <c r="A46" t="s" s="2">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
@@ -6930,16 +6922,16 @@
         <v>90</v>
       </c>
       <c r="K46" t="s" s="2">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="L46" t="s" s="2">
+        <v>294</v>
+      </c>
+      <c r="M46" t="s" s="2">
+        <v>295</v>
+      </c>
+      <c r="N46" t="s" s="2">
         <v>296</v>
-      </c>
-      <c r="M46" t="s" s="2">
-        <v>297</v>
-      </c>
-      <c r="N46" t="s" s="2">
-        <v>298</v>
       </c>
       <c r="O46" s="2"/>
       <c r="P46" t="s" s="2">
@@ -6989,7 +6981,7 @@
         <v>81</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>79</v>
@@ -6998,7 +6990,7 @@
         <v>89</v>
       </c>
       <c r="AI46" t="s" s="2">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="AJ46" t="s" s="2">
         <v>81</v>
@@ -7024,10 +7016,10 @@
     </row>
     <row r="47" hidden="true">
       <c r="A47" t="s" s="2">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
@@ -7050,16 +7042,16 @@
         <v>90</v>
       </c>
       <c r="K47" t="s" s="2">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="L47" t="s" s="2">
+        <v>300</v>
+      </c>
+      <c r="M47" t="s" s="2">
+        <v>301</v>
+      </c>
+      <c r="N47" t="s" s="2">
         <v>302</v>
-      </c>
-      <c r="M47" t="s" s="2">
-        <v>303</v>
-      </c>
-      <c r="N47" t="s" s="2">
-        <v>304</v>
       </c>
       <c r="O47" s="2"/>
       <c r="P47" t="s" s="2">
@@ -7109,7 +7101,7 @@
         <v>81</v>
       </c>
       <c r="AF47" t="s" s="2">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="AG47" t="s" s="2">
         <v>79</v>
@@ -7136,7 +7128,7 @@
         <v>81</v>
       </c>
       <c r="AO47" t="s" s="2">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="AP47" t="s" s="2">
         <v>81</v>
@@ -7144,10 +7136,10 @@
     </row>
     <row r="48" hidden="true">
       <c r="A48" t="s" s="2">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
@@ -7170,16 +7162,16 @@
         <v>90</v>
       </c>
       <c r="K48" t="s" s="2">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="L48" t="s" s="2">
+        <v>306</v>
+      </c>
+      <c r="M48" t="s" s="2">
+        <v>307</v>
+      </c>
+      <c r="N48" t="s" s="2">
         <v>308</v>
-      </c>
-      <c r="M48" t="s" s="2">
-        <v>309</v>
-      </c>
-      <c r="N48" t="s" s="2">
-        <v>310</v>
       </c>
       <c r="O48" s="2"/>
       <c r="P48" t="s" s="2">
@@ -7229,7 +7221,7 @@
         <v>81</v>
       </c>
       <c r="AF48" t="s" s="2">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="AG48" t="s" s="2">
         <v>79</v>
@@ -7264,10 +7256,10 @@
     </row>
     <row r="49" hidden="true">
       <c r="A49" t="s" s="2">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" t="s" s="2">
@@ -7290,13 +7282,13 @@
         <v>90</v>
       </c>
       <c r="K49" t="s" s="2">
+        <v>311</v>
+      </c>
+      <c r="L49" t="s" s="2">
+        <v>312</v>
+      </c>
+      <c r="M49" t="s" s="2">
         <v>313</v>
-      </c>
-      <c r="L49" t="s" s="2">
-        <v>314</v>
-      </c>
-      <c r="M49" t="s" s="2">
-        <v>315</v>
       </c>
       <c r="N49" s="2"/>
       <c r="O49" s="2"/>
@@ -7347,7 +7339,7 @@
         <v>81</v>
       </c>
       <c r="AF49" t="s" s="2">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="AG49" t="s" s="2">
         <v>79</v>
@@ -7377,15 +7369,15 @@
         <v>81</v>
       </c>
       <c r="AP49" t="s" s="2">
-        <v>316</v>
+        <v>314</v>
       </c>
     </row>
     <row r="50" hidden="true">
       <c r="A50" t="s" s="2">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" t="s" s="2">
@@ -7408,13 +7400,13 @@
         <v>81</v>
       </c>
       <c r="K50" t="s" s="2">
+        <v>149</v>
+      </c>
+      <c r="L50" t="s" s="2">
+        <v>150</v>
+      </c>
+      <c r="M50" t="s" s="2">
         <v>151</v>
-      </c>
-      <c r="L50" t="s" s="2">
-        <v>152</v>
-      </c>
-      <c r="M50" t="s" s="2">
-        <v>153</v>
       </c>
       <c r="N50" s="2"/>
       <c r="O50" s="2"/>
@@ -7465,7 +7457,7 @@
         <v>81</v>
       </c>
       <c r="AF50" t="s" s="2">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="AG50" t="s" s="2">
         <v>79</v>
@@ -7492,7 +7484,7 @@
         <v>81</v>
       </c>
       <c r="AO50" t="s" s="2">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="AP50" t="s" s="2">
         <v>81</v>
@@ -7500,14 +7492,14 @@
     </row>
     <row r="51" hidden="true">
       <c r="A51" t="s" s="2">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" t="s" s="2">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="E51" s="2"/>
       <c r="F51" t="s" s="2">
@@ -7529,13 +7521,13 @@
         <v>134</v>
       </c>
       <c r="L51" t="s" s="2">
+        <v>157</v>
+      </c>
+      <c r="M51" t="s" s="2">
+        <v>158</v>
+      </c>
+      <c r="N51" t="s" s="2">
         <v>159</v>
-      </c>
-      <c r="M51" t="s" s="2">
-        <v>160</v>
-      </c>
-      <c r="N51" t="s" s="2">
-        <v>161</v>
       </c>
       <c r="O51" s="2"/>
       <c r="P51" t="s" s="2">
@@ -7576,7 +7568,7 @@
         <v>137</v>
       </c>
       <c r="AC51" t="s" s="2">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="AD51" t="s" s="2">
         <v>81</v>
@@ -7585,7 +7577,7 @@
         <v>138</v>
       </c>
       <c r="AF51" t="s" s="2">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="AG51" t="s" s="2">
         <v>79</v>
@@ -7612,7 +7604,7 @@
         <v>81</v>
       </c>
       <c r="AO51" t="s" s="2">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="AP51" t="s" s="2">
         <v>81</v>
@@ -7620,14 +7612,14 @@
     </row>
     <row r="52" hidden="true">
       <c r="A52" t="s" s="2">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="B52" t="s" s="2">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="C52" s="2"/>
       <c r="D52" t="s" s="2">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="E52" s="2"/>
       <c r="F52" t="s" s="2">
@@ -7646,16 +7638,16 @@
         <v>90</v>
       </c>
       <c r="K52" t="s" s="2">
+        <v>319</v>
+      </c>
+      <c r="L52" t="s" s="2">
+        <v>320</v>
+      </c>
+      <c r="M52" t="s" s="2">
         <v>321</v>
       </c>
-      <c r="L52" t="s" s="2">
+      <c r="N52" t="s" s="2">
         <v>322</v>
-      </c>
-      <c r="M52" t="s" s="2">
-        <v>323</v>
-      </c>
-      <c r="N52" t="s" s="2">
-        <v>324</v>
       </c>
       <c r="O52" s="2"/>
       <c r="P52" t="s" s="2">
@@ -7669,70 +7661,70 @@
         <v>81</v>
       </c>
       <c r="T52" t="s" s="2">
+        <v>323</v>
+      </c>
+      <c r="U52" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="V52" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="W52" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="X52" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Y52" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Z52" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AA52" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AB52" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AC52" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AD52" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AE52" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AF52" t="s" s="2">
+        <v>324</v>
+      </c>
+      <c r="AG52" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH52" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="AI52" t="s" s="2">
         <v>325</v>
       </c>
-      <c r="U52" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="V52" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="W52" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="X52" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="Y52" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="Z52" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AA52" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AB52" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AC52" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AD52" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AE52" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AF52" t="s" s="2">
+      <c r="AJ52" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK52" t="s" s="2">
         <v>326</v>
       </c>
-      <c r="AG52" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH52" t="s" s="2">
-        <v>89</v>
-      </c>
-      <c r="AI52" t="s" s="2">
+      <c r="AL52" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM52" t="s" s="2">
+        <v>326</v>
+      </c>
+      <c r="AN52" t="s" s="2">
+        <v>326</v>
+      </c>
+      <c r="AO52" t="s" s="2">
         <v>327</v>
-      </c>
-      <c r="AJ52" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AK52" t="s" s="2">
-        <v>328</v>
-      </c>
-      <c r="AL52" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AM52" t="s" s="2">
-        <v>328</v>
-      </c>
-      <c r="AN52" t="s" s="2">
-        <v>328</v>
-      </c>
-      <c r="AO52" t="s" s="2">
-        <v>329</v>
       </c>
       <c r="AP52" t="s" s="2">
         <v>81</v>
@@ -7740,10 +7732,10 @@
     </row>
     <row r="53" hidden="true">
       <c r="A53" t="s" s="2">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" t="s" s="2">
@@ -7766,95 +7758,95 @@
         <v>90</v>
       </c>
       <c r="K53" t="s" s="2">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="L53" t="s" s="2">
+        <v>329</v>
+      </c>
+      <c r="M53" t="s" s="2">
+        <v>330</v>
+      </c>
+      <c r="N53" t="s" s="2">
         <v>331</v>
-      </c>
-      <c r="M53" t="s" s="2">
-        <v>332</v>
-      </c>
-      <c r="N53" t="s" s="2">
-        <v>333</v>
       </c>
       <c r="O53" s="2"/>
       <c r="P53" t="s" s="2">
         <v>81</v>
       </c>
       <c r="Q53" t="s" s="2">
+        <v>332</v>
+      </c>
+      <c r="R53" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="S53" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="T53" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="U53" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="V53" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="W53" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="X53" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Y53" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Z53" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AA53" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AB53" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AC53" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AD53" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AE53" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AF53" t="s" s="2">
+        <v>333</v>
+      </c>
+      <c r="AG53" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH53" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="AI53" t="s" s="2">
+        <v>325</v>
+      </c>
+      <c r="AJ53" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK53" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL53" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM53" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AN53" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AO53" t="s" s="2">
         <v>334</v>
-      </c>
-      <c r="R53" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="S53" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="T53" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="U53" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="V53" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="W53" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="X53" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="Y53" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="Z53" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AA53" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AB53" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AC53" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AD53" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AE53" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AF53" t="s" s="2">
-        <v>335</v>
-      </c>
-      <c r="AG53" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH53" t="s" s="2">
-        <v>89</v>
-      </c>
-      <c r="AI53" t="s" s="2">
-        <v>327</v>
-      </c>
-      <c r="AJ53" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AK53" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AL53" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AM53" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AN53" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AO53" t="s" s="2">
-        <v>336</v>
       </c>
       <c r="AP53" t="s" s="2">
         <v>81</v>
@@ -7862,10 +7854,10 @@
     </row>
     <row r="54" hidden="true">
       <c r="A54" t="s" s="2">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="B54" t="s" s="2">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="C54" s="2"/>
       <c r="D54" t="s" s="2">
@@ -7888,16 +7880,16 @@
         <v>90</v>
       </c>
       <c r="K54" t="s" s="2">
+        <v>336</v>
+      </c>
+      <c r="L54" t="s" s="2">
+        <v>337</v>
+      </c>
+      <c r="M54" t="s" s="2">
         <v>338</v>
       </c>
-      <c r="L54" t="s" s="2">
+      <c r="N54" t="s" s="2">
         <v>339</v>
-      </c>
-      <c r="M54" t="s" s="2">
-        <v>340</v>
-      </c>
-      <c r="N54" t="s" s="2">
-        <v>341</v>
       </c>
       <c r="O54" s="2"/>
       <c r="P54" t="s" s="2">
@@ -7947,7 +7939,7 @@
         <v>81</v>
       </c>
       <c r="AF54" t="s" s="2">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="AG54" t="s" s="2">
         <v>79</v>
@@ -7977,15 +7969,15 @@
         <v>81</v>
       </c>
       <c r="AP54" t="s" s="2">
-        <v>316</v>
+        <v>314</v>
       </c>
     </row>
     <row r="55" hidden="true">
       <c r="A55" t="s" s="2">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" t="s" s="2">
@@ -8008,13 +8000,13 @@
         <v>90</v>
       </c>
       <c r="K55" t="s" s="2">
+        <v>341</v>
+      </c>
+      <c r="L55" t="s" s="2">
+        <v>342</v>
+      </c>
+      <c r="M55" t="s" s="2">
         <v>343</v>
-      </c>
-      <c r="L55" t="s" s="2">
-        <v>344</v>
-      </c>
-      <c r="M55" t="s" s="2">
-        <v>345</v>
       </c>
       <c r="N55" s="2"/>
       <c r="O55" s="2"/>
@@ -8065,7 +8057,7 @@
         <v>81</v>
       </c>
       <c r="AF55" t="s" s="2">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="AG55" t="s" s="2">
         <v>79</v>
@@ -8083,27 +8075,27 @@
         <v>81</v>
       </c>
       <c r="AL55" t="s" s="2">
+        <v>344</v>
+      </c>
+      <c r="AM55" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AN55" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AO55" t="s" s="2">
+        <v>345</v>
+      </c>
+      <c r="AP55" t="s" s="2">
         <v>346</v>
-      </c>
-      <c r="AM55" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AN55" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AO55" t="s" s="2">
-        <v>347</v>
-      </c>
-      <c r="AP55" t="s" s="2">
-        <v>348</v>
       </c>
     </row>
     <row r="56" hidden="true">
       <c r="A56" t="s" s="2">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="B56" t="s" s="2">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="C56" s="2"/>
       <c r="D56" t="s" s="2">
@@ -8126,13 +8118,13 @@
         <v>81</v>
       </c>
       <c r="K56" t="s" s="2">
+        <v>149</v>
+      </c>
+      <c r="L56" t="s" s="2">
+        <v>150</v>
+      </c>
+      <c r="M56" t="s" s="2">
         <v>151</v>
-      </c>
-      <c r="L56" t="s" s="2">
-        <v>152</v>
-      </c>
-      <c r="M56" t="s" s="2">
-        <v>153</v>
       </c>
       <c r="N56" s="2"/>
       <c r="O56" s="2"/>
@@ -8183,7 +8175,7 @@
         <v>81</v>
       </c>
       <c r="AF56" t="s" s="2">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="AG56" t="s" s="2">
         <v>79</v>
@@ -8210,7 +8202,7 @@
         <v>81</v>
       </c>
       <c r="AO56" t="s" s="2">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="AP56" t="s" s="2">
         <v>81</v>
@@ -8218,10 +8210,10 @@
     </row>
     <row r="57" hidden="true">
       <c r="A57" t="s" s="2">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="B57" t="s" s="2">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="C57" s="2"/>
       <c r="D57" t="s" s="2">
@@ -8292,7 +8284,7 @@
         <v>137</v>
       </c>
       <c r="AC57" t="s" s="2">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="AD57" t="s" s="2">
         <v>81</v>
@@ -8301,7 +8293,7 @@
         <v>138</v>
       </c>
       <c r="AF57" t="s" s="2">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="AG57" t="s" s="2">
         <v>79</v>
@@ -8336,13 +8328,13 @@
     </row>
     <row r="58" hidden="true">
       <c r="A58" t="s" s="2">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="B58" t="s" s="2">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="C58" t="s" s="2">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="D58" t="s" s="2">
         <v>81</v>
@@ -8364,13 +8356,13 @@
         <v>81</v>
       </c>
       <c r="K58" t="s" s="2">
+        <v>290</v>
+      </c>
+      <c r="L58" t="s" s="2">
+        <v>291</v>
+      </c>
+      <c r="M58" t="s" s="2">
         <v>292</v>
-      </c>
-      <c r="L58" t="s" s="2">
-        <v>293</v>
-      </c>
-      <c r="M58" t="s" s="2">
-        <v>294</v>
       </c>
       <c r="N58" s="2"/>
       <c r="O58" s="2"/>
@@ -8421,7 +8413,7 @@
         <v>81</v>
       </c>
       <c r="AF58" t="s" s="2">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="AG58" t="s" s="2">
         <v>79</v>
@@ -8456,10 +8448,10 @@
     </row>
     <row r="59" hidden="true">
       <c r="A59" t="s" s="2">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B59" t="s" s="2">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="C59" s="2"/>
       <c r="D59" t="s" s="2">
@@ -8482,16 +8474,16 @@
         <v>90</v>
       </c>
       <c r="K59" t="s" s="2">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="L59" t="s" s="2">
+        <v>294</v>
+      </c>
+      <c r="M59" t="s" s="2">
+        <v>295</v>
+      </c>
+      <c r="N59" t="s" s="2">
         <v>296</v>
-      </c>
-      <c r="M59" t="s" s="2">
-        <v>297</v>
-      </c>
-      <c r="N59" t="s" s="2">
-        <v>298</v>
       </c>
       <c r="O59" s="2"/>
       <c r="P59" t="s" s="2">
@@ -8541,7 +8533,7 @@
         <v>81</v>
       </c>
       <c r="AF59" t="s" s="2">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="AG59" t="s" s="2">
         <v>79</v>
@@ -8550,7 +8542,7 @@
         <v>89</v>
       </c>
       <c r="AI59" t="s" s="2">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="AJ59" t="s" s="2">
         <v>81</v>
@@ -8576,10 +8568,10 @@
     </row>
     <row r="60" hidden="true">
       <c r="A60" t="s" s="2">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="B60" t="s" s="2">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="C60" s="2"/>
       <c r="D60" t="s" s="2">
@@ -8602,16 +8594,16 @@
         <v>90</v>
       </c>
       <c r="K60" t="s" s="2">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="L60" t="s" s="2">
+        <v>300</v>
+      </c>
+      <c r="M60" t="s" s="2">
+        <v>301</v>
+      </c>
+      <c r="N60" t="s" s="2">
         <v>302</v>
-      </c>
-      <c r="M60" t="s" s="2">
-        <v>303</v>
-      </c>
-      <c r="N60" t="s" s="2">
-        <v>304</v>
       </c>
       <c r="O60" s="2"/>
       <c r="P60" t="s" s="2">
@@ -8661,7 +8653,7 @@
         <v>81</v>
       </c>
       <c r="AF60" t="s" s="2">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="AG60" t="s" s="2">
         <v>79</v>
@@ -8688,7 +8680,7 @@
         <v>81</v>
       </c>
       <c r="AO60" t="s" s="2">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="AP60" t="s" s="2">
         <v>81</v>
@@ -8696,10 +8688,10 @@
     </row>
     <row r="61" hidden="true">
       <c r="A61" t="s" s="2">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="B61" t="s" s="2">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="C61" s="2"/>
       <c r="D61" t="s" s="2">
@@ -8722,16 +8714,16 @@
         <v>90</v>
       </c>
       <c r="K61" t="s" s="2">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="L61" t="s" s="2">
+        <v>306</v>
+      </c>
+      <c r="M61" t="s" s="2">
+        <v>307</v>
+      </c>
+      <c r="N61" t="s" s="2">
         <v>308</v>
-      </c>
-      <c r="M61" t="s" s="2">
-        <v>309</v>
-      </c>
-      <c r="N61" t="s" s="2">
-        <v>310</v>
       </c>
       <c r="O61" s="2"/>
       <c r="P61" t="s" s="2">
@@ -8781,7 +8773,7 @@
         <v>81</v>
       </c>
       <c r="AF61" t="s" s="2">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="AG61" t="s" s="2">
         <v>79</v>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@3f939d9d0a488b992904da01a096a36c4fba3db3 🚀
</commit_message>
<xml_diff>
--- a/StructureDefinition-Flag.xlsx
+++ b/StructureDefinition-Flag.xlsx
@@ -10,13 +10,13 @@
     <sheet name="Elements" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AP$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AP$47</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2351" uniqueCount="354">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1817" uniqueCount="312">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-12-10T07:51:08+00:00</t>
+    <t>2024-12-10T08:19:29+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -704,112 +704,6 @@
     <t>union(., ./translation)</t>
   </si>
   <si>
-    <t>Flag.category.coding.id</t>
-  </si>
-  <si>
-    <t>Flag.category.coding.extension</t>
-  </si>
-  <si>
-    <t>Flag.category.coding.system</t>
-  </si>
-  <si>
-    <t>Identity of the terminology system</t>
-  </si>
-  <si>
-    <t>The identification of the code system that defines the meaning of the symbol in the code.</t>
-  </si>
-  <si>
-    <t>The URI may be an OID (urn:oid:...) or a UUID (urn:uuid:...).  OIDs and UUIDs SHALL be references to the HL7 OID registry. Otherwise, the URI should come from HL7's list of FHIR defined special URIs or it should de-reference to some definition that establish the system clearly and unambiguously.</t>
-  </si>
-  <si>
-    <t>Need to be unambiguous about the source of the definition of the symbol.</t>
-  </si>
-  <si>
-    <t>Coding.system</t>
-  </si>
-  <si>
-    <t>./codeSystem</t>
-  </si>
-  <si>
-    <t>Flag.category.coding.version</t>
-  </si>
-  <si>
-    <t>Version of the system - if relevant</t>
-  </si>
-  <si>
-    <t>The version of the code system which was used when choosing this code. Note that a well-maintained code system does not need the version reported, because the meaning of codes is consistent across versions. However this cannot consistently be assured. and when the meaning is not guaranteed to be consistent, the version SHOULD be exchanged.</t>
-  </si>
-  <si>
-    <t>Where the terminology does not clearly define what string should be used to identify code system versions, the recommendation is to use the date (expressed in FHIR date format) on which that version was officially published as the version date.</t>
-  </si>
-  <si>
-    <t>Coding.version</t>
-  </si>
-  <si>
-    <t>./codeSystemVersion</t>
-  </si>
-  <si>
-    <t>Flag.category.coding.code</t>
-  </si>
-  <si>
-    <t>Symbol in syntax defined by the system</t>
-  </si>
-  <si>
-    <t>A symbol in syntax defined by the system. The symbol may be a predefined code or an expression in a syntax defined by the coding system (e.g. post-coordination).</t>
-  </si>
-  <si>
-    <t>Need to refer to a particular code in the system.</t>
-  </si>
-  <si>
-    <t>Coding.code</t>
-  </si>
-  <si>
-    <t>./code</t>
-  </si>
-  <si>
-    <t>Flag.category.coding.display</t>
-  </si>
-  <si>
-    <t>Representation defined by the system</t>
-  </si>
-  <si>
-    <t>A representation of the meaning of the code in the system, following the rules of the system.</t>
-  </si>
-  <si>
-    <t>Need to be able to carry a human-readable meaning of the code for readers that do not know  the system.</t>
-  </si>
-  <si>
-    <t>Coding.display</t>
-  </si>
-  <si>
-    <t>CV.displayName</t>
-  </si>
-  <si>
-    <t>Flag.category.coding.userSelected</t>
-  </si>
-  <si>
-    <t xml:space="preserve">boolean
-</t>
-  </si>
-  <si>
-    <t>If this coding was chosen directly by the user</t>
-  </si>
-  <si>
-    <t>Indicates that this coding was chosen by a user directly - i.e. off a pick list of available items (codes or displays).</t>
-  </si>
-  <si>
-    <t>Amongst a set of alternatives, a directly chosen code is the most appropriate starting point for new translations. There is some ambiguity about what exactly 'directly chosen' implies, and trading partner agreement may be needed to clarify the use of this element and its consequences more completely.</t>
-  </si>
-  <si>
-    <t>This has been identified as a clinical safety criterium - that this exact system/code pair was chosen explicitly, rather than inferred by the system based on some rules or language processing.</t>
-  </si>
-  <si>
-    <t>Coding.userSelected</t>
-  </si>
-  <si>
-    <t>CD.codingRationale</t>
-  </si>
-  <si>
     <t>Flag.category.text</t>
   </si>
   <si>
@@ -876,27 +770,6 @@
   </si>
   <si>
     <t>Flag.code.coding</t>
-  </si>
-  <si>
-    <t>Flag.code.coding.id</t>
-  </si>
-  <si>
-    <t>Flag.code.coding.extension</t>
-  </si>
-  <si>
-    <t>Flag.code.coding.system</t>
-  </si>
-  <si>
-    <t>Flag.code.coding.version</t>
-  </si>
-  <si>
-    <t>Flag.code.coding.code</t>
-  </si>
-  <si>
-    <t>Flag.code.coding.display</t>
-  </si>
-  <si>
-    <t>Flag.code.coding.userSelected</t>
   </si>
   <si>
     <t>Flag.code.text</t>
@@ -1455,11 +1328,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AP61"/>
+  <dimension ref="A1:AP47"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="61.9609375" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="32.8203125" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="29.39453125" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="18.015625" customWidth="true" bestFit="true" hidden="true"/>
     <col min="4" max="4" width="39.9140625" customWidth="true" bestFit="true" hidden="true"/>
     <col min="5" max="5" width="6.77734375" customWidth="true" bestFit="true"/>
@@ -4036,25 +3909,29 @@
         <v>90</v>
       </c>
       <c r="H22" t="s" s="2">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="I22" t="s" s="2">
         <v>82</v>
       </c>
       <c r="J22" t="s" s="2">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="K22" t="s" s="2">
         <v>150</v>
       </c>
       <c r="L22" t="s" s="2">
-        <v>151</v>
+        <v>219</v>
       </c>
       <c r="M22" t="s" s="2">
-        <v>152</v>
-      </c>
-      <c r="N22" s="2"/>
-      <c r="O22" s="2"/>
+        <v>220</v>
+      </c>
+      <c r="N22" t="s" s="2">
+        <v>221</v>
+      </c>
+      <c r="O22" t="s" s="2">
+        <v>222</v>
+      </c>
       <c r="P22" t="s" s="2">
         <v>82</v>
       </c>
@@ -4102,7 +3979,7 @@
         <v>82</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>153</v>
+        <v>223</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>80</v>
@@ -4129,7 +4006,7 @@
         <v>82</v>
       </c>
       <c r="AO22" t="s" s="2">
-        <v>154</v>
+        <v>224</v>
       </c>
       <c r="AP22" t="s" s="2">
         <v>82</v>
@@ -4137,21 +4014,21 @@
     </row>
     <row r="23" hidden="true">
       <c r="A23" t="s" s="2">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
-        <v>157</v>
+        <v>226</v>
       </c>
       <c r="E23" s="2"/>
       <c r="F23" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G23" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="H23" t="s" s="2">
         <v>82</v>
@@ -4160,19 +4037,19 @@
         <v>82</v>
       </c>
       <c r="J23" t="s" s="2">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="K23" t="s" s="2">
-        <v>135</v>
+        <v>200</v>
       </c>
       <c r="L23" t="s" s="2">
-        <v>158</v>
+        <v>227</v>
       </c>
       <c r="M23" t="s" s="2">
-        <v>159</v>
+        <v>228</v>
       </c>
       <c r="N23" t="s" s="2">
-        <v>160</v>
+        <v>229</v>
       </c>
       <c r="O23" s="2"/>
       <c r="P23" t="s" s="2">
@@ -4186,7 +4063,7 @@
         <v>82</v>
       </c>
       <c r="T23" t="s" s="2">
-        <v>82</v>
+        <v>230</v>
       </c>
       <c r="U23" t="s" s="2">
         <v>82</v>
@@ -4198,37 +4075,35 @@
         <v>82</v>
       </c>
       <c r="X23" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y23" t="s" s="2">
-        <v>82</v>
-      </c>
+        <v>113</v>
+      </c>
+      <c r="Y23" s="2"/>
       <c r="Z23" t="s" s="2">
-        <v>82</v>
+        <v>231</v>
       </c>
       <c r="AA23" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AB23" t="s" s="2">
-        <v>138</v>
+        <v>82</v>
       </c>
       <c r="AC23" t="s" s="2">
-        <v>161</v>
+        <v>82</v>
       </c>
       <c r="AD23" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AE23" t="s" s="2">
-        <v>139</v>
+        <v>82</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>162</v>
+        <v>225</v>
       </c>
       <c r="AG23" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="AH23" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="AI23" t="s" s="2">
         <v>82</v>
@@ -4237,30 +4112,30 @@
         <v>82</v>
       </c>
       <c r="AK23" t="s" s="2">
-        <v>82</v>
+        <v>232</v>
       </c>
       <c r="AL23" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AM23" t="s" s="2">
-        <v>82</v>
+        <v>232</v>
       </c>
       <c r="AN23" t="s" s="2">
-        <v>82</v>
+        <v>232</v>
       </c>
       <c r="AO23" t="s" s="2">
-        <v>154</v>
+        <v>233</v>
       </c>
       <c r="AP23" t="s" s="2">
-        <v>82</v>
+        <v>234</v>
       </c>
     </row>
     <row r="24" hidden="true">
       <c r="A24" t="s" s="2">
-        <v>220</v>
+        <v>235</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>220</v>
+        <v>235</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -4280,23 +4155,19 @@
         <v>82</v>
       </c>
       <c r="J24" t="s" s="2">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="K24" t="s" s="2">
-        <v>103</v>
+        <v>150</v>
       </c>
       <c r="L24" t="s" s="2">
-        <v>221</v>
+        <v>151</v>
       </c>
       <c r="M24" t="s" s="2">
-        <v>222</v>
-      </c>
-      <c r="N24" t="s" s="2">
-        <v>223</v>
-      </c>
-      <c r="O24" t="s" s="2">
-        <v>224</v>
-      </c>
+        <v>152</v>
+      </c>
+      <c r="N24" s="2"/>
+      <c r="O24" s="2"/>
       <c r="P24" t="s" s="2">
         <v>82</v>
       </c>
@@ -4344,7 +4215,7 @@
         <v>82</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>225</v>
+        <v>153</v>
       </c>
       <c r="AG24" t="s" s="2">
         <v>80</v>
@@ -4371,7 +4242,7 @@
         <v>82</v>
       </c>
       <c r="AO24" t="s" s="2">
-        <v>226</v>
+        <v>154</v>
       </c>
       <c r="AP24" t="s" s="2">
         <v>82</v>
@@ -4379,21 +4250,21 @@
     </row>
     <row r="25" hidden="true">
       <c r="A25" t="s" s="2">
-        <v>227</v>
+        <v>236</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>227</v>
+        <v>236</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
-        <v>82</v>
+        <v>157</v>
       </c>
       <c r="E25" s="2"/>
       <c r="F25" t="s" s="2">
         <v>80</v>
       </c>
       <c r="G25" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="H25" t="s" s="2">
         <v>82</v>
@@ -4402,19 +4273,19 @@
         <v>82</v>
       </c>
       <c r="J25" t="s" s="2">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="K25" t="s" s="2">
-        <v>150</v>
+        <v>135</v>
       </c>
       <c r="L25" t="s" s="2">
-        <v>228</v>
+        <v>158</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>229</v>
+        <v>159</v>
       </c>
       <c r="N25" t="s" s="2">
-        <v>230</v>
+        <v>160</v>
       </c>
       <c r="O25" s="2"/>
       <c r="P25" t="s" s="2">
@@ -4452,25 +4323,25 @@
         <v>82</v>
       </c>
       <c r="AB25" t="s" s="2">
-        <v>82</v>
+        <v>138</v>
       </c>
       <c r="AC25" t="s" s="2">
-        <v>82</v>
+        <v>161</v>
       </c>
       <c r="AD25" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AE25" t="s" s="2">
-        <v>82</v>
+        <v>139</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>231</v>
+        <v>162</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH25" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="AI25" t="s" s="2">
         <v>82</v>
@@ -4491,7 +4362,7 @@
         <v>82</v>
       </c>
       <c r="AO25" t="s" s="2">
-        <v>232</v>
+        <v>154</v>
       </c>
       <c r="AP25" t="s" s="2">
         <v>82</v>
@@ -4499,10 +4370,10 @@
     </row>
     <row r="26" hidden="true">
       <c r="A26" t="s" s="2">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
@@ -4513,7 +4384,7 @@
         <v>80</v>
       </c>
       <c r="G26" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="H26" t="s" s="2">
         <v>82</v>
@@ -4525,17 +4396,19 @@
         <v>91</v>
       </c>
       <c r="K26" t="s" s="2">
-        <v>109</v>
+        <v>211</v>
       </c>
       <c r="L26" t="s" s="2">
-        <v>234</v>
+        <v>212</v>
       </c>
       <c r="M26" t="s" s="2">
-        <v>235</v>
-      </c>
-      <c r="N26" s="2"/>
+        <v>213</v>
+      </c>
+      <c r="N26" t="s" s="2">
+        <v>214</v>
+      </c>
       <c r="O26" t="s" s="2">
-        <v>236</v>
+        <v>215</v>
       </c>
       <c r="P26" t="s" s="2">
         <v>82</v>
@@ -4584,13 +4457,13 @@
         <v>82</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>237</v>
+        <v>216</v>
       </c>
       <c r="AG26" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH26" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="AI26" t="s" s="2">
         <v>82</v>
@@ -4611,7 +4484,7 @@
         <v>82</v>
       </c>
       <c r="AO26" t="s" s="2">
-        <v>238</v>
+        <v>217</v>
       </c>
       <c r="AP26" t="s" s="2">
         <v>82</v>
@@ -4619,10 +4492,10 @@
     </row>
     <row r="27" hidden="true">
       <c r="A27" t="s" s="2">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
@@ -4648,14 +4521,16 @@
         <v>150</v>
       </c>
       <c r="L27" t="s" s="2">
-        <v>240</v>
+        <v>219</v>
       </c>
       <c r="M27" t="s" s="2">
-        <v>241</v>
-      </c>
-      <c r="N27" s="2"/>
+        <v>220</v>
+      </c>
+      <c r="N27" t="s" s="2">
+        <v>221</v>
+      </c>
       <c r="O27" t="s" s="2">
-        <v>242</v>
+        <v>222</v>
       </c>
       <c r="P27" t="s" s="2">
         <v>82</v>
@@ -4704,7 +4579,7 @@
         <v>82</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>243</v>
+        <v>223</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>80</v>
@@ -4731,7 +4606,7 @@
         <v>82</v>
       </c>
       <c r="AO27" t="s" s="2">
-        <v>244</v>
+        <v>224</v>
       </c>
       <c r="AP27" t="s" s="2">
         <v>82</v>
@@ -4739,10 +4614,10 @@
     </row>
     <row r="28" hidden="true">
       <c r="A28" t="s" s="2">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -4750,7 +4625,7 @@
       </c>
       <c r="E28" s="2"/>
       <c r="F28" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G28" t="s" s="2">
         <v>90</v>
@@ -4765,20 +4640,16 @@
         <v>91</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>246</v>
+        <v>240</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>248</v>
-      </c>
-      <c r="N28" t="s" s="2">
-        <v>249</v>
-      </c>
-      <c r="O28" t="s" s="2">
-        <v>250</v>
-      </c>
+        <v>242</v>
+      </c>
+      <c r="N28" s="2"/>
+      <c r="O28" s="2"/>
       <c r="P28" t="s" s="2">
         <v>82</v>
       </c>
@@ -4826,10 +4697,10 @@
         <v>82</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>251</v>
+        <v>239</v>
       </c>
       <c r="AG28" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="AH28" t="s" s="2">
         <v>90</v>
@@ -4853,18 +4724,18 @@
         <v>82</v>
       </c>
       <c r="AO28" t="s" s="2">
-        <v>252</v>
+        <v>243</v>
       </c>
       <c r="AP28" t="s" s="2">
-        <v>82</v>
+        <v>244</v>
       </c>
     </row>
     <row r="29" hidden="true">
       <c r="A29" t="s" s="2">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -4878,29 +4749,25 @@
         <v>90</v>
       </c>
       <c r="H29" t="s" s="2">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="I29" t="s" s="2">
         <v>82</v>
       </c>
       <c r="J29" t="s" s="2">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="K29" t="s" s="2">
         <v>150</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>254</v>
+        <v>151</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>255</v>
-      </c>
-      <c r="N29" t="s" s="2">
-        <v>256</v>
-      </c>
-      <c r="O29" t="s" s="2">
-        <v>257</v>
-      </c>
+        <v>152</v>
+      </c>
+      <c r="N29" s="2"/>
+      <c r="O29" s="2"/>
       <c r="P29" t="s" s="2">
         <v>82</v>
       </c>
@@ -4948,7 +4815,7 @@
         <v>82</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>258</v>
+        <v>153</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>80</v>
@@ -4975,7 +4842,7 @@
         <v>82</v>
       </c>
       <c r="AO29" t="s" s="2">
-        <v>259</v>
+        <v>154</v>
       </c>
       <c r="AP29" t="s" s="2">
         <v>82</v>
@@ -4983,21 +4850,21 @@
     </row>
     <row r="30" hidden="true">
       <c r="A30" t="s" s="2">
-        <v>260</v>
+        <v>246</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>260</v>
+        <v>246</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
-        <v>261</v>
+        <v>82</v>
       </c>
       <c r="E30" s="2"/>
       <c r="F30" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="G30" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="H30" t="s" s="2">
         <v>82</v>
@@ -5006,20 +4873,18 @@
         <v>82</v>
       </c>
       <c r="J30" t="s" s="2">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>200</v>
+        <v>135</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>262</v>
+        <v>136</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>263</v>
-      </c>
-      <c r="N30" t="s" s="2">
-        <v>264</v>
-      </c>
+        <v>137</v>
+      </c>
+      <c r="N30" s="2"/>
       <c r="O30" s="2"/>
       <c r="P30" t="s" s="2">
         <v>82</v>
@@ -5032,7 +4897,7 @@
         <v>82</v>
       </c>
       <c r="T30" t="s" s="2">
-        <v>265</v>
+        <v>82</v>
       </c>
       <c r="U30" t="s" s="2">
         <v>82</v>
@@ -5044,35 +4909,37 @@
         <v>82</v>
       </c>
       <c r="X30" t="s" s="2">
-        <v>113</v>
-      </c>
-      <c r="Y30" s="2"/>
+        <v>82</v>
+      </c>
+      <c r="Y30" t="s" s="2">
+        <v>82</v>
+      </c>
       <c r="Z30" t="s" s="2">
-        <v>266</v>
+        <v>82</v>
       </c>
       <c r="AA30" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AB30" t="s" s="2">
-        <v>82</v>
+        <v>138</v>
       </c>
       <c r="AC30" t="s" s="2">
-        <v>82</v>
+        <v>161</v>
       </c>
       <c r="AD30" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AE30" t="s" s="2">
-        <v>82</v>
+        <v>139</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>260</v>
+        <v>162</v>
       </c>
       <c r="AG30" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="AH30" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="AI30" t="s" s="2">
         <v>82</v>
@@ -5081,32 +4948,34 @@
         <v>82</v>
       </c>
       <c r="AK30" t="s" s="2">
-        <v>267</v>
+        <v>82</v>
       </c>
       <c r="AL30" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AM30" t="s" s="2">
-        <v>267</v>
+        <v>82</v>
       </c>
       <c r="AN30" t="s" s="2">
-        <v>267</v>
+        <v>82</v>
       </c>
       <c r="AO30" t="s" s="2">
-        <v>268</v>
+        <v>82</v>
       </c>
       <c r="AP30" t="s" s="2">
-        <v>269</v>
+        <v>82</v>
       </c>
     </row>
     <row r="31" hidden="true">
       <c r="A31" t="s" s="2">
-        <v>270</v>
+        <v>247</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>270</v>
-      </c>
-      <c r="C31" s="2"/>
+        <v>246</v>
+      </c>
+      <c r="C31" t="s" s="2">
+        <v>248</v>
+      </c>
       <c r="D31" t="s" s="2">
         <v>82</v>
       </c>
@@ -5127,13 +4996,13 @@
         <v>82</v>
       </c>
       <c r="K31" t="s" s="2">
-        <v>150</v>
+        <v>249</v>
       </c>
       <c r="L31" t="s" s="2">
-        <v>151</v>
+        <v>250</v>
       </c>
       <c r="M31" t="s" s="2">
-        <v>152</v>
+        <v>251</v>
       </c>
       <c r="N31" s="2"/>
       <c r="O31" s="2"/>
@@ -5184,13 +5053,13 @@
         <v>82</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>153</v>
+        <v>162</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH31" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="AI31" t="s" s="2">
         <v>82</v>
@@ -5211,7 +5080,7 @@
         <v>82</v>
       </c>
       <c r="AO31" t="s" s="2">
-        <v>154</v>
+        <v>133</v>
       </c>
       <c r="AP31" t="s" s="2">
         <v>82</v>
@@ -5219,21 +5088,21 @@
     </row>
     <row r="32" hidden="true">
       <c r="A32" t="s" s="2">
-        <v>271</v>
+        <v>252</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>271</v>
+        <v>252</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
-        <v>157</v>
+        <v>82</v>
       </c>
       <c r="E32" s="2"/>
       <c r="F32" t="s" s="2">
         <v>80</v>
       </c>
       <c r="G32" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="H32" t="s" s="2">
         <v>82</v>
@@ -5242,19 +5111,19 @@
         <v>82</v>
       </c>
       <c r="J32" t="s" s="2">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="K32" t="s" s="2">
-        <v>135</v>
+        <v>150</v>
       </c>
       <c r="L32" t="s" s="2">
-        <v>158</v>
+        <v>253</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>159</v>
+        <v>254</v>
       </c>
       <c r="N32" t="s" s="2">
-        <v>160</v>
+        <v>255</v>
       </c>
       <c r="O32" s="2"/>
       <c r="P32" t="s" s="2">
@@ -5292,28 +5161,28 @@
         <v>82</v>
       </c>
       <c r="AB32" t="s" s="2">
-        <v>138</v>
+        <v>82</v>
       </c>
       <c r="AC32" t="s" s="2">
-        <v>161</v>
+        <v>82</v>
       </c>
       <c r="AD32" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AE32" t="s" s="2">
-        <v>139</v>
+        <v>82</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>162</v>
+        <v>256</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH32" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="AI32" t="s" s="2">
-        <v>82</v>
+        <v>257</v>
       </c>
       <c r="AJ32" t="s" s="2">
         <v>82</v>
@@ -5331,7 +5200,7 @@
         <v>82</v>
       </c>
       <c r="AO32" t="s" s="2">
-        <v>154</v>
+        <v>133</v>
       </c>
       <c r="AP32" t="s" s="2">
         <v>82</v>
@@ -5339,10 +5208,10 @@
     </row>
     <row r="33" hidden="true">
       <c r="A33" t="s" s="2">
-        <v>272</v>
+        <v>258</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>272</v>
+        <v>258</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
@@ -5353,7 +5222,7 @@
         <v>80</v>
       </c>
       <c r="G33" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="H33" t="s" s="2">
         <v>82</v>
@@ -5365,20 +5234,18 @@
         <v>91</v>
       </c>
       <c r="K33" t="s" s="2">
-        <v>211</v>
+        <v>183</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>212</v>
+        <v>259</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>213</v>
+        <v>260</v>
       </c>
       <c r="N33" t="s" s="2">
-        <v>214</v>
-      </c>
-      <c r="O33" t="s" s="2">
-        <v>215</v>
-      </c>
+        <v>261</v>
+      </c>
+      <c r="O33" s="2"/>
       <c r="P33" t="s" s="2">
         <v>82</v>
       </c>
@@ -5426,13 +5293,13 @@
         <v>82</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>216</v>
+        <v>262</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH33" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="AI33" t="s" s="2">
         <v>82</v>
@@ -5453,7 +5320,7 @@
         <v>82</v>
       </c>
       <c r="AO33" t="s" s="2">
-        <v>217</v>
+        <v>263</v>
       </c>
       <c r="AP33" t="s" s="2">
         <v>82</v>
@@ -5461,10 +5328,10 @@
     </row>
     <row r="34" hidden="true">
       <c r="A34" t="s" s="2">
-        <v>273</v>
+        <v>264</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>273</v>
+        <v>264</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
@@ -5484,18 +5351,20 @@
         <v>82</v>
       </c>
       <c r="J34" t="s" s="2">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="K34" t="s" s="2">
         <v>150</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>151</v>
+        <v>265</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>152</v>
-      </c>
-      <c r="N34" s="2"/>
+        <v>266</v>
+      </c>
+      <c r="N34" t="s" s="2">
+        <v>267</v>
+      </c>
       <c r="O34" s="2"/>
       <c r="P34" t="s" s="2">
         <v>82</v>
@@ -5544,7 +5413,7 @@
         <v>82</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>153</v>
+        <v>268</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>80</v>
@@ -5571,7 +5440,7 @@
         <v>82</v>
       </c>
       <c r="AO34" t="s" s="2">
-        <v>154</v>
+        <v>133</v>
       </c>
       <c r="AP34" t="s" s="2">
         <v>82</v>
@@ -5579,21 +5448,21 @@
     </row>
     <row r="35" hidden="true">
       <c r="A35" t="s" s="2">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
-        <v>157</v>
+        <v>82</v>
       </c>
       <c r="E35" s="2"/>
       <c r="F35" t="s" s="2">
         <v>80</v>
       </c>
       <c r="G35" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="H35" t="s" s="2">
         <v>82</v>
@@ -5602,20 +5471,18 @@
         <v>82</v>
       </c>
       <c r="J35" t="s" s="2">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>135</v>
+        <v>270</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>158</v>
+        <v>271</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>159</v>
-      </c>
-      <c r="N35" t="s" s="2">
-        <v>160</v>
-      </c>
+        <v>272</v>
+      </c>
+      <c r="N35" s="2"/>
       <c r="O35" s="2"/>
       <c r="P35" t="s" s="2">
         <v>82</v>
@@ -5652,25 +5519,25 @@
         <v>82</v>
       </c>
       <c r="AB35" t="s" s="2">
-        <v>138</v>
+        <v>82</v>
       </c>
       <c r="AC35" t="s" s="2">
-        <v>161</v>
+        <v>82</v>
       </c>
       <c r="AD35" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AE35" t="s" s="2">
-        <v>139</v>
+        <v>82</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>162</v>
+        <v>269</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH35" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="AI35" t="s" s="2">
         <v>82</v>
@@ -5691,18 +5558,18 @@
         <v>82</v>
       </c>
       <c r="AO35" t="s" s="2">
-        <v>154</v>
+        <v>82</v>
       </c>
       <c r="AP35" t="s" s="2">
-        <v>82</v>
+        <v>273</v>
       </c>
     </row>
     <row r="36" hidden="true">
       <c r="A36" t="s" s="2">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
@@ -5722,23 +5589,19 @@
         <v>82</v>
       </c>
       <c r="J36" t="s" s="2">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="K36" t="s" s="2">
-        <v>103</v>
+        <v>150</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>221</v>
+        <v>151</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>222</v>
-      </c>
-      <c r="N36" t="s" s="2">
-        <v>223</v>
-      </c>
-      <c r="O36" t="s" s="2">
-        <v>224</v>
-      </c>
+        <v>152</v>
+      </c>
+      <c r="N36" s="2"/>
+      <c r="O36" s="2"/>
       <c r="P36" t="s" s="2">
         <v>82</v>
       </c>
@@ -5786,7 +5649,7 @@
         <v>82</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>225</v>
+        <v>153</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>80</v>
@@ -5813,7 +5676,7 @@
         <v>82</v>
       </c>
       <c r="AO36" t="s" s="2">
-        <v>226</v>
+        <v>154</v>
       </c>
       <c r="AP36" t="s" s="2">
         <v>82</v>
@@ -5821,21 +5684,21 @@
     </row>
     <row r="37" hidden="true">
       <c r="A37" t="s" s="2">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
-        <v>82</v>
+        <v>157</v>
       </c>
       <c r="E37" s="2"/>
       <c r="F37" t="s" s="2">
         <v>80</v>
       </c>
       <c r="G37" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="H37" t="s" s="2">
         <v>82</v>
@@ -5844,19 +5707,19 @@
         <v>82</v>
       </c>
       <c r="J37" t="s" s="2">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="K37" t="s" s="2">
-        <v>150</v>
+        <v>135</v>
       </c>
       <c r="L37" t="s" s="2">
-        <v>228</v>
+        <v>158</v>
       </c>
       <c r="M37" t="s" s="2">
-        <v>229</v>
+        <v>159</v>
       </c>
       <c r="N37" t="s" s="2">
-        <v>230</v>
+        <v>160</v>
       </c>
       <c r="O37" s="2"/>
       <c r="P37" t="s" s="2">
@@ -5894,25 +5757,25 @@
         <v>82</v>
       </c>
       <c r="AB37" t="s" s="2">
-        <v>82</v>
+        <v>138</v>
       </c>
       <c r="AC37" t="s" s="2">
-        <v>82</v>
+        <v>161</v>
       </c>
       <c r="AD37" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AE37" t="s" s="2">
-        <v>82</v>
+        <v>139</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>231</v>
+        <v>162</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH37" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="AI37" t="s" s="2">
         <v>82</v>
@@ -5933,7 +5796,7 @@
         <v>82</v>
       </c>
       <c r="AO37" t="s" s="2">
-        <v>232</v>
+        <v>154</v>
       </c>
       <c r="AP37" t="s" s="2">
         <v>82</v>
@@ -5941,14 +5804,14 @@
     </row>
     <row r="38" hidden="true">
       <c r="A38" t="s" s="2">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
-        <v>82</v>
+        <v>277</v>
       </c>
       <c r="E38" s="2"/>
       <c r="F38" t="s" s="2">
@@ -5958,7 +5821,7 @@
         <v>90</v>
       </c>
       <c r="H38" t="s" s="2">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="I38" t="s" s="2">
         <v>82</v>
@@ -5967,18 +5830,18 @@
         <v>91</v>
       </c>
       <c r="K38" t="s" s="2">
-        <v>109</v>
+        <v>278</v>
       </c>
       <c r="L38" t="s" s="2">
-        <v>234</v>
+        <v>279</v>
       </c>
       <c r="M38" t="s" s="2">
-        <v>235</v>
-      </c>
-      <c r="N38" s="2"/>
-      <c r="O38" t="s" s="2">
-        <v>236</v>
-      </c>
+        <v>280</v>
+      </c>
+      <c r="N38" t="s" s="2">
+        <v>281</v>
+      </c>
+      <c r="O38" s="2"/>
       <c r="P38" t="s" s="2">
         <v>82</v>
       </c>
@@ -5990,7 +5853,7 @@
         <v>82</v>
       </c>
       <c r="T38" t="s" s="2">
-        <v>82</v>
+        <v>282</v>
       </c>
       <c r="U38" t="s" s="2">
         <v>82</v>
@@ -6026,7 +5889,7 @@
         <v>82</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>237</v>
+        <v>283</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>80</v>
@@ -6035,25 +5898,25 @@
         <v>90</v>
       </c>
       <c r="AI38" t="s" s="2">
-        <v>82</v>
+        <v>284</v>
       </c>
       <c r="AJ38" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AK38" t="s" s="2">
-        <v>82</v>
+        <v>285</v>
       </c>
       <c r="AL38" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AM38" t="s" s="2">
-        <v>82</v>
+        <v>285</v>
       </c>
       <c r="AN38" t="s" s="2">
-        <v>82</v>
+        <v>285</v>
       </c>
       <c r="AO38" t="s" s="2">
-        <v>238</v>
+        <v>286</v>
       </c>
       <c r="AP38" t="s" s="2">
         <v>82</v>
@@ -6061,10 +5924,10 @@
     </row>
     <row r="39" hidden="true">
       <c r="A39" t="s" s="2">
-        <v>278</v>
+        <v>287</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>278</v>
+        <v>287</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
@@ -6078,7 +5941,7 @@
         <v>90</v>
       </c>
       <c r="H39" t="s" s="2">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="I39" t="s" s="2">
         <v>82</v>
@@ -6087,22 +5950,24 @@
         <v>91</v>
       </c>
       <c r="K39" t="s" s="2">
-        <v>150</v>
+        <v>278</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>240</v>
+        <v>288</v>
       </c>
       <c r="M39" t="s" s="2">
-        <v>241</v>
-      </c>
-      <c r="N39" s="2"/>
-      <c r="O39" t="s" s="2">
-        <v>242</v>
-      </c>
+        <v>289</v>
+      </c>
+      <c r="N39" t="s" s="2">
+        <v>290</v>
+      </c>
+      <c r="O39" s="2"/>
       <c r="P39" t="s" s="2">
         <v>82</v>
       </c>
-      <c r="Q39" s="2"/>
+      <c r="Q39" t="s" s="2">
+        <v>291</v>
+      </c>
       <c r="R39" t="s" s="2">
         <v>82</v>
       </c>
@@ -6146,7 +6011,7 @@
         <v>82</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>243</v>
+        <v>292</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>80</v>
@@ -6155,7 +6020,7 @@
         <v>90</v>
       </c>
       <c r="AI39" t="s" s="2">
-        <v>82</v>
+        <v>284</v>
       </c>
       <c r="AJ39" t="s" s="2">
         <v>82</v>
@@ -6173,7 +6038,7 @@
         <v>82</v>
       </c>
       <c r="AO39" t="s" s="2">
-        <v>244</v>
+        <v>293</v>
       </c>
       <c r="AP39" t="s" s="2">
         <v>82</v>
@@ -6181,10 +6046,10 @@
     </row>
     <row r="40" hidden="true">
       <c r="A40" t="s" s="2">
-        <v>279</v>
+        <v>294</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>279</v>
+        <v>294</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -6207,20 +6072,18 @@
         <v>91</v>
       </c>
       <c r="K40" t="s" s="2">
-        <v>246</v>
+        <v>295</v>
       </c>
       <c r="L40" t="s" s="2">
-        <v>247</v>
+        <v>296</v>
       </c>
       <c r="M40" t="s" s="2">
-        <v>248</v>
+        <v>297</v>
       </c>
       <c r="N40" t="s" s="2">
-        <v>249</v>
-      </c>
-      <c r="O40" t="s" s="2">
-        <v>250</v>
-      </c>
+        <v>298</v>
+      </c>
+      <c r="O40" s="2"/>
       <c r="P40" t="s" s="2">
         <v>82</v>
       </c>
@@ -6268,7 +6131,7 @@
         <v>82</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>251</v>
+        <v>294</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>80</v>
@@ -6295,18 +6158,18 @@
         <v>82</v>
       </c>
       <c r="AO40" t="s" s="2">
-        <v>252</v>
+        <v>82</v>
       </c>
       <c r="AP40" t="s" s="2">
-        <v>82</v>
+        <v>273</v>
       </c>
     </row>
     <row r="41" hidden="true">
       <c r="A41" t="s" s="2">
-        <v>280</v>
+        <v>299</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>280</v>
+        <v>299</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
@@ -6320,7 +6183,7 @@
         <v>90</v>
       </c>
       <c r="H41" t="s" s="2">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="I41" t="s" s="2">
         <v>82</v>
@@ -6329,20 +6192,16 @@
         <v>91</v>
       </c>
       <c r="K41" t="s" s="2">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="L41" t="s" s="2">
-        <v>254</v>
+        <v>301</v>
       </c>
       <c r="M41" t="s" s="2">
-        <v>255</v>
-      </c>
-      <c r="N41" t="s" s="2">
-        <v>256</v>
-      </c>
-      <c r="O41" t="s" s="2">
-        <v>257</v>
-      </c>
+        <v>302</v>
+      </c>
+      <c r="N41" s="2"/>
+      <c r="O41" s="2"/>
       <c r="P41" t="s" s="2">
         <v>82</v>
       </c>
@@ -6390,7 +6249,7 @@
         <v>82</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>258</v>
+        <v>299</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>80</v>
@@ -6408,7 +6267,7 @@
         <v>82</v>
       </c>
       <c r="AL41" t="s" s="2">
-        <v>82</v>
+        <v>303</v>
       </c>
       <c r="AM41" t="s" s="2">
         <v>82</v>
@@ -6417,18 +6276,18 @@
         <v>82</v>
       </c>
       <c r="AO41" t="s" s="2">
-        <v>259</v>
+        <v>304</v>
       </c>
       <c r="AP41" t="s" s="2">
-        <v>82</v>
+        <v>305</v>
       </c>
     </row>
     <row r="42" hidden="true">
       <c r="A42" t="s" s="2">
-        <v>281</v>
+        <v>306</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>281</v>
+        <v>306</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
@@ -6436,7 +6295,7 @@
       </c>
       <c r="E42" s="2"/>
       <c r="F42" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="G42" t="s" s="2">
         <v>90</v>
@@ -6448,16 +6307,16 @@
         <v>82</v>
       </c>
       <c r="J42" t="s" s="2">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="K42" t="s" s="2">
-        <v>282</v>
+        <v>150</v>
       </c>
       <c r="L42" t="s" s="2">
-        <v>283</v>
+        <v>151</v>
       </c>
       <c r="M42" t="s" s="2">
-        <v>284</v>
+        <v>152</v>
       </c>
       <c r="N42" s="2"/>
       <c r="O42" s="2"/>
@@ -6508,10 +6367,10 @@
         <v>82</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>281</v>
+        <v>153</v>
       </c>
       <c r="AG42" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="AH42" t="s" s="2">
         <v>90</v>
@@ -6535,18 +6394,18 @@
         <v>82</v>
       </c>
       <c r="AO42" t="s" s="2">
-        <v>285</v>
+        <v>154</v>
       </c>
       <c r="AP42" t="s" s="2">
-        <v>286</v>
+        <v>82</v>
       </c>
     </row>
     <row r="43" hidden="true">
       <c r="A43" t="s" s="2">
-        <v>287</v>
+        <v>307</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>287</v>
+        <v>307</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
@@ -6557,7 +6416,7 @@
         <v>80</v>
       </c>
       <c r="G43" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="H43" t="s" s="2">
         <v>82</v>
@@ -6569,13 +6428,13 @@
         <v>82</v>
       </c>
       <c r="K43" t="s" s="2">
-        <v>150</v>
+        <v>135</v>
       </c>
       <c r="L43" t="s" s="2">
-        <v>151</v>
+        <v>136</v>
       </c>
       <c r="M43" t="s" s="2">
-        <v>152</v>
+        <v>137</v>
       </c>
       <c r="N43" s="2"/>
       <c r="O43" s="2"/>
@@ -6614,25 +6473,25 @@
         <v>82</v>
       </c>
       <c r="AB43" t="s" s="2">
-        <v>82</v>
+        <v>138</v>
       </c>
       <c r="AC43" t="s" s="2">
-        <v>82</v>
+        <v>161</v>
       </c>
       <c r="AD43" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AE43" t="s" s="2">
-        <v>82</v>
+        <v>139</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>153</v>
+        <v>162</v>
       </c>
       <c r="AG43" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH43" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="AI43" t="s" s="2">
         <v>82</v>
@@ -6653,7 +6512,7 @@
         <v>82</v>
       </c>
       <c r="AO43" t="s" s="2">
-        <v>154</v>
+        <v>82</v>
       </c>
       <c r="AP43" t="s" s="2">
         <v>82</v>
@@ -6661,12 +6520,14 @@
     </row>
     <row r="44" hidden="true">
       <c r="A44" t="s" s="2">
-        <v>288</v>
+        <v>308</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>288</v>
-      </c>
-      <c r="C44" s="2"/>
+        <v>307</v>
+      </c>
+      <c r="C44" t="s" s="2">
+        <v>248</v>
+      </c>
       <c r="D44" t="s" s="2">
         <v>82</v>
       </c>
@@ -6675,7 +6536,7 @@
         <v>80</v>
       </c>
       <c r="G44" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="H44" t="s" s="2">
         <v>82</v>
@@ -6687,13 +6548,13 @@
         <v>82</v>
       </c>
       <c r="K44" t="s" s="2">
-        <v>135</v>
+        <v>249</v>
       </c>
       <c r="L44" t="s" s="2">
-        <v>136</v>
+        <v>250</v>
       </c>
       <c r="M44" t="s" s="2">
-        <v>137</v>
+        <v>251</v>
       </c>
       <c r="N44" s="2"/>
       <c r="O44" s="2"/>
@@ -6732,16 +6593,16 @@
         <v>82</v>
       </c>
       <c r="AB44" t="s" s="2">
-        <v>138</v>
+        <v>82</v>
       </c>
       <c r="AC44" t="s" s="2">
-        <v>161</v>
+        <v>82</v>
       </c>
       <c r="AD44" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AE44" t="s" s="2">
-        <v>139</v>
+        <v>82</v>
       </c>
       <c r="AF44" t="s" s="2">
         <v>162</v>
@@ -6771,7 +6632,7 @@
         <v>82</v>
       </c>
       <c r="AO44" t="s" s="2">
-        <v>82</v>
+        <v>133</v>
       </c>
       <c r="AP44" t="s" s="2">
         <v>82</v>
@@ -6779,14 +6640,12 @@
     </row>
     <row r="45" hidden="true">
       <c r="A45" t="s" s="2">
-        <v>289</v>
+        <v>309</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>288</v>
-      </c>
-      <c r="C45" t="s" s="2">
-        <v>290</v>
-      </c>
+        <v>309</v>
+      </c>
+      <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
         <v>82</v>
       </c>
@@ -6804,18 +6663,20 @@
         <v>82</v>
       </c>
       <c r="J45" t="s" s="2">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="K45" t="s" s="2">
-        <v>291</v>
+        <v>150</v>
       </c>
       <c r="L45" t="s" s="2">
-        <v>292</v>
+        <v>253</v>
       </c>
       <c r="M45" t="s" s="2">
-        <v>293</v>
-      </c>
-      <c r="N45" s="2"/>
+        <v>254</v>
+      </c>
+      <c r="N45" t="s" s="2">
+        <v>255</v>
+      </c>
       <c r="O45" s="2"/>
       <c r="P45" t="s" s="2">
         <v>82</v>
@@ -6864,16 +6725,16 @@
         <v>82</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>162</v>
+        <v>256</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH45" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="AI45" t="s" s="2">
-        <v>82</v>
+        <v>257</v>
       </c>
       <c r="AJ45" t="s" s="2">
         <v>82</v>
@@ -6899,10 +6760,10 @@
     </row>
     <row r="46" hidden="true">
       <c r="A46" t="s" s="2">
-        <v>294</v>
+        <v>310</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>294</v>
+        <v>310</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
@@ -6925,16 +6786,16 @@
         <v>91</v>
       </c>
       <c r="K46" t="s" s="2">
-        <v>150</v>
+        <v>183</v>
       </c>
       <c r="L46" t="s" s="2">
-        <v>295</v>
+        <v>259</v>
       </c>
       <c r="M46" t="s" s="2">
-        <v>296</v>
+        <v>260</v>
       </c>
       <c r="N46" t="s" s="2">
-        <v>297</v>
+        <v>261</v>
       </c>
       <c r="O46" s="2"/>
       <c r="P46" t="s" s="2">
@@ -6984,7 +6845,7 @@
         <v>82</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>298</v>
+        <v>262</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>80</v>
@@ -6993,7 +6854,7 @@
         <v>90</v>
       </c>
       <c r="AI46" t="s" s="2">
-        <v>299</v>
+        <v>82</v>
       </c>
       <c r="AJ46" t="s" s="2">
         <v>82</v>
@@ -7011,7 +6872,7 @@
         <v>82</v>
       </c>
       <c r="AO46" t="s" s="2">
-        <v>133</v>
+        <v>263</v>
       </c>
       <c r="AP46" t="s" s="2">
         <v>82</v>
@@ -7019,10 +6880,10 @@
     </row>
     <row r="47" hidden="true">
       <c r="A47" t="s" s="2">
-        <v>300</v>
+        <v>311</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>300</v>
+        <v>311</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
@@ -7045,16 +6906,16 @@
         <v>91</v>
       </c>
       <c r="K47" t="s" s="2">
-        <v>183</v>
+        <v>150</v>
       </c>
       <c r="L47" t="s" s="2">
-        <v>301</v>
+        <v>265</v>
       </c>
       <c r="M47" t="s" s="2">
-        <v>302</v>
+        <v>266</v>
       </c>
       <c r="N47" t="s" s="2">
-        <v>303</v>
+        <v>267</v>
       </c>
       <c r="O47" s="2"/>
       <c r="P47" t="s" s="2">
@@ -7104,7 +6965,7 @@
         <v>82</v>
       </c>
       <c r="AF47" t="s" s="2">
-        <v>304</v>
+        <v>268</v>
       </c>
       <c r="AG47" t="s" s="2">
         <v>80</v>
@@ -7131,1686 +6992,14 @@
         <v>82</v>
       </c>
       <c r="AO47" t="s" s="2">
-        <v>305</v>
+        <v>133</v>
       </c>
       <c r="AP47" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="48" hidden="true">
-      <c r="A48" t="s" s="2">
-        <v>306</v>
-      </c>
-      <c r="B48" t="s" s="2">
-        <v>306</v>
-      </c>
-      <c r="C48" s="2"/>
-      <c r="D48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E48" s="2"/>
-      <c r="F48" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G48" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="H48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J48" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="K48" t="s" s="2">
-        <v>150</v>
-      </c>
-      <c r="L48" t="s" s="2">
-        <v>307</v>
-      </c>
-      <c r="M48" t="s" s="2">
-        <v>308</v>
-      </c>
-      <c r="N48" t="s" s="2">
-        <v>309</v>
-      </c>
-      <c r="O48" s="2"/>
-      <c r="P48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q48" s="2"/>
-      <c r="R48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF48" t="s" s="2">
-        <v>310</v>
-      </c>
-      <c r="AG48" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH48" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="AI48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AK48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN48" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO48" t="s" s="2">
-        <v>133</v>
-      </c>
-      <c r="AP48" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="49" hidden="true">
-      <c r="A49" t="s" s="2">
-        <v>311</v>
-      </c>
-      <c r="B49" t="s" s="2">
-        <v>311</v>
-      </c>
-      <c r="C49" s="2"/>
-      <c r="D49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E49" s="2"/>
-      <c r="F49" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G49" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="H49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J49" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="K49" t="s" s="2">
-        <v>312</v>
-      </c>
-      <c r="L49" t="s" s="2">
-        <v>313</v>
-      </c>
-      <c r="M49" t="s" s="2">
-        <v>314</v>
-      </c>
-      <c r="N49" s="2"/>
-      <c r="O49" s="2"/>
-      <c r="P49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q49" s="2"/>
-      <c r="R49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF49" t="s" s="2">
-        <v>311</v>
-      </c>
-      <c r="AG49" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH49" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="AI49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AK49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AP49" t="s" s="2">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="50" hidden="true">
-      <c r="A50" t="s" s="2">
-        <v>316</v>
-      </c>
-      <c r="B50" t="s" s="2">
-        <v>316</v>
-      </c>
-      <c r="C50" s="2"/>
-      <c r="D50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E50" s="2"/>
-      <c r="F50" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G50" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="H50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="K50" t="s" s="2">
-        <v>150</v>
-      </c>
-      <c r="L50" t="s" s="2">
-        <v>151</v>
-      </c>
-      <c r="M50" t="s" s="2">
-        <v>152</v>
-      </c>
-      <c r="N50" s="2"/>
-      <c r="O50" s="2"/>
-      <c r="P50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q50" s="2"/>
-      <c r="R50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF50" t="s" s="2">
-        <v>153</v>
-      </c>
-      <c r="AG50" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH50" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="AI50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AK50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO50" t="s" s="2">
-        <v>154</v>
-      </c>
-      <c r="AP50" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="51" hidden="true">
-      <c r="A51" t="s" s="2">
-        <v>317</v>
-      </c>
-      <c r="B51" t="s" s="2">
-        <v>317</v>
-      </c>
-      <c r="C51" s="2"/>
-      <c r="D51" t="s" s="2">
-        <v>157</v>
-      </c>
-      <c r="E51" s="2"/>
-      <c r="F51" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G51" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="H51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="K51" t="s" s="2">
-        <v>135</v>
-      </c>
-      <c r="L51" t="s" s="2">
-        <v>158</v>
-      </c>
-      <c r="M51" t="s" s="2">
-        <v>159</v>
-      </c>
-      <c r="N51" t="s" s="2">
-        <v>160</v>
-      </c>
-      <c r="O51" s="2"/>
-      <c r="P51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q51" s="2"/>
-      <c r="R51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB51" t="s" s="2">
-        <v>138</v>
-      </c>
-      <c r="AC51" t="s" s="2">
-        <v>161</v>
-      </c>
-      <c r="AD51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE51" t="s" s="2">
-        <v>139</v>
-      </c>
-      <c r="AF51" t="s" s="2">
-        <v>162</v>
-      </c>
-      <c r="AG51" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH51" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AI51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AK51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO51" t="s" s="2">
-        <v>154</v>
-      </c>
-      <c r="AP51" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="52" hidden="true">
-      <c r="A52" t="s" s="2">
-        <v>318</v>
-      </c>
-      <c r="B52" t="s" s="2">
-        <v>318</v>
-      </c>
-      <c r="C52" s="2"/>
-      <c r="D52" t="s" s="2">
-        <v>319</v>
-      </c>
-      <c r="E52" s="2"/>
-      <c r="F52" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G52" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="H52" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="I52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J52" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="K52" t="s" s="2">
-        <v>320</v>
-      </c>
-      <c r="L52" t="s" s="2">
-        <v>321</v>
-      </c>
-      <c r="M52" t="s" s="2">
-        <v>322</v>
-      </c>
-      <c r="N52" t="s" s="2">
-        <v>323</v>
-      </c>
-      <c r="O52" s="2"/>
-      <c r="P52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q52" s="2"/>
-      <c r="R52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T52" t="s" s="2">
-        <v>324</v>
-      </c>
-      <c r="U52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF52" t="s" s="2">
-        <v>325</v>
-      </c>
-      <c r="AG52" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH52" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="AI52" t="s" s="2">
-        <v>326</v>
-      </c>
-      <c r="AJ52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AK52" t="s" s="2">
-        <v>327</v>
-      </c>
-      <c r="AL52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM52" t="s" s="2">
-        <v>327</v>
-      </c>
-      <c r="AN52" t="s" s="2">
-        <v>327</v>
-      </c>
-      <c r="AO52" t="s" s="2">
-        <v>328</v>
-      </c>
-      <c r="AP52" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="53" hidden="true">
-      <c r="A53" t="s" s="2">
-        <v>329</v>
-      </c>
-      <c r="B53" t="s" s="2">
-        <v>329</v>
-      </c>
-      <c r="C53" s="2"/>
-      <c r="D53" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E53" s="2"/>
-      <c r="F53" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G53" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="H53" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I53" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J53" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="K53" t="s" s="2">
-        <v>320</v>
-      </c>
-      <c r="L53" t="s" s="2">
-        <v>330</v>
-      </c>
-      <c r="M53" t="s" s="2">
-        <v>331</v>
-      </c>
-      <c r="N53" t="s" s="2">
-        <v>332</v>
-      </c>
-      <c r="O53" s="2"/>
-      <c r="P53" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q53" t="s" s="2">
-        <v>333</v>
-      </c>
-      <c r="R53" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S53" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T53" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U53" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V53" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W53" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X53" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y53" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z53" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA53" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB53" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC53" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD53" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE53" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF53" t="s" s="2">
-        <v>334</v>
-      </c>
-      <c r="AG53" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH53" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="AI53" t="s" s="2">
-        <v>326</v>
-      </c>
-      <c r="AJ53" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AK53" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL53" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM53" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN53" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO53" t="s" s="2">
-        <v>335</v>
-      </c>
-      <c r="AP53" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="54" hidden="true">
-      <c r="A54" t="s" s="2">
-        <v>336</v>
-      </c>
-      <c r="B54" t="s" s="2">
-        <v>336</v>
-      </c>
-      <c r="C54" s="2"/>
-      <c r="D54" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E54" s="2"/>
-      <c r="F54" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G54" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="H54" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I54" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J54" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="K54" t="s" s="2">
-        <v>337</v>
-      </c>
-      <c r="L54" t="s" s="2">
-        <v>338</v>
-      </c>
-      <c r="M54" t="s" s="2">
-        <v>339</v>
-      </c>
-      <c r="N54" t="s" s="2">
-        <v>340</v>
-      </c>
-      <c r="O54" s="2"/>
-      <c r="P54" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q54" s="2"/>
-      <c r="R54" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S54" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T54" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U54" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V54" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W54" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X54" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y54" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z54" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA54" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB54" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC54" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD54" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE54" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF54" t="s" s="2">
-        <v>336</v>
-      </c>
-      <c r="AG54" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH54" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="AI54" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ54" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AK54" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL54" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM54" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN54" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO54" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AP54" t="s" s="2">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="55" hidden="true">
-      <c r="A55" t="s" s="2">
-        <v>341</v>
-      </c>
-      <c r="B55" t="s" s="2">
-        <v>341</v>
-      </c>
-      <c r="C55" s="2"/>
-      <c r="D55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E55" s="2"/>
-      <c r="F55" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G55" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="H55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J55" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="K55" t="s" s="2">
-        <v>342</v>
-      </c>
-      <c r="L55" t="s" s="2">
-        <v>343</v>
-      </c>
-      <c r="M55" t="s" s="2">
-        <v>344</v>
-      </c>
-      <c r="N55" s="2"/>
-      <c r="O55" s="2"/>
-      <c r="P55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q55" s="2"/>
-      <c r="R55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF55" t="s" s="2">
-        <v>341</v>
-      </c>
-      <c r="AG55" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH55" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="AI55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AK55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL55" t="s" s="2">
-        <v>345</v>
-      </c>
-      <c r="AM55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO55" t="s" s="2">
-        <v>346</v>
-      </c>
-      <c r="AP55" t="s" s="2">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="56" hidden="true">
-      <c r="A56" t="s" s="2">
-        <v>348</v>
-      </c>
-      <c r="B56" t="s" s="2">
-        <v>348</v>
-      </c>
-      <c r="C56" s="2"/>
-      <c r="D56" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E56" s="2"/>
-      <c r="F56" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G56" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="H56" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I56" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J56" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="K56" t="s" s="2">
-        <v>150</v>
-      </c>
-      <c r="L56" t="s" s="2">
-        <v>151</v>
-      </c>
-      <c r="M56" t="s" s="2">
-        <v>152</v>
-      </c>
-      <c r="N56" s="2"/>
-      <c r="O56" s="2"/>
-      <c r="P56" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q56" s="2"/>
-      <c r="R56" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S56" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T56" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U56" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V56" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W56" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X56" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y56" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z56" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA56" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB56" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC56" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD56" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE56" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF56" t="s" s="2">
-        <v>153</v>
-      </c>
-      <c r="AG56" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH56" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="AI56" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ56" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AK56" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL56" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM56" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN56" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO56" t="s" s="2">
-        <v>154</v>
-      </c>
-      <c r="AP56" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="57" hidden="true">
-      <c r="A57" t="s" s="2">
-        <v>349</v>
-      </c>
-      <c r="B57" t="s" s="2">
-        <v>349</v>
-      </c>
-      <c r="C57" s="2"/>
-      <c r="D57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E57" s="2"/>
-      <c r="F57" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G57" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="H57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="K57" t="s" s="2">
-        <v>135</v>
-      </c>
-      <c r="L57" t="s" s="2">
-        <v>136</v>
-      </c>
-      <c r="M57" t="s" s="2">
-        <v>137</v>
-      </c>
-      <c r="N57" s="2"/>
-      <c r="O57" s="2"/>
-      <c r="P57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q57" s="2"/>
-      <c r="R57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB57" t="s" s="2">
-        <v>138</v>
-      </c>
-      <c r="AC57" t="s" s="2">
-        <v>161</v>
-      </c>
-      <c r="AD57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE57" t="s" s="2">
-        <v>139</v>
-      </c>
-      <c r="AF57" t="s" s="2">
-        <v>162</v>
-      </c>
-      <c r="AG57" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH57" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AI57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AK57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AP57" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="58" hidden="true">
-      <c r="A58" t="s" s="2">
-        <v>350</v>
-      </c>
-      <c r="B58" t="s" s="2">
-        <v>349</v>
-      </c>
-      <c r="C58" t="s" s="2">
-        <v>290</v>
-      </c>
-      <c r="D58" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E58" s="2"/>
-      <c r="F58" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G58" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="H58" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I58" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J58" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="K58" t="s" s="2">
-        <v>291</v>
-      </c>
-      <c r="L58" t="s" s="2">
-        <v>292</v>
-      </c>
-      <c r="M58" t="s" s="2">
-        <v>293</v>
-      </c>
-      <c r="N58" s="2"/>
-      <c r="O58" s="2"/>
-      <c r="P58" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q58" s="2"/>
-      <c r="R58" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S58" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T58" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U58" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V58" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W58" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X58" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y58" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z58" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA58" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB58" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC58" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD58" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE58" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF58" t="s" s="2">
-        <v>162</v>
-      </c>
-      <c r="AG58" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH58" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AI58" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ58" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AK58" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL58" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM58" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN58" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO58" t="s" s="2">
-        <v>133</v>
-      </c>
-      <c r="AP58" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="59" hidden="true">
-      <c r="A59" t="s" s="2">
-        <v>351</v>
-      </c>
-      <c r="B59" t="s" s="2">
-        <v>351</v>
-      </c>
-      <c r="C59" s="2"/>
-      <c r="D59" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E59" s="2"/>
-      <c r="F59" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G59" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="H59" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I59" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J59" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="K59" t="s" s="2">
-        <v>150</v>
-      </c>
-      <c r="L59" t="s" s="2">
-        <v>295</v>
-      </c>
-      <c r="M59" t="s" s="2">
-        <v>296</v>
-      </c>
-      <c r="N59" t="s" s="2">
-        <v>297</v>
-      </c>
-      <c r="O59" s="2"/>
-      <c r="P59" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q59" s="2"/>
-      <c r="R59" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S59" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T59" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U59" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V59" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W59" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X59" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y59" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z59" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA59" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB59" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC59" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD59" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE59" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF59" t="s" s="2">
-        <v>298</v>
-      </c>
-      <c r="AG59" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH59" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="AI59" t="s" s="2">
-        <v>299</v>
-      </c>
-      <c r="AJ59" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AK59" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL59" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM59" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN59" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO59" t="s" s="2">
-        <v>133</v>
-      </c>
-      <c r="AP59" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="60" hidden="true">
-      <c r="A60" t="s" s="2">
-        <v>352</v>
-      </c>
-      <c r="B60" t="s" s="2">
-        <v>352</v>
-      </c>
-      <c r="C60" s="2"/>
-      <c r="D60" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E60" s="2"/>
-      <c r="F60" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G60" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="H60" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I60" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J60" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="K60" t="s" s="2">
-        <v>183</v>
-      </c>
-      <c r="L60" t="s" s="2">
-        <v>301</v>
-      </c>
-      <c r="M60" t="s" s="2">
-        <v>302</v>
-      </c>
-      <c r="N60" t="s" s="2">
-        <v>303</v>
-      </c>
-      <c r="O60" s="2"/>
-      <c r="P60" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q60" s="2"/>
-      <c r="R60" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S60" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T60" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U60" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V60" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W60" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X60" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y60" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z60" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA60" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB60" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC60" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD60" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE60" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF60" t="s" s="2">
-        <v>304</v>
-      </c>
-      <c r="AG60" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH60" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="AI60" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ60" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AK60" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL60" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM60" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN60" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO60" t="s" s="2">
-        <v>305</v>
-      </c>
-      <c r="AP60" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="61" hidden="true">
-      <c r="A61" t="s" s="2">
-        <v>353</v>
-      </c>
-      <c r="B61" t="s" s="2">
-        <v>353</v>
-      </c>
-      <c r="C61" s="2"/>
-      <c r="D61" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E61" s="2"/>
-      <c r="F61" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G61" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="H61" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I61" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J61" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="K61" t="s" s="2">
-        <v>150</v>
-      </c>
-      <c r="L61" t="s" s="2">
-        <v>307</v>
-      </c>
-      <c r="M61" t="s" s="2">
-        <v>308</v>
-      </c>
-      <c r="N61" t="s" s="2">
-        <v>309</v>
-      </c>
-      <c r="O61" s="2"/>
-      <c r="P61" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q61" s="2"/>
-      <c r="R61" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S61" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T61" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U61" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V61" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W61" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X61" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y61" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z61" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA61" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB61" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC61" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD61" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE61" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF61" t="s" s="2">
-        <v>310</v>
-      </c>
-      <c r="AG61" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH61" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="AI61" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ61" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AK61" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL61" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM61" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN61" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO61" t="s" s="2">
-        <v>133</v>
-      </c>
-      <c r="AP61" t="s" s="2">
         <v>82</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AP61">
+  <autoFilter ref="A1:AP47">
     <filterColumn colId="6">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
@@ -8820,7 +7009,7 @@
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>
-  <conditionalFormatting sqref="A2:AI60">
+  <conditionalFormatting sqref="A2:AI46">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$G2&lt;&gt;"Y"</formula>
     </cfRule>

</xml_diff>